<commit_message>
fix images pour github
</commit_message>
<xml_diff>
--- a/data/fc27-data.xlsx
+++ b/data/fc27-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexi\Desktop\Projets\builderproclubs\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFAD8D40-1DE4-4737-A256-6E30F3DDCE1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD776423-7328-4414-A646-90C6A81151BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="4" activeTab="18" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lisez-moi" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Boss!$A$3:$Z$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">Creator!$A$3:$Z$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">Disruptor!$A$3:$Z$39</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Facilitateur!$A$3:$Z$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Facilitateur!$A$3:$Y$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">Finisher!$A$3:$Z$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">Maestro!$A$3:$Z$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">Magician!$A$3:$Z$39</definedName>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2649" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2648" uniqueCount="281">
   <si>
     <t>Base de données — FC 27 Constructeur de build</t>
   </si>
@@ -892,6 +892,12 @@
   <si>
     <t>Forteresse aérienne</t>
   </si>
+  <si>
+    <t>61-64</t>
+  </si>
+  <si>
+    <t>65-69</t>
+  </si>
 </sst>
 </file>
 
@@ -945,7 +951,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -970,6 +976,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE9E2F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor theme="0" tint="-0.14999847407452621"/>
       </patternFill>
     </fill>
   </fills>
@@ -1015,7 +1027,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1046,6 +1058,10 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1109,9 +1125,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B25F6B7E-BDB4-4556-93D2-D823D0060FF6}" name="Table1" displayName="Table1" ref="A3:Z39" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1">
-  <autoFilter ref="A3:Z39" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
-  <tableColumns count="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B25F6B7E-BDB4-4556-93D2-D823D0060FF6}" name="Table1" displayName="Table1" ref="A3:Y39" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1">
+  <autoFilter ref="A3:Y39" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
+  <tableColumns count="25">
     <tableColumn id="1" xr3:uid="{EDC2B16E-8713-45EE-BE81-CDE8D764A76B}" name="attribut"/>
     <tableColumn id="2" xr3:uid="{3157AA01-579B-43D2-8D17-A25D980F28BC}" name="nom"/>
     <tableColumn id="3" xr3:uid="{27114B50-8405-4E8C-8DD1-B69EF2903F72}" name="categorie"/>
@@ -1120,9 +1136,8 @@
     <tableColumn id="6" xr3:uid="{B389CBC2-C9CD-4EA0-9CDB-9A7CE9443835}" name="limite_min"/>
     <tableColumn id="7" xr3:uid="{BF5EB726-211F-4EAB-8ACB-23D5C69CF0A9}" name="limite_max"/>
     <tableColumn id="8" xr3:uid="{35448435-384C-4432-9043-32D70AB74E83}" name="1-60"/>
-    <tableColumn id="9" xr3:uid="{EB7894A2-5261-491E-84A0-D8665EBA6661}" name="61-63"/>
-    <tableColumn id="10" xr3:uid="{B44CE625-67DD-4C6B-9402-D06B6FB9D428}" name="64-66"/>
-    <tableColumn id="11" xr3:uid="{EF63C3B4-6AB1-4407-A53A-15179A890598}" name="67-69"/>
+    <tableColumn id="9" xr3:uid="{EB7894A2-5261-491E-84A0-D8665EBA6661}" name="61-64"/>
+    <tableColumn id="11" xr3:uid="{EF63C3B4-6AB1-4407-A53A-15179A890598}" name="65-69"/>
     <tableColumn id="12" xr3:uid="{CB92E0C8-A8AA-424D-97C5-AC3C04CD327C}" name="70-74"/>
     <tableColumn id="13" xr3:uid="{86B602FA-60C5-4414-AB16-70F62753BADF}" name="75-79"/>
     <tableColumn id="14" xr3:uid="{5100757D-B350-4AA4-991C-DADAB95F5E41}" name="80-84"/>
@@ -3121,117 +3136,104 @@
       <c r="Z29" s="10"/>
     </row>
     <row r="30" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="18" t="s">
+        <v>166</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="C30" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="D30" s="18" t="s">
+        <v>211</v>
+      </c>
+      <c r="E30" s="18">
+        <v>65</v>
+      </c>
+      <c r="F30" s="18">
+        <v>65</v>
+      </c>
+      <c r="G30" s="18">
+        <v>92</v>
+      </c>
+      <c r="H30" s="18"/>
+      <c r="I30" s="18"/>
+      <c r="J30" s="18">
+        <v>3</v>
+      </c>
+      <c r="K30" s="18">
+        <v>4</v>
+      </c>
+      <c r="L30" s="18">
+        <v>5</v>
+      </c>
+      <c r="M30" s="18">
+        <v>8</v>
+      </c>
+      <c r="N30" s="18">
+        <v>11</v>
+      </c>
+      <c r="O30" s="18"/>
+      <c r="P30" s="18"/>
+      <c r="Q30" s="18"/>
+      <c r="R30" s="18"/>
+      <c r="S30" s="18"/>
+      <c r="T30" s="18"/>
+      <c r="U30" s="18"/>
+      <c r="V30" s="18"/>
+      <c r="W30" s="18"/>
+      <c r="X30" s="18"/>
+      <c r="Y30" s="19"/>
+      <c r="Z30" s="10"/>
+    </row>
+    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>164</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B31" t="s">
         <v>165</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C31" t="s">
         <v>163</v>
       </c>
-      <c r="D30" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="E30" s="7">
+      <c r="D31" t="s">
+        <v>211</v>
+      </c>
+      <c r="E31">
         <v>70</v>
       </c>
-      <c r="F30" s="7">
+      <c r="F31">
         <v>70</v>
       </c>
-      <c r="G30" s="7">
+      <c r="G31">
         <v>96</v>
       </c>
-      <c r="H30" s="9"/>
-      <c r="I30" s="10"/>
-      <c r="J30" s="10"/>
-      <c r="K30" s="10"/>
-      <c r="L30" s="7">
-        <v>4</v>
-      </c>
-      <c r="M30" s="7">
+      <c r="K31">
+        <v>4</v>
+      </c>
+      <c r="L31">
         <v>6</v>
       </c>
-      <c r="N30" s="7">
+      <c r="M31">
         <v>7</v>
       </c>
-      <c r="O30" s="7">
+      <c r="N31">
         <v>11</v>
       </c>
-      <c r="P30" s="7">
+      <c r="O31">
         <v>15</v>
       </c>
-      <c r="Q30" s="7">
+      <c r="P31">
         <v>20</v>
       </c>
-      <c r="R30" s="7">
+      <c r="Q31">
         <v>25</v>
       </c>
-      <c r="S30" s="7">
+      <c r="R31">
         <v>30</v>
       </c>
-      <c r="T30" s="10"/>
-      <c r="U30" s="10"/>
-      <c r="V30" s="10"/>
-      <c r="W30" s="9"/>
-      <c r="X30" s="10"/>
-      <c r="Y30" s="10"/>
-      <c r="Z30" s="10"/>
-    </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A31" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="E31" s="7">
-        <v>65</v>
-      </c>
-      <c r="F31" s="7">
-        <v>65</v>
-      </c>
-      <c r="G31" s="7">
-        <v>92</v>
-      </c>
-      <c r="H31" s="9"/>
-      <c r="I31" s="10"/>
-      <c r="J31" s="7">
-        <v>2</v>
-      </c>
-      <c r="K31" s="7">
-        <v>2</v>
-      </c>
-      <c r="L31" s="7">
-        <v>3</v>
-      </c>
-      <c r="M31" s="7">
-        <v>4</v>
-      </c>
-      <c r="N31" s="7">
-        <v>5</v>
-      </c>
-      <c r="O31" s="7">
-        <v>8</v>
-      </c>
-      <c r="P31" s="7">
-        <v>11</v>
-      </c>
-      <c r="Q31" s="10"/>
-      <c r="R31" s="10"/>
-      <c r="S31" s="10"/>
-      <c r="T31" s="10"/>
-      <c r="U31" s="10"/>
-      <c r="V31" s="10"/>
-      <c r="W31" s="9"/>
-      <c r="X31" s="10"/>
-      <c r="Y31" s="10"/>
+      <c r="Y31" s="14"/>
       <c r="Z31" s="10"/>
     </row>
     <row r="32" spans="1:26" x14ac:dyDescent="0.25">
@@ -5197,115 +5199,104 @@
       <c r="Z29" s="10"/>
     </row>
     <row r="30" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="18" t="s">
+        <v>166</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="C30" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="D30" s="18" t="s">
+        <v>211</v>
+      </c>
+      <c r="E30" s="18">
+        <v>65</v>
+      </c>
+      <c r="F30" s="18">
+        <v>65</v>
+      </c>
+      <c r="G30" s="18">
+        <v>92</v>
+      </c>
+      <c r="H30" s="18"/>
+      <c r="I30" s="18"/>
+      <c r="J30" s="18">
+        <v>3</v>
+      </c>
+      <c r="K30" s="18">
+        <v>4</v>
+      </c>
+      <c r="L30" s="18">
+        <v>5</v>
+      </c>
+      <c r="M30" s="18">
+        <v>8</v>
+      </c>
+      <c r="N30" s="18">
+        <v>11</v>
+      </c>
+      <c r="O30" s="18"/>
+      <c r="P30" s="18"/>
+      <c r="Q30" s="18"/>
+      <c r="R30" s="18"/>
+      <c r="S30" s="18"/>
+      <c r="T30" s="18"/>
+      <c r="U30" s="18"/>
+      <c r="V30" s="18"/>
+      <c r="W30" s="18"/>
+      <c r="X30" s="18"/>
+      <c r="Y30" s="19"/>
+      <c r="Z30" s="10"/>
+    </row>
+    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>164</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B31" t="s">
         <v>165</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C31" t="s">
         <v>163</v>
       </c>
-      <c r="D30" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="E30" s="7">
-        <v>65</v>
-      </c>
-      <c r="F30" s="7">
-        <v>65</v>
-      </c>
-      <c r="G30" s="7">
-        <v>92</v>
-      </c>
-      <c r="H30" s="9"/>
-      <c r="I30" s="10"/>
-      <c r="J30" s="7">
-        <v>3</v>
-      </c>
-      <c r="K30" s="7">
-        <v>3</v>
-      </c>
-      <c r="L30" s="7">
-        <v>4</v>
-      </c>
-      <c r="M30" s="7">
+      <c r="D31" t="s">
+        <v>211</v>
+      </c>
+      <c r="E31">
+        <v>70</v>
+      </c>
+      <c r="F31">
+        <v>70</v>
+      </c>
+      <c r="G31">
+        <v>96</v>
+      </c>
+      <c r="K31">
+        <v>4</v>
+      </c>
+      <c r="L31">
         <v>6</v>
       </c>
-      <c r="N30" s="7">
+      <c r="M31">
         <v>7</v>
       </c>
-      <c r="O30" s="7">
+      <c r="N31">
         <v>11</v>
       </c>
-      <c r="P30" s="7">
+      <c r="O31">
         <v>15</v>
       </c>
-      <c r="Q30" s="10"/>
-      <c r="R30" s="10"/>
-      <c r="S30" s="10"/>
-      <c r="T30" s="10"/>
-      <c r="U30" s="10"/>
-      <c r="V30" s="10"/>
-      <c r="W30" s="9"/>
-      <c r="X30" s="10"/>
-      <c r="Y30" s="10"/>
-      <c r="Z30" s="10"/>
-    </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A31" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="E31" s="7">
-        <v>65</v>
-      </c>
-      <c r="F31" s="7">
-        <v>65</v>
-      </c>
-      <c r="G31" s="7">
-        <v>92</v>
-      </c>
-      <c r="H31" s="9"/>
-      <c r="I31" s="10"/>
-      <c r="J31" s="7">
-        <v>3</v>
-      </c>
-      <c r="K31" s="7">
-        <v>3</v>
-      </c>
-      <c r="L31" s="7">
-        <v>4</v>
-      </c>
-      <c r="M31" s="7">
-        <v>6</v>
-      </c>
-      <c r="N31" s="7">
-        <v>7</v>
-      </c>
-      <c r="O31" s="7">
-        <v>11</v>
-      </c>
-      <c r="P31" s="7">
-        <v>15</v>
-      </c>
-      <c r="Q31" s="10"/>
-      <c r="R31" s="10"/>
-      <c r="S31" s="10"/>
-      <c r="T31" s="10"/>
-      <c r="U31" s="10"/>
-      <c r="V31" s="10"/>
-      <c r="W31" s="9"/>
-      <c r="X31" s="10"/>
-      <c r="Y31" s="10"/>
+      <c r="P31">
+        <v>20</v>
+      </c>
+      <c r="Q31">
+        <v>25</v>
+      </c>
+      <c r="R31">
+        <v>30</v>
+      </c>
+      <c r="Y31" s="14"/>
       <c r="Z31" s="10"/>
     </row>
     <row r="32" spans="1:26" x14ac:dyDescent="0.25">
@@ -7271,115 +7262,104 @@
       <c r="Z29" s="10"/>
     </row>
     <row r="30" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="18" t="s">
+        <v>166</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="C30" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="D30" s="18" t="s">
+        <v>211</v>
+      </c>
+      <c r="E30" s="18">
+        <v>65</v>
+      </c>
+      <c r="F30" s="18">
+        <v>65</v>
+      </c>
+      <c r="G30" s="18">
+        <v>92</v>
+      </c>
+      <c r="H30" s="18"/>
+      <c r="I30" s="18"/>
+      <c r="J30" s="18">
+        <v>3</v>
+      </c>
+      <c r="K30" s="18">
+        <v>4</v>
+      </c>
+      <c r="L30" s="18">
+        <v>5</v>
+      </c>
+      <c r="M30" s="18">
+        <v>8</v>
+      </c>
+      <c r="N30" s="18">
+        <v>11</v>
+      </c>
+      <c r="O30" s="18"/>
+      <c r="P30" s="18"/>
+      <c r="Q30" s="18"/>
+      <c r="R30" s="18"/>
+      <c r="S30" s="18"/>
+      <c r="T30" s="18"/>
+      <c r="U30" s="18"/>
+      <c r="V30" s="18"/>
+      <c r="W30" s="18"/>
+      <c r="X30" s="18"/>
+      <c r="Y30" s="19"/>
+      <c r="Z30" s="10"/>
+    </row>
+    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>164</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B31" t="s">
         <v>165</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C31" t="s">
         <v>163</v>
       </c>
-      <c r="D30" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="E30" s="7">
-        <v>65</v>
-      </c>
-      <c r="F30" s="7">
-        <v>65</v>
-      </c>
-      <c r="G30" s="7">
-        <v>92</v>
-      </c>
-      <c r="H30" s="9"/>
-      <c r="I30" s="10"/>
-      <c r="J30" s="7">
-        <v>3</v>
-      </c>
-      <c r="K30" s="7">
-        <v>3</v>
-      </c>
-      <c r="L30" s="7">
-        <v>4</v>
-      </c>
-      <c r="M30" s="7">
+      <c r="D31" t="s">
+        <v>211</v>
+      </c>
+      <c r="E31">
+        <v>70</v>
+      </c>
+      <c r="F31">
+        <v>70</v>
+      </c>
+      <c r="G31">
+        <v>96</v>
+      </c>
+      <c r="K31">
+        <v>4</v>
+      </c>
+      <c r="L31">
         <v>6</v>
       </c>
-      <c r="N30" s="7">
+      <c r="M31">
         <v>7</v>
       </c>
-      <c r="O30" s="7">
+      <c r="N31">
         <v>11</v>
       </c>
-      <c r="P30" s="7">
+      <c r="O31">
         <v>15</v>
       </c>
-      <c r="Q30" s="10"/>
-      <c r="R30" s="10"/>
-      <c r="S30" s="10"/>
-      <c r="T30" s="10"/>
-      <c r="U30" s="10"/>
-      <c r="V30" s="10"/>
-      <c r="W30" s="9"/>
-      <c r="X30" s="10"/>
-      <c r="Y30" s="10"/>
-      <c r="Z30" s="10"/>
-    </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A31" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="E31" s="7">
-        <v>65</v>
-      </c>
-      <c r="F31" s="7">
-        <v>65</v>
-      </c>
-      <c r="G31" s="7">
-        <v>92</v>
-      </c>
-      <c r="H31" s="9"/>
-      <c r="I31" s="10"/>
-      <c r="J31" s="7">
-        <v>3</v>
-      </c>
-      <c r="K31" s="7">
-        <v>3</v>
-      </c>
-      <c r="L31" s="7">
-        <v>4</v>
-      </c>
-      <c r="M31" s="7">
-        <v>6</v>
-      </c>
-      <c r="N31" s="7">
-        <v>7</v>
-      </c>
-      <c r="O31" s="7">
-        <v>11</v>
-      </c>
-      <c r="P31" s="7">
-        <v>15</v>
-      </c>
-      <c r="Q31" s="10"/>
-      <c r="R31" s="10"/>
-      <c r="S31" s="10"/>
-      <c r="T31" s="10"/>
-      <c r="U31" s="10"/>
-      <c r="V31" s="10"/>
-      <c r="W31" s="9"/>
-      <c r="X31" s="10"/>
-      <c r="Y31" s="10"/>
+      <c r="P31">
+        <v>20</v>
+      </c>
+      <c r="Q31">
+        <v>25</v>
+      </c>
+      <c r="R31">
+        <v>30</v>
+      </c>
+      <c r="Y31" s="14"/>
       <c r="Z31" s="10"/>
     </row>
     <row r="32" spans="1:26" x14ac:dyDescent="0.25">
@@ -9343,115 +9323,104 @@
       <c r="Z29" s="10"/>
     </row>
     <row r="30" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="18" t="s">
+        <v>166</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="C30" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="D30" s="18" t="s">
+        <v>211</v>
+      </c>
+      <c r="E30" s="18">
+        <v>65</v>
+      </c>
+      <c r="F30" s="18">
+        <v>65</v>
+      </c>
+      <c r="G30" s="18">
+        <v>92</v>
+      </c>
+      <c r="H30" s="18"/>
+      <c r="I30" s="18"/>
+      <c r="J30" s="18">
+        <v>3</v>
+      </c>
+      <c r="K30" s="18">
+        <v>4</v>
+      </c>
+      <c r="L30" s="18">
+        <v>5</v>
+      </c>
+      <c r="M30" s="18">
+        <v>8</v>
+      </c>
+      <c r="N30" s="18">
+        <v>11</v>
+      </c>
+      <c r="O30" s="18"/>
+      <c r="P30" s="18"/>
+      <c r="Q30" s="18"/>
+      <c r="R30" s="18"/>
+      <c r="S30" s="18"/>
+      <c r="T30" s="18"/>
+      <c r="U30" s="18"/>
+      <c r="V30" s="18"/>
+      <c r="W30" s="18"/>
+      <c r="X30" s="18"/>
+      <c r="Y30" s="19"/>
+      <c r="Z30" s="10"/>
+    </row>
+    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>164</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B31" t="s">
         <v>165</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C31" t="s">
         <v>163</v>
       </c>
-      <c r="D30" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="E30" s="7">
-        <v>65</v>
-      </c>
-      <c r="F30" s="7">
-        <v>65</v>
-      </c>
-      <c r="G30" s="7">
-        <v>92</v>
-      </c>
-      <c r="H30" s="9"/>
-      <c r="I30" s="10"/>
-      <c r="J30" s="7">
-        <v>3</v>
-      </c>
-      <c r="K30" s="7">
-        <v>3</v>
-      </c>
-      <c r="L30" s="7">
-        <v>4</v>
-      </c>
-      <c r="M30" s="7">
+      <c r="D31" t="s">
+        <v>211</v>
+      </c>
+      <c r="E31">
+        <v>70</v>
+      </c>
+      <c r="F31">
+        <v>70</v>
+      </c>
+      <c r="G31">
+        <v>96</v>
+      </c>
+      <c r="K31">
+        <v>4</v>
+      </c>
+      <c r="L31">
         <v>6</v>
       </c>
-      <c r="N30" s="7">
+      <c r="M31">
         <v>7</v>
       </c>
-      <c r="O30" s="7">
+      <c r="N31">
         <v>11</v>
       </c>
-      <c r="P30" s="7">
+      <c r="O31">
         <v>15</v>
       </c>
-      <c r="Q30" s="10"/>
-      <c r="R30" s="10"/>
-      <c r="S30" s="10"/>
-      <c r="T30" s="10"/>
-      <c r="U30" s="10"/>
-      <c r="V30" s="10"/>
-      <c r="W30" s="9"/>
-      <c r="X30" s="10"/>
-      <c r="Y30" s="10"/>
-      <c r="Z30" s="10"/>
-    </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A31" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="E31" s="7">
-        <v>65</v>
-      </c>
-      <c r="F31" s="7">
-        <v>65</v>
-      </c>
-      <c r="G31" s="7">
-        <v>92</v>
-      </c>
-      <c r="H31" s="9"/>
-      <c r="I31" s="10"/>
-      <c r="J31" s="7">
-        <v>3</v>
-      </c>
-      <c r="K31" s="7">
-        <v>3</v>
-      </c>
-      <c r="L31" s="7">
-        <v>4</v>
-      </c>
-      <c r="M31" s="7">
-        <v>6</v>
-      </c>
-      <c r="N31" s="7">
-        <v>7</v>
-      </c>
-      <c r="O31" s="7">
-        <v>11</v>
-      </c>
-      <c r="P31" s="7">
-        <v>15</v>
-      </c>
-      <c r="Q31" s="10"/>
-      <c r="R31" s="10"/>
-      <c r="S31" s="10"/>
-      <c r="T31" s="10"/>
-      <c r="U31" s="10"/>
-      <c r="V31" s="10"/>
-      <c r="W31" s="9"/>
-      <c r="X31" s="10"/>
-      <c r="Y31" s="10"/>
+      <c r="P31">
+        <v>20</v>
+      </c>
+      <c r="Q31">
+        <v>25</v>
+      </c>
+      <c r="R31">
+        <v>30</v>
+      </c>
+      <c r="Y31" s="14"/>
       <c r="Z31" s="10"/>
     </row>
     <row r="32" spans="1:26" x14ac:dyDescent="0.25">
@@ -11417,115 +11386,104 @@
       <c r="Z29" s="10"/>
     </row>
     <row r="30" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="18" t="s">
+        <v>166</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="C30" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="D30" s="18" t="s">
+        <v>211</v>
+      </c>
+      <c r="E30" s="18">
+        <v>65</v>
+      </c>
+      <c r="F30" s="18">
+        <v>65</v>
+      </c>
+      <c r="G30" s="18">
+        <v>92</v>
+      </c>
+      <c r="H30" s="18"/>
+      <c r="I30" s="18"/>
+      <c r="J30" s="18">
+        <v>3</v>
+      </c>
+      <c r="K30" s="18">
+        <v>4</v>
+      </c>
+      <c r="L30" s="18">
+        <v>5</v>
+      </c>
+      <c r="M30" s="18">
+        <v>8</v>
+      </c>
+      <c r="N30" s="18">
+        <v>11</v>
+      </c>
+      <c r="O30" s="18"/>
+      <c r="P30" s="18"/>
+      <c r="Q30" s="18"/>
+      <c r="R30" s="18"/>
+      <c r="S30" s="18"/>
+      <c r="T30" s="18"/>
+      <c r="U30" s="18"/>
+      <c r="V30" s="18"/>
+      <c r="W30" s="18"/>
+      <c r="X30" s="18"/>
+      <c r="Y30" s="19"/>
+      <c r="Z30" s="10"/>
+    </row>
+    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>164</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B31" t="s">
         <v>165</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C31" t="s">
         <v>163</v>
       </c>
-      <c r="D30" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="E30" s="7">
-        <v>65</v>
-      </c>
-      <c r="F30" s="7">
-        <v>65</v>
-      </c>
-      <c r="G30" s="7">
-        <v>92</v>
-      </c>
-      <c r="H30" s="9"/>
-      <c r="I30" s="10"/>
-      <c r="J30" s="7">
-        <v>3</v>
-      </c>
-      <c r="K30" s="7">
-        <v>3</v>
-      </c>
-      <c r="L30" s="7">
-        <v>4</v>
-      </c>
-      <c r="M30" s="7">
+      <c r="D31" t="s">
+        <v>211</v>
+      </c>
+      <c r="E31">
+        <v>70</v>
+      </c>
+      <c r="F31">
+        <v>70</v>
+      </c>
+      <c r="G31">
+        <v>96</v>
+      </c>
+      <c r="K31">
+        <v>4</v>
+      </c>
+      <c r="L31">
         <v>6</v>
       </c>
-      <c r="N30" s="7">
+      <c r="M31">
         <v>7</v>
       </c>
-      <c r="O30" s="7">
+      <c r="N31">
         <v>11</v>
       </c>
-      <c r="P30" s="7">
+      <c r="O31">
         <v>15</v>
       </c>
-      <c r="Q30" s="10"/>
-      <c r="R30" s="10"/>
-      <c r="S30" s="10"/>
-      <c r="T30" s="10"/>
-      <c r="U30" s="10"/>
-      <c r="V30" s="10"/>
-      <c r="W30" s="9"/>
-      <c r="X30" s="10"/>
-      <c r="Y30" s="10"/>
-      <c r="Z30" s="10"/>
-    </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A31" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="E31" s="7">
-        <v>65</v>
-      </c>
-      <c r="F31" s="7">
-        <v>65</v>
-      </c>
-      <c r="G31" s="7">
-        <v>92</v>
-      </c>
-      <c r="H31" s="9"/>
-      <c r="I31" s="10"/>
-      <c r="J31" s="7">
-        <v>3</v>
-      </c>
-      <c r="K31" s="7">
-        <v>3</v>
-      </c>
-      <c r="L31" s="7">
-        <v>4</v>
-      </c>
-      <c r="M31" s="7">
-        <v>6</v>
-      </c>
-      <c r="N31" s="7">
-        <v>7</v>
-      </c>
-      <c r="O31" s="7">
-        <v>11</v>
-      </c>
-      <c r="P31" s="7">
-        <v>15</v>
-      </c>
-      <c r="Q31" s="10"/>
-      <c r="R31" s="10"/>
-      <c r="S31" s="10"/>
-      <c r="T31" s="10"/>
-      <c r="U31" s="10"/>
-      <c r="V31" s="10"/>
-      <c r="W31" s="9"/>
-      <c r="X31" s="10"/>
-      <c r="Y31" s="10"/>
+      <c r="P31">
+        <v>20</v>
+      </c>
+      <c r="Q31">
+        <v>25</v>
+      </c>
+      <c r="R31">
+        <v>30</v>
+      </c>
+      <c r="Y31" s="14"/>
       <c r="Z31" s="10"/>
     </row>
     <row r="32" spans="1:26" x14ac:dyDescent="0.25">
@@ -18091,7 +18049,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -18403,10 +18361,10 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C30" s="7" t="s">
         <v>163</v>
@@ -18414,10 +18372,10 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C31" s="7" t="s">
         <v>163</v>
@@ -18510,6 +18468,11 @@
       <c r="C39" s="7" t="s">
         <v>183</v>
       </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" s="6"/>
+      <c r="B42" s="6"/>
+      <c r="C42" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -22478,7 +22441,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:Z39"/>
+  <dimension ref="A1:Y41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -22489,16 +22452,16 @@
     <col min="6" max="6" width="12.85546875" customWidth="1"/>
     <col min="7" max="7" width="13.140625" customWidth="1"/>
     <col min="8" max="8" width="8.140625" customWidth="1"/>
-    <col min="9" max="22" width="8" customWidth="1"/>
-    <col min="23" max="26" width="7" customWidth="1"/>
+    <col min="9" max="21" width="8" customWidth="1"/>
+    <col min="22" max="25" width="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>187</v>
       </c>
@@ -22524,61 +22487,58 @@
         <v>192</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>193</v>
+        <v>279</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>194</v>
+        <v>280</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="M3" s="5" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="N3" s="5" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>205</v>
-      </c>
-      <c r="V3" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="W3" s="8" t="s">
+      <c r="V3" s="8" t="s">
         <v>207</v>
       </c>
+      <c r="W3" s="5" t="s">
+        <v>208</v>
+      </c>
       <c r="X3" s="5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="Y3" s="5" t="s">
-        <v>209</v>
-      </c>
-      <c r="Z3" s="5" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>107</v>
       </c>
@@ -22600,24 +22560,24 @@
       <c r="G4">
         <v>92</v>
       </c>
+      <c r="K4">
+        <v>6</v>
+      </c>
       <c r="L4">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M4">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N4">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="O4">
-        <v>15</v>
-      </c>
-      <c r="P4">
         <v>20</v>
       </c>
-      <c r="Z4" s="14"/>
-    </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y4" s="14"/>
+    </row>
+    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>110</v>
       </c>
@@ -22639,24 +22599,24 @@
       <c r="G5">
         <v>92</v>
       </c>
+      <c r="K5">
+        <v>4</v>
+      </c>
       <c r="L5">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M5">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N5">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="O5">
-        <v>11</v>
-      </c>
-      <c r="P5">
         <v>15</v>
       </c>
-      <c r="Z5" s="14"/>
-    </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y5" s="14"/>
+    </row>
+    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>112</v>
       </c>
@@ -22679,47 +22639,44 @@
         <v>99</v>
       </c>
       <c r="J6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K6">
         <v>3</v>
       </c>
       <c r="L6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N6">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="O6">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="P6">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="Q6">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="R6">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="S6">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="T6">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="U6">
-        <v>35</v>
-      </c>
-      <c r="V6">
         <v>40</v>
       </c>
-      <c r="Z6" s="14"/>
-    </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y6" s="14"/>
+    </row>
+    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>114</v>
       </c>
@@ -22741,33 +22698,33 @@
       <c r="G7">
         <v>96</v>
       </c>
+      <c r="K7">
+        <v>4</v>
+      </c>
       <c r="L7">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N7">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="O7">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="P7">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="Q7">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="R7">
-        <v>25</v>
-      </c>
-      <c r="S7">
         <v>30</v>
       </c>
-      <c r="Z7" s="14"/>
-    </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y7" s="14"/>
+    </row>
+    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>115</v>
       </c>
@@ -22790,29 +22747,26 @@
         <v>92</v>
       </c>
       <c r="J8">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K8">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L8">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M8">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N8">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="O8">
-        <v>15</v>
-      </c>
-      <c r="P8">
         <v>20</v>
       </c>
-      <c r="Z8" s="14"/>
-    </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y8" s="14"/>
+    </row>
+    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>117</v>
       </c>
@@ -22834,30 +22788,30 @@
       <c r="G9">
         <v>96</v>
       </c>
+      <c r="L9">
+        <v>3</v>
+      </c>
       <c r="M9">
         <v>3</v>
       </c>
       <c r="N9">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="O9">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="P9">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q9">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="R9">
-        <v>15</v>
-      </c>
-      <c r="S9">
         <v>20</v>
       </c>
-      <c r="Z9" s="14"/>
-    </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y9" s="14"/>
+    </row>
+    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>119</v>
       </c>
@@ -22879,24 +22833,24 @@
       <c r="G10">
         <v>90</v>
       </c>
+      <c r="K10">
+        <v>3</v>
+      </c>
       <c r="L10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N10">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="O10">
-        <v>8</v>
-      </c>
-      <c r="P10">
         <v>11</v>
       </c>
-      <c r="Z10" s="14"/>
-    </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y10" s="14"/>
+    </row>
+    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>122</v>
       </c>
@@ -22925,26 +22879,23 @@
         <v>3</v>
       </c>
       <c r="J11">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K11">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L11">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M11">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N11">
-        <v>10</v>
-      </c>
-      <c r="O11">
         <v>15</v>
       </c>
-      <c r="Z11" s="14"/>
-    </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y11" s="14"/>
+    </row>
+    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>124</v>
       </c>
@@ -22970,26 +22921,23 @@
         <v>3</v>
       </c>
       <c r="K12">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L12">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M12">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N12">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="O12">
-        <v>11</v>
-      </c>
-      <c r="P12">
         <v>15</v>
       </c>
-      <c r="Z12" s="14"/>
-    </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y12" s="14"/>
+    </row>
+    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>126</v>
       </c>
@@ -23021,23 +22969,20 @@
         <v>3</v>
       </c>
       <c r="K13">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L13">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M13">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N13">
-        <v>7</v>
-      </c>
-      <c r="O13">
         <v>11</v>
       </c>
-      <c r="Z13" s="14"/>
-    </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y13" s="14"/>
+    </row>
+    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>128</v>
       </c>
@@ -23069,17 +23014,14 @@
         <v>2</v>
       </c>
       <c r="K14">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L14">
-        <v>3</v>
-      </c>
-      <c r="M14">
-        <v>4</v>
-      </c>
-      <c r="Z14" s="14"/>
-    </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+      <c r="Y14" s="14"/>
+    </row>
+    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>130</v>
       </c>
@@ -23105,26 +23047,23 @@
         <v>2</v>
       </c>
       <c r="K15">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L15">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M15">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N15">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="O15">
-        <v>8</v>
-      </c>
-      <c r="P15">
         <v>11</v>
       </c>
-      <c r="Z15" s="14"/>
-    </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y15" s="14"/>
+    </row>
+    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>132</v>
       </c>
@@ -23146,21 +23085,21 @@
       <c r="G16">
         <v>92</v>
       </c>
+      <c r="L16">
+        <v>6</v>
+      </c>
       <c r="M16">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N16">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="O16">
-        <v>11</v>
-      </c>
-      <c r="P16">
         <v>15</v>
       </c>
-      <c r="Z16" s="14"/>
-    </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y16" s="14"/>
+    </row>
+    <row r="17" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>135</v>
       </c>
@@ -23192,26 +23131,23 @@
         <v>3</v>
       </c>
       <c r="K17">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L17">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M17">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N17">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="O17">
-        <v>11</v>
-      </c>
-      <c r="P17">
         <v>15</v>
       </c>
-      <c r="Z17" s="14"/>
-    </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y17" s="14"/>
+    </row>
+    <row r="18" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>137</v>
       </c>
@@ -23240,29 +23176,26 @@
         <v>1</v>
       </c>
       <c r="J18">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K18">
         <v>3</v>
       </c>
       <c r="L18">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M18">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N18">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="O18">
-        <v>8</v>
-      </c>
-      <c r="P18">
         <v>11</v>
       </c>
-      <c r="Z18" s="14"/>
-    </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y18" s="14"/>
+    </row>
+    <row r="19" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>139</v>
       </c>
@@ -23284,30 +23217,30 @@
       <c r="G19">
         <v>96</v>
       </c>
+      <c r="L19">
+        <v>8</v>
+      </c>
       <c r="M19">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N19">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="O19">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="P19">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="Q19">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="R19">
-        <v>30</v>
-      </c>
-      <c r="S19">
         <v>35</v>
       </c>
-      <c r="Z19" s="14"/>
-    </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y19" s="14"/>
+    </row>
+    <row r="20" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>141</v>
       </c>
@@ -23329,27 +23262,27 @@
       <c r="G20">
         <v>96</v>
       </c>
+      <c r="L20">
+        <v>3</v>
+      </c>
       <c r="M20">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N20">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="O20">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="P20">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="Q20">
-        <v>15</v>
-      </c>
-      <c r="R20">
         <v>20</v>
       </c>
-      <c r="Z20" s="14"/>
-    </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y20" s="14"/>
+    </row>
+    <row r="21" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>143</v>
       </c>
@@ -23378,26 +23311,23 @@
         <v>1</v>
       </c>
       <c r="J21">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K21">
         <v>3</v>
       </c>
       <c r="L21">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M21">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N21">
-        <v>5</v>
-      </c>
-      <c r="O21">
         <v>8</v>
       </c>
-      <c r="Z21" s="14"/>
-    </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y21" s="14"/>
+    </row>
+    <row r="22" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>145</v>
       </c>
@@ -23419,30 +23349,30 @@
       <c r="G22">
         <v>96</v>
       </c>
+      <c r="L22">
+        <v>8</v>
+      </c>
       <c r="M22">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N22">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="O22">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="P22">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="Q22">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="R22">
-        <v>30</v>
-      </c>
-      <c r="S22">
         <v>35</v>
       </c>
-      <c r="Z22" s="14"/>
-    </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y22" s="14"/>
+    </row>
+    <row r="23" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>148</v>
       </c>
@@ -23464,30 +23394,30 @@
       <c r="G23">
         <v>96</v>
       </c>
+      <c r="L23">
+        <v>6</v>
+      </c>
       <c r="M23">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N23">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="O23">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="P23">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="Q23">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="R23">
-        <v>25</v>
-      </c>
-      <c r="S23">
         <v>30</v>
       </c>
-      <c r="Z23" s="14"/>
-    </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y23" s="14"/>
+    </row>
+    <row r="24" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>150</v>
       </c>
@@ -23509,39 +23439,39 @@
       <c r="G24">
         <v>99</v>
       </c>
+      <c r="L24">
+        <v>3</v>
+      </c>
       <c r="M24">
         <v>3</v>
       </c>
       <c r="N24">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="O24">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="P24">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="Q24">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="R24">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="S24">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="T24">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="U24">
-        <v>30</v>
-      </c>
-      <c r="V24">
         <v>35</v>
       </c>
-      <c r="Z24" s="14"/>
-    </row>
-    <row r="25" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y24" s="14"/>
+    </row>
+    <row r="25" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>152</v>
       </c>
@@ -23563,36 +23493,36 @@
       <c r="G25">
         <v>99</v>
       </c>
+      <c r="L25">
+        <v>3</v>
+      </c>
       <c r="M25">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N25">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="O25">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="P25">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="Q25">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="R25">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="S25">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="T25">
-        <v>30</v>
-      </c>
-      <c r="U25">
         <v>35</v>
       </c>
-      <c r="Z25" s="14"/>
-    </row>
-    <row r="26" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y25" s="14"/>
+    </row>
+    <row r="26" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>154</v>
       </c>
@@ -23614,30 +23544,30 @@
       <c r="G26">
         <v>96</v>
       </c>
+      <c r="L26">
+        <v>6</v>
+      </c>
       <c r="M26">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N26">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="O26">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="P26">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="Q26">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="R26">
-        <v>25</v>
-      </c>
-      <c r="S26">
         <v>30</v>
       </c>
-      <c r="Z26" s="14"/>
-    </row>
-    <row r="27" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y26" s="14"/>
+    </row>
+    <row r="27" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>156</v>
       </c>
@@ -23659,24 +23589,24 @@
       <c r="G27">
         <v>92</v>
       </c>
+      <c r="K27">
+        <v>6</v>
+      </c>
       <c r="L27">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M27">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N27">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="O27">
-        <v>15</v>
-      </c>
-      <c r="P27">
         <v>20</v>
       </c>
-      <c r="Z27" s="14"/>
-    </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y27" s="14"/>
+    </row>
+    <row r="28" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>159</v>
       </c>
@@ -23698,24 +23628,24 @@
       <c r="G28">
         <v>92</v>
       </c>
+      <c r="K28">
+        <v>6</v>
+      </c>
       <c r="L28">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M28">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N28">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="O28">
-        <v>15</v>
-      </c>
-      <c r="P28">
         <v>20</v>
       </c>
-      <c r="Z28" s="14"/>
-    </row>
-    <row r="29" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y28" s="14"/>
+    </row>
+    <row r="29" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>161</v>
       </c>
@@ -23737,44 +23667,44 @@
       <c r="G29">
         <v>99</v>
       </c>
+      <c r="L29">
+        <v>4</v>
+      </c>
       <c r="M29">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N29">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="O29">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="P29">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="Q29">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="R29">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="S29">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="T29">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="U29">
-        <v>35</v>
-      </c>
-      <c r="V29">
         <v>40</v>
       </c>
-      <c r="Z29" s="14"/>
-    </row>
-    <row r="30" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y29" s="14"/>
+    </row>
+    <row r="30" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B30" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C30" t="s">
         <v>163</v>
@@ -23783,46 +23713,37 @@
         <v>211</v>
       </c>
       <c r="E30">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="F30">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="G30">
-        <v>96</v>
+        <v>92</v>
+      </c>
+      <c r="J30">
+        <v>3</v>
+      </c>
+      <c r="K30">
+        <v>4</v>
       </c>
       <c r="L30">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M30">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="N30">
-        <v>7</v>
-      </c>
-      <c r="O30">
         <v>11</v>
       </c>
-      <c r="P30">
-        <v>15</v>
-      </c>
-      <c r="Q30">
-        <v>20</v>
-      </c>
-      <c r="R30">
-        <v>25</v>
-      </c>
-      <c r="S30">
-        <v>30</v>
-      </c>
-      <c r="Z30" s="14"/>
-    </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y30" s="14"/>
+    </row>
+    <row r="31" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B31" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C31" t="s">
         <v>163</v>
@@ -23831,35 +23752,41 @@
         <v>211</v>
       </c>
       <c r="E31">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="F31">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="G31">
-        <v>92</v>
-      </c>
-      <c r="J31">
-        <v>2</v>
+        <v>96</v>
       </c>
       <c r="K31">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L31">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M31">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N31">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="O31">
-        <v>11</v>
-      </c>
-      <c r="Z31" s="14"/>
-    </row>
-    <row r="32" spans="1:26" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="P31">
+        <v>20</v>
+      </c>
+      <c r="Q31">
+        <v>25</v>
+      </c>
+      <c r="R31">
+        <v>30</v>
+      </c>
+      <c r="Y31" s="14"/>
+    </row>
+    <row r="32" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>168</v>
       </c>
@@ -23885,32 +23812,29 @@
         <v>2</v>
       </c>
       <c r="K32">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L32">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M32">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N32">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="O32">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="P32">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="Q32">
-        <v>15</v>
-      </c>
-      <c r="R32">
         <v>20</v>
       </c>
-      <c r="Z32" s="14"/>
-    </row>
-    <row r="33" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y32" s="14"/>
+    </row>
+    <row r="33" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>170</v>
       </c>
@@ -23932,9 +23856,9 @@
       <c r="G33">
         <v>1</v>
       </c>
-      <c r="Z33" s="14"/>
-    </row>
-    <row r="34" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y33" s="14"/>
+    </row>
+    <row r="34" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>173</v>
       </c>
@@ -23956,9 +23880,9 @@
       <c r="G34">
         <v>1</v>
       </c>
-      <c r="Z34" s="14"/>
-    </row>
-    <row r="35" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y34" s="14"/>
+    </row>
+    <row r="35" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>175</v>
       </c>
@@ -23980,9 +23904,9 @@
       <c r="G35">
         <v>1</v>
       </c>
-      <c r="Z35" s="14"/>
-    </row>
-    <row r="36" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y35" s="14"/>
+    </row>
+    <row r="36" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>177</v>
       </c>
@@ -24004,9 +23928,9 @@
       <c r="G36">
         <v>1</v>
       </c>
-      <c r="Z36" s="14"/>
-    </row>
-    <row r="37" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y36" s="14"/>
+    </row>
+    <row r="37" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>179</v>
       </c>
@@ -24028,9 +23952,9 @@
       <c r="G37">
         <v>1</v>
       </c>
-      <c r="Z37" s="14"/>
-    </row>
-    <row r="38" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y37" s="14"/>
+    </row>
+    <row r="38" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>181</v>
       </c>
@@ -24052,15 +23976,15 @@
       <c r="G38">
         <v>4</v>
       </c>
+      <c r="W38">
+        <v>10</v>
+      </c>
       <c r="X38">
-        <v>10</v>
-      </c>
-      <c r="Y38">
         <v>20</v>
       </c>
-      <c r="Z38" s="14"/>
-    </row>
-    <row r="39" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="Y38" s="14"/>
+    </row>
+    <row r="39" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>184</v>
       </c>
@@ -24082,10 +24006,13 @@
       <c r="G39">
         <v>4</v>
       </c>
-      <c r="Y39">
+      <c r="X39">
         <v>25</v>
       </c>
-      <c r="Z39" s="14"/>
+      <c r="Y39" s="14"/>
+    </row>
+    <row r="41" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="Y41" s="14"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -25689,121 +25616,104 @@
       <c r="Z29" s="10"/>
     </row>
     <row r="30" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="18" t="s">
+        <v>166</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="C30" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="D30" s="18" t="s">
+        <v>211</v>
+      </c>
+      <c r="E30" s="18">
+        <v>65</v>
+      </c>
+      <c r="F30" s="18">
+        <v>65</v>
+      </c>
+      <c r="G30" s="18">
+        <v>92</v>
+      </c>
+      <c r="H30" s="18"/>
+      <c r="I30" s="18"/>
+      <c r="J30" s="18">
+        <v>3</v>
+      </c>
+      <c r="K30" s="18">
+        <v>4</v>
+      </c>
+      <c r="L30" s="18">
+        <v>5</v>
+      </c>
+      <c r="M30" s="18">
+        <v>8</v>
+      </c>
+      <c r="N30" s="18">
+        <v>11</v>
+      </c>
+      <c r="O30" s="18"/>
+      <c r="P30" s="18"/>
+      <c r="Q30" s="18"/>
+      <c r="R30" s="18"/>
+      <c r="S30" s="18"/>
+      <c r="T30" s="18"/>
+      <c r="U30" s="18"/>
+      <c r="V30" s="18"/>
+      <c r="W30" s="18"/>
+      <c r="X30" s="18"/>
+      <c r="Y30" s="19"/>
+      <c r="Z30" s="10"/>
+    </row>
+    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>164</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B31" t="s">
         <v>165</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C31" t="s">
         <v>163</v>
       </c>
-      <c r="D30" s="6" t="s">
-        <v>212</v>
-      </c>
-      <c r="E30" s="7">
-        <v>75</v>
-      </c>
-      <c r="F30" s="7">
-        <v>75</v>
-      </c>
-      <c r="G30" s="7">
-        <v>99</v>
-      </c>
-      <c r="H30" s="9"/>
-      <c r="I30" s="10"/>
-      <c r="J30" s="10"/>
-      <c r="K30" s="10"/>
-      <c r="L30" s="10"/>
-      <c r="M30" s="7">
-        <v>3</v>
-      </c>
-      <c r="N30" s="7">
-        <v>3</v>
-      </c>
-      <c r="O30" s="7">
+      <c r="D31" t="s">
+        <v>211</v>
+      </c>
+      <c r="E31">
+        <v>70</v>
+      </c>
+      <c r="F31">
+        <v>70</v>
+      </c>
+      <c r="G31">
+        <v>96</v>
+      </c>
+      <c r="K31">
+        <v>4</v>
+      </c>
+      <c r="L31">
         <v>6</v>
       </c>
-      <c r="P30" s="7">
-        <v>8</v>
-      </c>
-      <c r="Q30" s="7">
-        <v>10</v>
-      </c>
-      <c r="R30" s="7">
+      <c r="M31">
+        <v>7</v>
+      </c>
+      <c r="N31">
+        <v>11</v>
+      </c>
+      <c r="O31">
         <v>15</v>
       </c>
-      <c r="S30" s="7">
+      <c r="P31">
         <v>20</v>
       </c>
-      <c r="T30" s="7">
+      <c r="Q31">
         <v>25</v>
       </c>
-      <c r="U30" s="7">
+      <c r="R31">
         <v>30</v>
       </c>
-      <c r="V30" s="7">
-        <v>35</v>
-      </c>
-      <c r="W30" s="9"/>
-      <c r="X30" s="10"/>
-      <c r="Y30" s="10"/>
-      <c r="Z30" s="10"/>
-    </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A31" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="E31" s="7">
-        <v>65</v>
-      </c>
-      <c r="F31" s="7">
-        <v>65</v>
-      </c>
-      <c r="G31" s="7">
-        <v>92</v>
-      </c>
-      <c r="H31" s="9"/>
-      <c r="I31" s="10"/>
-      <c r="J31" s="7">
-        <v>3</v>
-      </c>
-      <c r="K31" s="7">
-        <v>3</v>
-      </c>
-      <c r="L31" s="7">
-        <v>4</v>
-      </c>
-      <c r="M31" s="7">
-        <v>6</v>
-      </c>
-      <c r="N31" s="7">
-        <v>7</v>
-      </c>
-      <c r="O31" s="7">
-        <v>11</v>
-      </c>
-      <c r="P31" s="7">
-        <v>15</v>
-      </c>
-      <c r="Q31" s="10"/>
-      <c r="R31" s="10"/>
-      <c r="S31" s="10"/>
-      <c r="T31" s="10"/>
-      <c r="U31" s="10"/>
-      <c r="V31" s="10"/>
-      <c r="W31" s="9"/>
-      <c r="X31" s="10"/>
-      <c r="Y31" s="10"/>
+      <c r="Y31" s="14"/>
       <c r="Z31" s="10"/>
     </row>
     <row r="32" spans="1:26" x14ac:dyDescent="0.25">
@@ -27765,121 +27675,104 @@
       <c r="Z29" s="10"/>
     </row>
     <row r="30" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="18" t="s">
+        <v>166</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="C30" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="D30" s="18" t="s">
+        <v>211</v>
+      </c>
+      <c r="E30" s="18">
+        <v>65</v>
+      </c>
+      <c r="F30" s="18">
+        <v>65</v>
+      </c>
+      <c r="G30" s="18">
+        <v>92</v>
+      </c>
+      <c r="H30" s="18"/>
+      <c r="I30" s="18"/>
+      <c r="J30" s="18">
+        <v>3</v>
+      </c>
+      <c r="K30" s="18">
+        <v>4</v>
+      </c>
+      <c r="L30" s="18">
+        <v>5</v>
+      </c>
+      <c r="M30" s="18">
+        <v>8</v>
+      </c>
+      <c r="N30" s="18">
+        <v>11</v>
+      </c>
+      <c r="O30" s="18"/>
+      <c r="P30" s="18"/>
+      <c r="Q30" s="18"/>
+      <c r="R30" s="18"/>
+      <c r="S30" s="18"/>
+      <c r="T30" s="18"/>
+      <c r="U30" s="18"/>
+      <c r="V30" s="18"/>
+      <c r="W30" s="18"/>
+      <c r="X30" s="18"/>
+      <c r="Y30" s="19"/>
+      <c r="Z30" s="10"/>
+    </row>
+    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>164</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B31" t="s">
         <v>165</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C31" t="s">
         <v>163</v>
       </c>
-      <c r="D30" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="E30" s="7">
-        <v>65</v>
-      </c>
-      <c r="F30" s="7">
-        <v>65</v>
-      </c>
-      <c r="G30" s="7">
-        <v>92</v>
-      </c>
-      <c r="H30" s="9"/>
-      <c r="I30" s="10"/>
-      <c r="J30" s="7">
-        <v>3</v>
-      </c>
-      <c r="K30" s="7">
-        <v>3</v>
-      </c>
-      <c r="L30" s="7">
-        <v>4</v>
-      </c>
-      <c r="M30" s="7">
+      <c r="D31" t="s">
+        <v>211</v>
+      </c>
+      <c r="E31">
+        <v>70</v>
+      </c>
+      <c r="F31">
+        <v>70</v>
+      </c>
+      <c r="G31">
+        <v>96</v>
+      </c>
+      <c r="K31">
+        <v>4</v>
+      </c>
+      <c r="L31">
         <v>6</v>
       </c>
-      <c r="N30" s="7">
+      <c r="M31">
         <v>7</v>
       </c>
-      <c r="O30" s="7">
+      <c r="N31">
         <v>11</v>
       </c>
-      <c r="P30" s="7">
+      <c r="O31">
         <v>15</v>
       </c>
-      <c r="Q30" s="10"/>
-      <c r="R30" s="10"/>
-      <c r="S30" s="10"/>
-      <c r="T30" s="10"/>
-      <c r="U30" s="10"/>
-      <c r="V30" s="10"/>
-      <c r="W30" s="9"/>
-      <c r="X30" s="10"/>
-      <c r="Y30" s="10"/>
-      <c r="Z30" s="10"/>
-    </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A31" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>212</v>
-      </c>
-      <c r="E31" s="7">
-        <v>75</v>
-      </c>
-      <c r="F31" s="7">
-        <v>75</v>
-      </c>
-      <c r="G31" s="7">
-        <v>99</v>
-      </c>
-      <c r="H31" s="9"/>
-      <c r="I31" s="10"/>
-      <c r="J31" s="10"/>
-      <c r="K31" s="10"/>
-      <c r="L31" s="10"/>
-      <c r="M31" s="7">
-        <v>3</v>
-      </c>
-      <c r="N31" s="7">
-        <v>3</v>
-      </c>
-      <c r="O31" s="7">
-        <v>6</v>
-      </c>
-      <c r="P31" s="7">
-        <v>8</v>
-      </c>
-      <c r="Q31" s="7">
-        <v>10</v>
-      </c>
-      <c r="R31" s="7">
-        <v>15</v>
-      </c>
-      <c r="S31" s="7">
+      <c r="P31">
         <v>20</v>
       </c>
-      <c r="T31" s="7">
+      <c r="Q31">
         <v>25</v>
       </c>
-      <c r="U31" s="7">
+      <c r="R31">
         <v>30</v>
       </c>
-      <c r="V31" s="7">
-        <v>35</v>
-      </c>
-      <c r="W31" s="9"/>
-      <c r="X31" s="10"/>
-      <c r="Y31" s="10"/>
+      <c r="Y31" s="14"/>
       <c r="Z31" s="10"/>
     </row>
     <row r="32" spans="1:26" x14ac:dyDescent="0.25">
@@ -29836,121 +29729,104 @@
       <c r="Z29" s="10"/>
     </row>
     <row r="30" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="18" t="s">
+        <v>166</v>
+      </c>
+      <c r="B30" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="C30" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="D30" s="18" t="s">
+        <v>211</v>
+      </c>
+      <c r="E30" s="18">
+        <v>65</v>
+      </c>
+      <c r="F30" s="18">
+        <v>65</v>
+      </c>
+      <c r="G30" s="18">
+        <v>92</v>
+      </c>
+      <c r="H30" s="18"/>
+      <c r="I30" s="18"/>
+      <c r="J30" s="18">
+        <v>3</v>
+      </c>
+      <c r="K30" s="18">
+        <v>4</v>
+      </c>
+      <c r="L30" s="18">
+        <v>5</v>
+      </c>
+      <c r="M30" s="18">
+        <v>8</v>
+      </c>
+      <c r="N30" s="18">
+        <v>11</v>
+      </c>
+      <c r="O30" s="18"/>
+      <c r="P30" s="18"/>
+      <c r="Q30" s="18"/>
+      <c r="R30" s="18"/>
+      <c r="S30" s="18"/>
+      <c r="T30" s="18"/>
+      <c r="U30" s="18"/>
+      <c r="V30" s="18"/>
+      <c r="W30" s="18"/>
+      <c r="X30" s="18"/>
+      <c r="Y30" s="19"/>
+      <c r="Z30" s="10"/>
+    </row>
+    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>164</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B31" t="s">
         <v>165</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C31" t="s">
         <v>163</v>
       </c>
-      <c r="D30" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="E30" s="7">
-        <v>65</v>
-      </c>
-      <c r="F30" s="7">
-        <v>65</v>
-      </c>
-      <c r="G30" s="7">
-        <v>92</v>
-      </c>
-      <c r="H30" s="9"/>
-      <c r="I30" s="10"/>
-      <c r="J30" s="7">
-        <v>3</v>
-      </c>
-      <c r="K30" s="7">
-        <v>3</v>
-      </c>
-      <c r="L30" s="7">
-        <v>4</v>
-      </c>
-      <c r="M30" s="7">
+      <c r="D31" t="s">
+        <v>211</v>
+      </c>
+      <c r="E31">
+        <v>70</v>
+      </c>
+      <c r="F31">
+        <v>70</v>
+      </c>
+      <c r="G31">
+        <v>96</v>
+      </c>
+      <c r="K31">
+        <v>4</v>
+      </c>
+      <c r="L31">
         <v>6</v>
       </c>
-      <c r="N30" s="7">
+      <c r="M31">
         <v>7</v>
       </c>
-      <c r="O30" s="7">
+      <c r="N31">
         <v>11</v>
       </c>
-      <c r="P30" s="7">
+      <c r="O31">
         <v>15</v>
       </c>
-      <c r="Q30" s="10"/>
-      <c r="R30" s="10"/>
-      <c r="S30" s="10"/>
-      <c r="T30" s="10"/>
-      <c r="U30" s="10"/>
-      <c r="V30" s="10"/>
-      <c r="W30" s="9"/>
-      <c r="X30" s="10"/>
-      <c r="Y30" s="10"/>
-      <c r="Z30" s="10"/>
-    </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A31" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>212</v>
-      </c>
-      <c r="E31" s="7">
-        <v>75</v>
-      </c>
-      <c r="F31" s="7">
-        <v>75</v>
-      </c>
-      <c r="G31" s="7">
-        <v>99</v>
-      </c>
-      <c r="H31" s="9"/>
-      <c r="I31" s="10"/>
-      <c r="J31" s="10"/>
-      <c r="K31" s="10"/>
-      <c r="L31" s="10"/>
-      <c r="M31" s="7">
-        <v>3</v>
-      </c>
-      <c r="N31" s="7">
-        <v>3</v>
-      </c>
-      <c r="O31" s="7">
-        <v>6</v>
-      </c>
-      <c r="P31" s="7">
-        <v>8</v>
-      </c>
-      <c r="Q31" s="7">
-        <v>10</v>
-      </c>
-      <c r="R31" s="7">
-        <v>15</v>
-      </c>
-      <c r="S31" s="7">
+      <c r="P31">
         <v>20</v>
       </c>
-      <c r="T31" s="7">
+      <c r="Q31">
         <v>25</v>
       </c>
-      <c r="U31" s="7">
+      <c r="R31">
         <v>30</v>
       </c>
-      <c r="V31" s="7">
-        <v>35</v>
-      </c>
-      <c r="W31" s="9"/>
-      <c r="X31" s="10"/>
-      <c r="Y31" s="10"/>
+      <c r="Y31" s="14"/>
       <c r="Z31" s="10"/>
     </row>
     <row r="32" spans="1:26" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
ajout coté informatif pour les playstyles gris
</commit_message>
<xml_diff>
--- a/data/fc27-data.xlsx
+++ b/data/fc27-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexi\Desktop\Projets\builderproclubs\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{797BC33C-B528-42FD-8965-D858287F81EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{590780C4-0CB7-4D14-8AF9-3E9A57491093}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="692" firstSheet="1" activeTab="18" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="692" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lisez-moi" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2779" uniqueCount="340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2790" uniqueCount="347">
   <si>
     <t>Base de données — FC 27 Constructeur de build</t>
   </si>
@@ -1072,13 +1072,34 @@
   </si>
   <si>
     <t>Spécialisations</t>
+  </si>
+  <si>
+    <t>Traqueur</t>
+  </si>
+  <si>
+    <t>Trouble-fête</t>
+  </si>
+  <si>
+    <t>Récupérateur</t>
+  </si>
+  <si>
+    <t>Créateur</t>
+  </si>
+  <si>
+    <t>Étincelle</t>
+  </si>
+  <si>
+    <t>Magicien</t>
+  </si>
+  <si>
+    <t>Finisseur</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1119,6 +1140,17 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF434343"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF434343"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="7">
@@ -1197,7 +1229,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1231,52 +1263,50 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="25">
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
+        <b/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -1292,6 +1322,50 @@
         <scheme val="minor"/>
       </font>
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color rgb="FFBFBFBF"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="9"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF1F3446"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color rgb="FFBFBFBF"/>
+        </left>
+        <right style="thin">
+          <color rgb="FFBFBFBF"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -1453,82 +1527,8 @@
       </border>
     </dxf>
     <dxf>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color rgb="FFBFBFBF"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="9"/>
-        <color rgb="FFFFFFFF"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF1F3446"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color rgb="FFBFBFBF"/>
-        </left>
-        <right style="thin">
-          <color rgb="FFBFBFBF"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
+        <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -1544,6 +1544,24 @@
         <scheme val="minor"/>
       </font>
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1593,36 +1611,36 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{CC3F8001-1B73-43A9-94C9-BB5696F6479C}" name="Table2" displayName="Table2" ref="A1:I47" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{CC3F8001-1B73-43A9-94C9-BB5696F6479C}" name="Table2" displayName="Table2" ref="A1:I47" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
   <autoFilter ref="A1:I47" xr:uid="{CC3F8001-1B73-43A9-94C9-BB5696F6479C}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{4D8515F7-FCFC-4D0B-9E2E-ED020872A71E}" name="Column1" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{E1CE08EB-FD8F-4FDB-812F-62051DED4309}" name="Column2" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{1DDE626F-8446-4AAA-BAEC-91B9F295FBAF}" name="Column3" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{3A478CDF-C161-49FB-8433-DF67E340241C}" name="Column4" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{A2E41BA0-F3DF-4321-AEEC-F420E91FB4FA}" name="Column5" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{2F504979-EEC5-4973-A536-5F5E9EF6946D}" name="Column6" dataDxfId="17"/>
-    <tableColumn id="7" xr3:uid="{E317D236-B058-448C-9911-BB25C087ABEC}" name="Column7" dataDxfId="16"/>
-    <tableColumn id="8" xr3:uid="{B7A64CF3-41C2-4B56-A413-99AB7CE2C76D}" name="Column8" dataDxfId="15"/>
-    <tableColumn id="9" xr3:uid="{A123165B-4CC7-4FFA-B6C1-808173D9747D}" name="Column9" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{4D8515F7-FCFC-4D0B-9E2E-ED020872A71E}" name="Column1" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{E1CE08EB-FD8F-4FDB-812F-62051DED4309}" name="Column2" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{1DDE626F-8446-4AAA-BAEC-91B9F295FBAF}" name="Column3" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{3A478CDF-C161-49FB-8433-DF67E340241C}" name="Column4" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{A2E41BA0-F3DF-4321-AEEC-F420E91FB4FA}" name="Column5" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{2F504979-EEC5-4973-A536-5F5E9EF6946D}" name="Column6" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{E317D236-B058-448C-9911-BB25C087ABEC}" name="Column7" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{B7A64CF3-41C2-4B56-A413-99AB7CE2C76D}" name="Column8" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{A123165B-4CC7-4FFA-B6C1-808173D9747D}" name="Column9" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6A81EE77-924D-4A27-95C1-CE9387CD8489}" name="Table3" displayName="Table3" ref="A3:I47" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1" tableBorderDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6A81EE77-924D-4A27-95C1-CE9387CD8489}" name="Table3" displayName="Table3" ref="A3:I47" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23" tableBorderDxfId="22">
   <autoFilter ref="A3:I47" xr:uid="{6A81EE77-924D-4A27-95C1-CE9387CD8489}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{12AC2442-EFF1-4896-9682-029BD4855046}" name="archetype"/>
-    <tableColumn id="2" xr3:uid="{B0F8B123-2089-4583-98A2-1995CD85B977}" name="specialisation" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{D6662864-025C-46A1-8303-CE0241C67FAC}" name="archetype_gagne" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{097C53EC-F167-40A0-88C4-6CEFF6FF8BCE}" name="attribut_1" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{E92A705B-E623-4A97-8682-9EC30D60A096}" name="seuil_1" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{BF3FD942-E38F-4482-BCB6-E799211ADE0D}" name="attribut_2" dataDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{056E39F8-4575-4903-82BA-79D150ED3762}" name="seuil_2" dataDxfId="4"/>
-    <tableColumn id="8" xr3:uid="{EAE8CCB1-E087-4202-8112-99A7DBD7D58B}" name="attribut_3" dataDxfId="3"/>
-    <tableColumn id="9" xr3:uid="{105A4E71-173F-44F1-B3FE-A54F63DAC055}" name="seuil_3" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{B0F8B123-2089-4583-98A2-1995CD85B977}" name="specialisation" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{D6662864-025C-46A1-8303-CE0241C67FAC}" name="archetype_gagne" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{097C53EC-F167-40A0-88C4-6CEFF6FF8BCE}" name="attribut_1" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{E92A705B-E623-4A97-8682-9EC30D60A096}" name="seuil_1" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{BF3FD942-E38F-4482-BCB6-E799211ADE0D}" name="attribut_2" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{056E39F8-4575-4903-82BA-79D150ED3762}" name="seuil_2" dataDxfId="16"/>
+    <tableColumn id="8" xr3:uid="{EAE8CCB1-E087-4202-8112-99A7DBD7D58B}" name="attribut_3" dataDxfId="15"/>
+    <tableColumn id="9" xr3:uid="{105A4E71-173F-44F1-B3FE-A54F63DAC055}" name="seuil_3" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -15226,207 +15244,207 @@
       <c r="A3" s="13" t="s">
         <v>214</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" t="s">
         <v>328</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" t="s">
         <v>329</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" t="s">
         <v>226</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" t="s">
         <v>227</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" t="s">
         <v>228</v>
       </c>
-      <c r="G3" s="19" t="s">
+      <c r="G3" t="s">
         <v>229</v>
       </c>
-      <c r="H3" s="19" t="s">
+      <c r="H3" t="s">
         <v>230</v>
       </c>
-      <c r="I3" s="19" t="s">
+      <c r="I3" t="s">
         <v>231</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="B4" s="20" t="s">
         <v>269</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="20" t="s">
         <v>270</v>
       </c>
-      <c r="D4" s="21"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="22"/>
-      <c r="H4" s="21"/>
-      <c r="I4" s="22"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="18"/>
+      <c r="H4" s="20"/>
+      <c r="I4" s="18"/>
     </row>
     <row r="5" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B5" s="23" t="s">
+      <c r="B5" s="16" t="s">
         <v>271</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="C5" s="16" t="s">
         <v>272</v>
       </c>
-      <c r="D5" s="23" t="s">
+      <c r="D5" s="16" t="s">
         <v>131</v>
       </c>
-      <c r="E5" s="24">
+      <c r="E5" s="14">
         <v>90</v>
       </c>
-      <c r="F5" s="23" t="s">
+      <c r="F5" s="16" t="s">
         <v>140</v>
       </c>
-      <c r="G5" s="24">
+      <c r="G5" s="14">
         <v>90</v>
       </c>
-      <c r="H5" s="23" t="s">
+      <c r="H5" s="16" t="s">
         <v>142</v>
       </c>
-      <c r="I5" s="24">
+      <c r="I5" s="14">
         <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="20" t="s">
         <v>273</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="C6" s="20" t="s">
         <v>274</v>
       </c>
-      <c r="D6" s="21" t="s">
+      <c r="D6" s="20" t="s">
         <v>131</v>
       </c>
-      <c r="E6" s="22">
+      <c r="E6" s="18">
         <v>90</v>
       </c>
-      <c r="F6" s="21" t="s">
+      <c r="F6" s="20" t="s">
         <v>129</v>
       </c>
-      <c r="G6" s="22">
+      <c r="G6" s="18">
         <v>90</v>
       </c>
-      <c r="H6" s="21" t="s">
+      <c r="H6" s="20" t="s">
         <v>105</v>
       </c>
-      <c r="I6" s="22">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="I6" s="18">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="23" t="s">
+      <c r="B7" s="16" t="s">
         <v>275</v>
       </c>
-      <c r="C7" s="23" t="s">
+      <c r="C7" s="16" t="s">
         <v>276</v>
       </c>
-      <c r="D7" s="23" t="s">
+      <c r="D7" s="16" t="s">
         <v>149</v>
       </c>
-      <c r="E7" s="24">
+      <c r="E7" s="14">
         <v>90</v>
       </c>
-      <c r="F7" s="23" t="s">
+      <c r="F7" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="G7" s="24">
+      <c r="G7" s="14">
         <v>90</v>
       </c>
-      <c r="H7" s="23" t="s">
+      <c r="H7" s="16" t="s">
         <v>146</v>
       </c>
-      <c r="I7" s="24">
+      <c r="I7" s="14">
         <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="20" t="s">
+      <c r="A8" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="B8" s="20" t="s">
         <v>269</v>
       </c>
-      <c r="C8" s="21" t="s">
+      <c r="C8" s="20" t="s">
         <v>277</v>
       </c>
-      <c r="D8" s="21"/>
-      <c r="E8" s="22"/>
-      <c r="F8" s="21"/>
-      <c r="G8" s="22"/>
-      <c r="H8" s="21"/>
-      <c r="I8" s="22"/>
-    </row>
-    <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="D8" s="20"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="20"/>
+      <c r="I8" s="18"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="16" t="s">
         <v>278</v>
       </c>
-      <c r="C9" s="23" t="s">
+      <c r="C9" s="16" t="s">
         <v>279</v>
       </c>
-      <c r="D9" s="23" t="s">
+      <c r="D9" s="16" t="s">
         <v>154</v>
       </c>
-      <c r="E9" s="24">
+      <c r="E9" s="14">
         <v>90</v>
       </c>
-      <c r="F9" s="23" t="s">
+      <c r="F9" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="G9" s="24">
+      <c r="G9" s="14">
         <v>90</v>
       </c>
-      <c r="H9" s="23" t="s">
+      <c r="H9" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="I9" s="24">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" ht="60" x14ac:dyDescent="0.25">
-      <c r="A10" s="20" t="s">
+      <c r="I9" s="14">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="20" t="s">
         <v>265</v>
       </c>
-      <c r="C10" s="21" t="s">
+      <c r="C10" s="20" t="s">
         <v>280</v>
       </c>
-      <c r="D10" s="21" t="s">
+      <c r="D10" s="20" t="s">
         <v>107</v>
       </c>
-      <c r="E10" s="22">
-        <v>92</v>
-      </c>
-      <c r="F10" s="21" t="s">
+      <c r="E10" s="18">
+        <v>92</v>
+      </c>
+      <c r="F10" s="20" t="s">
         <v>122</v>
       </c>
-      <c r="G10" s="22">
+      <c r="G10" s="18">
         <v>90</v>
       </c>
-      <c r="H10" s="21" t="s">
+      <c r="H10" s="20" t="s">
         <v>104</v>
       </c>
-      <c r="I10" s="22">
+      <c r="I10" s="18">
         <v>90</v>
       </c>
     </row>
@@ -15434,103 +15452,103 @@
       <c r="A11" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="16" t="s">
         <v>281</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="C11" s="16" t="s">
         <v>282</v>
       </c>
-      <c r="D11" s="23" t="s">
+      <c r="D11" s="16" t="s">
         <v>140</v>
       </c>
-      <c r="E11" s="24">
-        <v>92</v>
-      </c>
-      <c r="F11" s="23" t="s">
+      <c r="E11" s="14">
+        <v>92</v>
+      </c>
+      <c r="F11" s="16" t="s">
         <v>102</v>
       </c>
-      <c r="G11" s="24">
+      <c r="G11" s="14">
         <v>90</v>
       </c>
-      <c r="H11" s="23" t="s">
+      <c r="H11" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="I11" s="24">
+      <c r="I11" s="14">
         <v>90</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" s="20" t="s">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="B12" s="21" t="s">
+      <c r="B12" s="20" t="s">
         <v>269</v>
       </c>
-      <c r="C12" s="21" t="s">
+      <c r="C12" s="20" t="s">
         <v>276</v>
       </c>
-      <c r="D12" s="21"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="21"/>
-      <c r="G12" s="22"/>
-      <c r="H12" s="21"/>
-      <c r="I12" s="22"/>
-    </row>
-    <row r="13" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="D12" s="20"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="20"/>
+      <c r="I12" s="18"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B13" s="23" t="s">
+      <c r="B13" s="16" t="s">
         <v>283</v>
       </c>
-      <c r="C13" s="23" t="s">
+      <c r="C13" s="16" t="s">
         <v>279</v>
       </c>
-      <c r="D13" s="23" t="s">
+      <c r="D13" s="16" t="s">
         <v>149</v>
       </c>
-      <c r="E13" s="24">
-        <v>92</v>
-      </c>
-      <c r="F13" s="23" t="s">
+      <c r="E13" s="14">
+        <v>92</v>
+      </c>
+      <c r="F13" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="G13" s="24">
+      <c r="G13" s="14">
         <v>90</v>
       </c>
-      <c r="H13" s="23" t="s">
+      <c r="H13" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="I13" s="24">
+      <c r="I13" s="14">
         <v>90</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="20" t="s">
+      <c r="A14" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="B14" s="21" t="s">
+      <c r="B14" s="20" t="s">
         <v>284</v>
       </c>
-      <c r="C14" s="21" t="s">
+      <c r="C14" s="20" t="s">
         <v>285</v>
       </c>
-      <c r="D14" s="21" t="s">
+      <c r="D14" s="20" t="s">
         <v>105</v>
       </c>
-      <c r="E14" s="22">
+      <c r="E14" s="18">
         <v>90</v>
       </c>
-      <c r="F14" s="21" t="s">
+      <c r="F14" s="20" t="s">
         <v>149</v>
       </c>
-      <c r="G14" s="22">
-        <v>92</v>
-      </c>
-      <c r="H14" s="21" t="s">
+      <c r="G14" s="18">
+        <v>92</v>
+      </c>
+      <c r="H14" s="20" t="s">
         <v>146</v>
       </c>
-      <c r="I14" s="22">
+      <c r="I14" s="18">
         <v>90</v>
       </c>
     </row>
@@ -15538,103 +15556,103 @@
       <c r="A15" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B15" s="23" t="s">
+      <c r="B15" s="16" t="s">
         <v>286</v>
       </c>
-      <c r="C15" s="23" t="s">
+      <c r="C15" s="16" t="s">
         <v>277</v>
       </c>
-      <c r="D15" s="23" t="s">
+      <c r="D15" s="16" t="s">
         <v>154</v>
       </c>
-      <c r="E15" s="24">
-        <v>92</v>
-      </c>
-      <c r="F15" s="23" t="s">
+      <c r="E15" s="14">
+        <v>92</v>
+      </c>
+      <c r="F15" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="G15" s="24">
+      <c r="G15" s="14">
         <v>90</v>
       </c>
-      <c r="H15" s="23" t="s">
+      <c r="H15" s="16" t="s">
         <v>140</v>
       </c>
-      <c r="I15" s="24">
+      <c r="I15" s="14">
         <v>90</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="20" t="s">
+      <c r="A16" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="B16" s="21" t="s">
+      <c r="B16" s="20" t="s">
         <v>269</v>
       </c>
-      <c r="C16" s="21" t="s">
+      <c r="C16" s="20" t="s">
         <v>272</v>
       </c>
-      <c r="D16" s="21"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="21"/>
-      <c r="G16" s="22"/>
-      <c r="H16" s="21"/>
-      <c r="I16" s="22"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="18"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="18"/>
+      <c r="H16" s="20"/>
+      <c r="I16" s="18"/>
     </row>
     <row r="17" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B17" s="23" t="s">
+      <c r="B17" s="16" t="s">
         <v>287</v>
       </c>
-      <c r="C17" s="23" t="s">
+      <c r="C17" s="16" t="s">
         <v>288</v>
       </c>
-      <c r="D17" s="23" t="s">
+      <c r="D17" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="E17" s="24">
+      <c r="E17" s="14">
         <v>90</v>
       </c>
-      <c r="F17" s="23" t="s">
+      <c r="F17" s="16" t="s">
         <v>102</v>
       </c>
-      <c r="G17" s="24">
+      <c r="G17" s="14">
         <v>90</v>
       </c>
-      <c r="H17" s="23" t="s">
+      <c r="H17" s="16" t="s">
         <v>135</v>
       </c>
-      <c r="I17" s="24">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="20" t="s">
+      <c r="I17" s="14">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="B18" s="21" t="s">
+      <c r="B18" s="20" t="s">
         <v>289</v>
       </c>
-      <c r="C18" s="21" t="s">
+      <c r="C18" s="20" t="s">
         <v>279</v>
       </c>
-      <c r="D18" s="21" t="s">
+      <c r="D18" s="20" t="s">
         <v>149</v>
       </c>
-      <c r="E18" s="22">
+      <c r="E18" s="18">
         <v>90</v>
       </c>
-      <c r="F18" s="21" t="s">
+      <c r="F18" s="20" t="s">
         <v>154</v>
       </c>
-      <c r="G18" s="22">
-        <v>92</v>
-      </c>
-      <c r="H18" s="21" t="s">
+      <c r="G18" s="18">
+        <v>92</v>
+      </c>
+      <c r="H18" s="20" t="s">
         <v>144</v>
       </c>
-      <c r="I18" s="22">
+      <c r="I18" s="18">
         <v>90</v>
       </c>
     </row>
@@ -15642,103 +15660,103 @@
       <c r="A19" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B19" s="23" t="s">
+      <c r="B19" s="16" t="s">
         <v>290</v>
       </c>
-      <c r="C19" s="23" t="s">
+      <c r="C19" s="16" t="s">
         <v>277</v>
       </c>
-      <c r="D19" s="23" t="s">
+      <c r="D19" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="E19" s="24">
+      <c r="E19" s="14">
         <v>90</v>
       </c>
-      <c r="F19" s="23" t="s">
+      <c r="F19" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="G19" s="24">
+      <c r="G19" s="14">
         <v>90</v>
       </c>
-      <c r="H19" s="23" t="s">
+      <c r="H19" s="16" t="s">
         <v>129</v>
       </c>
-      <c r="I19" s="24">
+      <c r="I19" s="14">
         <v>92</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="20" t="s">
+      <c r="A20" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="B20" s="21" t="s">
+      <c r="B20" s="20" t="s">
         <v>269</v>
       </c>
-      <c r="C20" s="21" t="s">
+      <c r="C20" s="20" t="s">
         <v>288</v>
       </c>
-      <c r="D20" s="21"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="21"/>
-      <c r="G20" s="22"/>
-      <c r="H20" s="21"/>
-      <c r="I20" s="22"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="18"/>
+      <c r="F20" s="20"/>
+      <c r="G20" s="18"/>
+      <c r="H20" s="20"/>
+      <c r="I20" s="18"/>
     </row>
     <row r="21" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="B21" s="23" t="s">
+      <c r="B21" s="16" t="s">
         <v>291</v>
       </c>
-      <c r="C21" s="23" t="s">
+      <c r="C21" s="16" t="s">
         <v>274</v>
       </c>
-      <c r="D21" s="23" t="s">
+      <c r="D21" s="16" t="s">
         <v>154</v>
       </c>
-      <c r="E21" s="24">
+      <c r="E21" s="14">
         <v>90</v>
       </c>
-      <c r="F21" s="23" t="s">
+      <c r="F21" s="16" t="s">
         <v>131</v>
       </c>
-      <c r="G21" s="24">
+      <c r="G21" s="14">
         <v>90</v>
       </c>
-      <c r="H21" s="23" t="s">
+      <c r="H21" s="16" t="s">
         <v>129</v>
       </c>
-      <c r="I21" s="24">
+      <c r="I21" s="14">
         <v>92</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="A22" s="20" t="s">
+      <c r="A22" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="B22" s="21" t="s">
+      <c r="B22" s="20" t="s">
         <v>292</v>
       </c>
-      <c r="C22" s="21" t="s">
+      <c r="C22" s="20" t="s">
         <v>293</v>
       </c>
-      <c r="D22" s="21" t="s">
+      <c r="D22" s="20" t="s">
         <v>149</v>
       </c>
-      <c r="E22" s="22">
+      <c r="E22" s="18">
         <v>90</v>
       </c>
-      <c r="F22" s="21" t="s">
+      <c r="F22" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="G22" s="22">
-        <v>92</v>
-      </c>
-      <c r="H22" s="21" t="s">
+      <c r="G22" s="18">
+        <v>92</v>
+      </c>
+      <c r="H22" s="20" t="s">
         <v>154</v>
       </c>
-      <c r="I22" s="22">
+      <c r="I22" s="18">
         <v>90</v>
       </c>
     </row>
@@ -15746,103 +15764,103 @@
       <c r="A23" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="B23" s="23" t="s">
+      <c r="B23" s="16" t="s">
         <v>294</v>
       </c>
-      <c r="C23" s="23" t="s">
+      <c r="C23" s="16" t="s">
         <v>295</v>
       </c>
-      <c r="D23" s="23" t="s">
+      <c r="D23" s="16" t="s">
         <v>135</v>
       </c>
-      <c r="E23" s="24">
+      <c r="E23" s="14">
         <v>90</v>
       </c>
-      <c r="F23" s="23" t="s">
+      <c r="F23" s="16" t="s">
         <v>140</v>
       </c>
-      <c r="G23" s="24">
+      <c r="G23" s="14">
         <v>90</v>
       </c>
-      <c r="H23" s="23" t="s">
+      <c r="H23" s="16" t="s">
         <v>142</v>
       </c>
-      <c r="I23" s="24">
+      <c r="I23" s="14">
         <v>92</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A24" s="20" t="s">
+      <c r="A24" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="B24" s="21" t="s">
+      <c r="B24" s="20" t="s">
         <v>269</v>
       </c>
-      <c r="C24" s="21" t="s">
+      <c r="C24" s="20" t="s">
         <v>274</v>
       </c>
-      <c r="D24" s="21"/>
-      <c r="E24" s="22"/>
-      <c r="F24" s="21"/>
-      <c r="G24" s="22"/>
-      <c r="H24" s="21"/>
-      <c r="I24" s="22"/>
+      <c r="D24" s="20"/>
+      <c r="E24" s="18"/>
+      <c r="F24" s="20"/>
+      <c r="G24" s="18"/>
+      <c r="H24" s="20"/>
+      <c r="I24" s="18"/>
     </row>
     <row r="25" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B25" s="23" t="s">
+      <c r="B25" s="16" t="s">
         <v>296</v>
       </c>
-      <c r="C25" s="23" t="s">
+      <c r="C25" s="16" t="s">
         <v>297</v>
       </c>
-      <c r="D25" s="23" t="s">
+      <c r="D25" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="E25" s="24">
+      <c r="E25" s="14">
         <v>90</v>
       </c>
-      <c r="F25" s="23" t="s">
+      <c r="F25" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="G25" s="24">
-        <v>92</v>
-      </c>
-      <c r="H25" s="23" t="s">
+      <c r="G25" s="14">
+        <v>92</v>
+      </c>
+      <c r="H25" s="16" t="s">
         <v>105</v>
       </c>
-      <c r="I25" s="24">
+      <c r="I25" s="14">
         <v>90</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A26" s="20" t="s">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="B26" s="21" t="s">
+      <c r="B26" s="20" t="s">
         <v>298</v>
       </c>
-      <c r="C26" s="21" t="s">
+      <c r="C26" s="20" t="s">
         <v>299</v>
       </c>
-      <c r="D26" s="21" t="s">
+      <c r="D26" s="20" t="s">
         <v>112</v>
       </c>
-      <c r="E26" s="22">
+      <c r="E26" s="18">
         <v>90</v>
       </c>
-      <c r="F26" s="21" t="s">
+      <c r="F26" s="20" t="s">
         <v>104</v>
       </c>
-      <c r="G26" s="22">
+      <c r="G26" s="18">
         <v>90</v>
       </c>
-      <c r="H26" s="21" t="s">
+      <c r="H26" s="20" t="s">
         <v>107</v>
       </c>
-      <c r="I26" s="22">
+      <c r="I26" s="18">
         <v>92</v>
       </c>
     </row>
@@ -15850,311 +15868,311 @@
       <c r="A27" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B27" s="23" t="s">
+      <c r="B27" s="16" t="s">
         <v>300</v>
       </c>
-      <c r="C27" s="23" t="s">
+      <c r="C27" s="16" t="s">
         <v>301</v>
       </c>
-      <c r="D27" s="23" t="s">
+      <c r="D27" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="E27" s="24">
-        <v>92</v>
-      </c>
-      <c r="F27" s="23" t="s">
+      <c r="E27" s="14">
+        <v>92</v>
+      </c>
+      <c r="F27" s="16" t="s">
         <v>156</v>
       </c>
-      <c r="G27" s="24">
+      <c r="G27" s="14">
         <v>90</v>
       </c>
-      <c r="H27" s="23" t="s">
+      <c r="H27" s="16" t="s">
         <v>158</v>
       </c>
-      <c r="I27" s="24">
+      <c r="I27" s="14">
         <v>90</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A28" s="20" t="s">
+      <c r="A28" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="B28" s="21" t="s">
+      <c r="B28" s="20" t="s">
         <v>269</v>
       </c>
-      <c r="C28" s="21" t="s">
+      <c r="C28" s="20" t="s">
         <v>302</v>
       </c>
-      <c r="D28" s="21"/>
-      <c r="E28" s="22"/>
-      <c r="F28" s="21"/>
-      <c r="G28" s="22"/>
-      <c r="H28" s="21"/>
-      <c r="I28" s="22"/>
-    </row>
-    <row r="29" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="D28" s="20"/>
+      <c r="E28" s="18"/>
+      <c r="F28" s="20"/>
+      <c r="G28" s="18"/>
+      <c r="H28" s="20"/>
+      <c r="I28" s="18"/>
+    </row>
+    <row r="29" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="B29" s="23" t="s">
+      <c r="B29" s="16" t="s">
         <v>303</v>
       </c>
-      <c r="C29" s="23" t="s">
+      <c r="C29" s="16" t="s">
         <v>304</v>
       </c>
-      <c r="D29" s="23" t="s">
+      <c r="D29" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="E29" s="24">
-        <v>92</v>
-      </c>
-      <c r="F29" s="23" t="s">
+      <c r="E29" s="14">
+        <v>92</v>
+      </c>
+      <c r="F29" s="16" t="s">
         <v>125</v>
       </c>
-      <c r="G29" s="24">
+      <c r="G29" s="14">
         <v>90</v>
       </c>
-      <c r="H29" s="23" t="s">
+      <c r="H29" s="16" t="s">
         <v>131</v>
       </c>
-      <c r="I29" s="24">
+      <c r="I29" s="14">
         <v>90</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="A30" s="20" t="s">
+    <row r="30" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A30" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="B30" s="21" t="s">
+      <c r="B30" s="20" t="s">
         <v>305</v>
       </c>
-      <c r="C30" s="21" t="s">
+      <c r="C30" s="20" t="s">
         <v>306</v>
       </c>
-      <c r="D30" s="21" t="s">
+      <c r="D30" s="20" t="s">
         <v>125</v>
       </c>
-      <c r="E30" s="22">
-        <v>92</v>
-      </c>
-      <c r="F30" s="21" t="s">
+      <c r="E30" s="18">
+        <v>92</v>
+      </c>
+      <c r="F30" s="20" t="s">
         <v>127</v>
       </c>
-      <c r="G30" s="22">
+      <c r="G30" s="18">
         <v>90</v>
       </c>
-      <c r="H30" s="21" t="s">
+      <c r="H30" s="20" t="s">
         <v>114</v>
       </c>
-      <c r="I30" s="22">
+      <c r="I30" s="18">
         <v>90</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="B31" s="23" t="s">
+      <c r="B31" s="16" t="s">
         <v>307</v>
       </c>
-      <c r="C31" s="23" t="s">
+      <c r="C31" s="16" t="s">
         <v>308</v>
       </c>
-      <c r="D31" s="23" t="s">
+      <c r="D31" s="16" t="s">
         <v>112</v>
       </c>
-      <c r="E31" s="24">
+      <c r="E31" s="14">
         <v>90</v>
       </c>
-      <c r="F31" s="23" t="s">
+      <c r="F31" s="16" t="s">
         <v>114</v>
       </c>
-      <c r="G31" s="24">
-        <v>92</v>
-      </c>
-      <c r="H31" s="23" t="s">
+      <c r="G31" s="14">
+        <v>92</v>
+      </c>
+      <c r="H31" s="16" t="s">
         <v>116</v>
       </c>
-      <c r="I31" s="24">
+      <c r="I31" s="14">
         <v>90</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A32" s="20" t="s">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="B32" s="21" t="s">
+      <c r="B32" s="20" t="s">
         <v>269</v>
       </c>
-      <c r="C32" s="21" t="s">
+      <c r="C32" s="20" t="s">
         <v>309</v>
       </c>
-      <c r="D32" s="21"/>
-      <c r="E32" s="22"/>
-      <c r="F32" s="21"/>
-      <c r="G32" s="22"/>
-      <c r="H32" s="21"/>
-      <c r="I32" s="22"/>
-    </row>
-    <row r="33" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="D32" s="20"/>
+      <c r="E32" s="18"/>
+      <c r="F32" s="20"/>
+      <c r="G32" s="18"/>
+      <c r="H32" s="20"/>
+      <c r="I32" s="18"/>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B33" s="23" t="s">
+      <c r="B33" s="16" t="s">
         <v>310</v>
       </c>
-      <c r="C33" s="23" t="s">
+      <c r="C33" s="16" t="s">
         <v>276</v>
       </c>
-      <c r="D33" s="23" t="s">
+      <c r="D33" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="E33" s="24">
-        <v>92</v>
-      </c>
-      <c r="F33" s="23" t="s">
+      <c r="E33" s="14">
+        <v>92</v>
+      </c>
+      <c r="F33" s="16" t="s">
         <v>149</v>
       </c>
-      <c r="G33" s="24">
+      <c r="G33" s="14">
         <v>90</v>
       </c>
-      <c r="H33" s="23" t="s">
+      <c r="H33" s="16" t="s">
         <v>146</v>
       </c>
-      <c r="I33" s="24">
+      <c r="I33" s="14">
         <v>90</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="A34" s="20" t="s">
+    <row r="34" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A34" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="B34" s="21" t="s">
+      <c r="B34" s="20" t="s">
         <v>311</v>
       </c>
-      <c r="C34" s="21" t="s">
+      <c r="C34" s="20" t="s">
         <v>304</v>
       </c>
-      <c r="D34" s="21" t="s">
+      <c r="D34" s="20" t="s">
         <v>109</v>
       </c>
-      <c r="E34" s="22">
+      <c r="E34" s="18">
         <v>90</v>
       </c>
-      <c r="F34" s="21" t="s">
+      <c r="F34" s="20" t="s">
         <v>125</v>
       </c>
-      <c r="G34" s="22">
-        <v>92</v>
-      </c>
-      <c r="H34" s="21" t="s">
+      <c r="G34" s="18">
+        <v>92</v>
+      </c>
+      <c r="H34" s="20" t="s">
         <v>131</v>
       </c>
-      <c r="I34" s="22">
+      <c r="I34" s="18">
         <v>90</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="B35" s="23" t="s">
+      <c r="B35" s="16" t="s">
         <v>312</v>
       </c>
-      <c r="C35" s="23" t="s">
+      <c r="C35" s="16" t="s">
         <v>313</v>
       </c>
-      <c r="D35" s="23" t="s">
+      <c r="D35" s="16" t="s">
         <v>102</v>
       </c>
-      <c r="E35" s="24">
+      <c r="E35" s="14">
         <v>90</v>
       </c>
-      <c r="F35" s="23" t="s">
+      <c r="F35" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="G35" s="24">
+      <c r="G35" s="14">
         <v>90</v>
       </c>
-      <c r="H35" s="23" t="s">
+      <c r="H35" s="16" t="s">
         <v>112</v>
       </c>
-      <c r="I35" s="24">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A36" s="20" t="s">
+      <c r="I35" s="14">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A36" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="B36" s="21" t="s">
+      <c r="B36" s="20" t="s">
         <v>269</v>
       </c>
-      <c r="C36" s="21" t="s">
+      <c r="C36" s="20" t="s">
         <v>297</v>
       </c>
-      <c r="D36" s="21"/>
-      <c r="E36" s="22"/>
-      <c r="F36" s="21"/>
-      <c r="G36" s="22"/>
-      <c r="H36" s="21"/>
-      <c r="I36" s="22"/>
-    </row>
-    <row r="37" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="D36" s="20"/>
+      <c r="E36" s="18"/>
+      <c r="F36" s="20"/>
+      <c r="G36" s="18"/>
+      <c r="H36" s="20"/>
+      <c r="I36" s="18"/>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="B37" s="23" t="s">
+      <c r="B37" s="16" t="s">
         <v>314</v>
       </c>
-      <c r="C37" s="23" t="s">
+      <c r="C37" s="16" t="s">
         <v>299</v>
       </c>
-      <c r="D37" s="23" t="s">
+      <c r="D37" s="16" t="s">
         <v>146</v>
       </c>
-      <c r="E37" s="24">
+      <c r="E37" s="14">
         <v>90</v>
       </c>
-      <c r="F37" s="23" t="s">
+      <c r="F37" s="16" t="s">
         <v>107</v>
       </c>
-      <c r="G37" s="24">
+      <c r="G37" s="14">
         <v>90</v>
       </c>
-      <c r="H37" s="23" t="s">
+      <c r="H37" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="I37" s="24">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="A38" s="20" t="s">
+      <c r="I37" s="14">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A38" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="B38" s="21" t="s">
+      <c r="B38" s="20" t="s">
         <v>315</v>
       </c>
-      <c r="C38" s="21" t="s">
+      <c r="C38" s="20" t="s">
         <v>308</v>
       </c>
-      <c r="D38" s="21" t="s">
+      <c r="D38" s="20" t="s">
         <v>112</v>
       </c>
-      <c r="E38" s="22">
+      <c r="E38" s="18">
         <v>90</v>
       </c>
-      <c r="F38" s="21" t="s">
+      <c r="F38" s="20" t="s">
         <v>114</v>
       </c>
-      <c r="G38" s="22">
-        <v>92</v>
-      </c>
-      <c r="H38" s="21" t="s">
+      <c r="G38" s="18">
+        <v>92</v>
+      </c>
+      <c r="H38" s="20" t="s">
         <v>116</v>
       </c>
-      <c r="I38" s="22">
+      <c r="I38" s="18">
         <v>90</v>
       </c>
     </row>
@@ -16162,236 +16180,236 @@
       <c r="A39" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="B39" s="23" t="s">
+      <c r="B39" s="16" t="s">
         <v>316</v>
       </c>
-      <c r="C39" s="23" t="s">
+      <c r="C39" s="16" t="s">
         <v>302</v>
       </c>
-      <c r="D39" s="23" t="s">
+      <c r="D39" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="E39" s="24">
+      <c r="E39" s="14">
         <v>90</v>
       </c>
-      <c r="F39" s="23" t="s">
+      <c r="F39" s="16" t="s">
         <v>122</v>
       </c>
-      <c r="G39" s="24">
+      <c r="G39" s="14">
         <v>90</v>
       </c>
-      <c r="H39" s="23" t="s">
+      <c r="H39" s="16" t="s">
         <v>131</v>
       </c>
-      <c r="I39" s="24">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A40" s="20" t="s">
+      <c r="I39" s="14">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A40" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="B40" s="21" t="s">
+      <c r="B40" s="20" t="s">
         <v>269</v>
       </c>
-      <c r="C40" s="21" t="s">
+      <c r="C40" s="20" t="s">
         <v>317</v>
       </c>
-      <c r="D40" s="21"/>
-      <c r="E40" s="22"/>
-      <c r="F40" s="21"/>
-      <c r="G40" s="22"/>
-      <c r="H40" s="21"/>
-      <c r="I40" s="22"/>
-    </row>
-    <row r="41" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="D40" s="20"/>
+      <c r="E40" s="18"/>
+      <c r="F40" s="20"/>
+      <c r="G40" s="18"/>
+      <c r="H40" s="20"/>
+      <c r="I40" s="18"/>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="B41" s="23" t="s">
+      <c r="B41" s="16" t="s">
         <v>318</v>
       </c>
-      <c r="C41" s="23" t="s">
+      <c r="C41" s="16" t="s">
         <v>313</v>
       </c>
-      <c r="D41" s="23" t="s">
+      <c r="D41" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="E41" s="24">
+      <c r="E41" s="14">
         <v>90</v>
       </c>
-      <c r="F41" s="23" t="s">
+      <c r="F41" s="16" t="s">
         <v>107</v>
       </c>
-      <c r="G41" s="24">
-        <v>92</v>
-      </c>
-      <c r="H41" s="23" t="s">
+      <c r="G41" s="14">
+        <v>92</v>
+      </c>
+      <c r="H41" s="16" t="s">
         <v>102</v>
       </c>
-      <c r="I41" s="24">
+      <c r="I41" s="14">
         <v>90</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A42" s="20" t="s">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A42" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="B42" s="21" t="s">
+      <c r="B42" s="20" t="s">
         <v>319</v>
       </c>
-      <c r="C42" s="21" t="s">
+      <c r="C42" s="20" t="s">
         <v>301</v>
       </c>
-      <c r="D42" s="21" t="s">
+      <c r="D42" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="E42" s="22">
+      <c r="E42" s="18">
         <v>90</v>
       </c>
-      <c r="F42" s="21" t="s">
+      <c r="F42" s="20" t="s">
         <v>156</v>
       </c>
-      <c r="G42" s="22">
-        <v>92</v>
-      </c>
-      <c r="H42" s="21" t="s">
+      <c r="G42" s="18">
+        <v>92</v>
+      </c>
+      <c r="H42" s="20" t="s">
         <v>158</v>
       </c>
-      <c r="I42" s="22">
+      <c r="I42" s="18">
         <v>90</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="B43" s="23" t="s">
+      <c r="B43" s="16" t="s">
         <v>320</v>
       </c>
-      <c r="C43" s="23" t="s">
+      <c r="C43" s="16" t="s">
         <v>321</v>
       </c>
-      <c r="D43" s="23" t="s">
+      <c r="D43" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="E43" s="24">
+      <c r="E43" s="14">
         <v>90</v>
       </c>
-      <c r="F43" s="23" t="s">
+      <c r="F43" s="16" t="s">
         <v>112</v>
       </c>
-      <c r="G43" s="24">
+      <c r="G43" s="14">
         <v>90</v>
       </c>
-      <c r="H43" s="23" t="s">
+      <c r="H43" s="16" t="s">
         <v>133</v>
       </c>
-      <c r="I43" s="24">
+      <c r="I43" s="14">
         <v>92</v>
       </c>
     </row>
     <row r="44" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A44" s="21" t="s">
+      <c r="A44" s="20" t="s">
         <v>322</v>
       </c>
-      <c r="B44" s="21" t="s">
+      <c r="B44" s="20" t="s">
         <v>269</v>
       </c>
-      <c r="C44" s="21" t="s">
+      <c r="C44" s="20" t="s">
         <v>323</v>
       </c>
-      <c r="D44" s="21"/>
-      <c r="E44" s="22"/>
-      <c r="F44" s="21"/>
-      <c r="G44" s="22"/>
-      <c r="H44" s="21"/>
-      <c r="I44" s="22"/>
+      <c r="D44" s="20"/>
+      <c r="E44" s="18"/>
+      <c r="F44" s="20"/>
+      <c r="G44" s="18"/>
+      <c r="H44" s="20"/>
+      <c r="I44" s="18"/>
     </row>
     <row r="45" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A45" s="23" t="s">
+      <c r="A45" s="16" t="s">
         <v>322</v>
       </c>
-      <c r="B45" s="23" t="s">
+      <c r="B45" s="16" t="s">
         <v>324</v>
       </c>
-      <c r="C45" s="23" t="s">
+      <c r="C45" s="16" t="s">
         <v>325</v>
       </c>
-      <c r="D45" s="23" t="s">
+      <c r="D45" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="E45" s="24">
+      <c r="E45" s="14">
         <v>90</v>
       </c>
-      <c r="F45" s="23" t="s">
+      <c r="F45" s="16" t="s">
         <v>151</v>
       </c>
-      <c r="G45" s="24">
-        <v>92</v>
-      </c>
-      <c r="H45" s="23" t="s">
+      <c r="G45" s="14">
+        <v>92</v>
+      </c>
+      <c r="H45" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="I45" s="24">
+      <c r="I45" s="14">
         <v>90</v>
       </c>
     </row>
     <row r="46" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A46" s="21" t="s">
+      <c r="A46" s="20" t="s">
         <v>322</v>
       </c>
-      <c r="B46" s="21" t="s">
+      <c r="B46" s="20" t="s">
         <v>326</v>
       </c>
-      <c r="C46" s="21" t="s">
+      <c r="C46" s="20" t="s">
         <v>302</v>
       </c>
-      <c r="D46" s="21" t="s">
+      <c r="D46" s="20" t="s">
         <v>122</v>
       </c>
-      <c r="E46" s="22">
+      <c r="E46" s="18">
         <v>90</v>
       </c>
-      <c r="F46" s="21" t="s">
+      <c r="F46" s="20" t="s">
         <v>131</v>
       </c>
-      <c r="G46" s="22">
+      <c r="G46" s="18">
         <v>90</v>
       </c>
-      <c r="H46" s="21" t="s">
+      <c r="H46" s="20" t="s">
         <v>129</v>
       </c>
-      <c r="I46" s="22">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="A47" s="25" t="s">
+      <c r="I46" s="18">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A47" s="16" t="s">
         <v>322</v>
       </c>
-      <c r="B47" s="25" t="s">
+      <c r="B47" s="16" t="s">
         <v>327</v>
       </c>
-      <c r="C47" s="25" t="s">
+      <c r="C47" s="16" t="s">
         <v>293</v>
       </c>
-      <c r="D47" s="25" t="s">
+      <c r="D47" s="16" t="s">
         <v>149</v>
       </c>
-      <c r="E47" s="26">
-        <v>92</v>
-      </c>
-      <c r="F47" s="25" t="s">
+      <c r="E47" s="14">
+        <v>92</v>
+      </c>
+      <c r="F47" s="16" t="s">
         <v>154</v>
       </c>
-      <c r="G47" s="26">
+      <c r="G47" s="14">
         <v>90</v>
       </c>
-      <c r="H47" s="25" t="s">
+      <c r="H47" s="16" t="s">
         <v>109</v>
       </c>
-      <c r="I47" s="26">
+      <c r="I47" s="14">
         <v>90</v>
       </c>
     </row>
@@ -16482,7 +16500,9 @@
       <c r="B6" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="7"/>
+      <c r="C6" s="21" t="s">
+        <v>33</v>
+      </c>
       <c r="D6" s="7" t="s">
         <v>33</v>
       </c>
@@ -16509,7 +16529,9 @@
       <c r="B7" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="C7" s="7"/>
+      <c r="C7" s="21" t="s">
+        <v>40</v>
+      </c>
       <c r="D7" s="7" t="s">
         <v>40</v>
       </c>
@@ -16536,7 +16558,9 @@
       <c r="B8" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="C8" s="7"/>
+      <c r="C8" s="22" t="s">
+        <v>340</v>
+      </c>
       <c r="D8" s="7" t="s">
         <v>45</v>
       </c>
@@ -16563,7 +16587,9 @@
       <c r="B9" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C9" s="7"/>
+      <c r="C9" s="22" t="s">
+        <v>341</v>
+      </c>
       <c r="D9" s="7" t="s">
         <v>51</v>
       </c>
@@ -16590,7 +16616,9 @@
       <c r="B10" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="C10" s="7"/>
+      <c r="C10" s="22" t="s">
+        <v>342</v>
+      </c>
       <c r="D10" s="7" t="s">
         <v>58</v>
       </c>
@@ -16617,7 +16645,9 @@
       <c r="B11" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="C11" s="7"/>
+      <c r="C11" s="22" t="s">
+        <v>64</v>
+      </c>
       <c r="D11" s="7" t="s">
         <v>64</v>
       </c>
@@ -16644,7 +16674,9 @@
       <c r="B12" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="C12" s="7"/>
+      <c r="C12" s="22" t="s">
+        <v>343</v>
+      </c>
       <c r="D12" s="7" t="s">
         <v>70</v>
       </c>
@@ -16671,7 +16703,9 @@
       <c r="B13" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="C13" s="7"/>
+      <c r="C13" s="22" t="s">
+        <v>344</v>
+      </c>
       <c r="D13" s="7" t="s">
         <v>76</v>
       </c>
@@ -16698,7 +16732,9 @@
       <c r="B14" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="C14" s="7"/>
+      <c r="C14" s="22" t="s">
+        <v>345</v>
+      </c>
       <c r="D14" s="7" t="s">
         <v>82</v>
       </c>
@@ -16725,7 +16761,9 @@
       <c r="B15" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="C15" s="7"/>
+      <c r="C15" s="22" t="s">
+        <v>346</v>
+      </c>
       <c r="D15" s="7" t="s">
         <v>87</v>
       </c>
@@ -16752,7 +16790,9 @@
       <c r="B16" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="C16" s="7"/>
+      <c r="C16" s="22" t="s">
+        <v>322</v>
+      </c>
       <c r="D16" s="7" t="s">
         <v>92</v>
       </c>

</xml_diff>

<commit_message>
vérif facilitateur et boss
</commit_message>
<xml_diff>
--- a/data/fc27-data.xlsx
+++ b/data/fc27-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexi\Desktop\Projets\builderproclubs\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC922586-0AA6-4655-9966-B5538CB2A1E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E225EA9-2F4F-489C-A574-7B67E659CBE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4710" yWindow="2070" windowWidth="28800" windowHeight="15300" tabRatio="692" firstSheet="1" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4710" yWindow="2070" windowWidth="28800" windowHeight="15300" tabRatio="692" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lisez-moi" sheetId="1" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2382" uniqueCount="411">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2384" uniqueCount="409">
   <si>
     <t>Base de données — FC 27 Constructeur de build</t>
   </si>
@@ -799,12 +799,6 @@
   </si>
   <si>
     <t>Forteresse aérienne</t>
-  </si>
-  <si>
-    <t>61-64</t>
-  </si>
-  <si>
-    <t>65-69</t>
   </si>
   <si>
     <t>Aucune</t>
@@ -1576,7 +1570,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1609,8 +1603,14 @@
         <bgColor theme="0" tint="-0.14999847407452621"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F3446"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -1772,11 +1772,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1846,6 +1859,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2391,9 +2407,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B25F6B7E-BDB4-4556-93D2-D823D0060FF6}" name="Table1" displayName="Table1" ref="A3:Y39" totalsRowShown="0" headerRowDxfId="24" headerRowBorderDxfId="23">
-  <autoFilter ref="A3:Y39" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
-  <tableColumns count="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B25F6B7E-BDB4-4556-93D2-D823D0060FF6}" name="Table1" displayName="Table1" ref="A3:Z39" totalsRowShown="0" headerRowDxfId="24" headerRowBorderDxfId="23">
+  <autoFilter ref="A3:Z39" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
+  <tableColumns count="26">
     <tableColumn id="1" xr3:uid="{EDC2B16E-8713-45EE-BE81-CDE8D764A76B}" name="attribut"/>
     <tableColumn id="2" xr3:uid="{3157AA01-579B-43D2-8D17-A25D980F28BC}" name="nom"/>
     <tableColumn id="3" xr3:uid="{27114B50-8405-4E8C-8DD1-B69EF2903F72}" name="categorie"/>
@@ -2402,23 +2418,24 @@
     <tableColumn id="6" xr3:uid="{B389CBC2-C9CD-4EA0-9CDB-9A7CE9443835}" name="limite_min"/>
     <tableColumn id="7" xr3:uid="{BF5EB726-211F-4EAB-8ACB-23D5C69CF0A9}" name="limite_max"/>
     <tableColumn id="8" xr3:uid="{35448435-384C-4432-9043-32D70AB74E83}" name="1-60"/>
-    <tableColumn id="9" xr3:uid="{EB7894A2-5261-491E-84A0-D8665EBA6661}" name="61-64"/>
-    <tableColumn id="11" xr3:uid="{EF63C3B4-6AB1-4407-A53A-15179A890598}" name="65-69"/>
-    <tableColumn id="12" xr3:uid="{CB92E0C8-A8AA-424D-97C5-AC3C04CD327C}" name="70-74"/>
-    <tableColumn id="13" xr3:uid="{86B602FA-60C5-4414-AB16-70F62753BADF}" name="75-79"/>
-    <tableColumn id="14" xr3:uid="{5100757D-B350-4AA4-991C-DADAB95F5E41}" name="80-84"/>
-    <tableColumn id="15" xr3:uid="{51B1C7C9-7D94-4954-872E-EFEE087E7251}" name="85-89"/>
-    <tableColumn id="16" xr3:uid="{7EB94AD7-6DA8-4314-A6D4-13E20D84F369}" name="90-92"/>
-    <tableColumn id="17" xr3:uid="{108A2761-76D1-41FC-8DAD-DE5C0BD2731A}" name="93-94"/>
-    <tableColumn id="18" xr3:uid="{A02D6A40-79CC-4695-A9C2-9FF62F9D859C}" name="95"/>
-    <tableColumn id="19" xr3:uid="{E6DC1908-AC0A-4802-BBB1-DA9F08429FCF}" name="96"/>
-    <tableColumn id="20" xr3:uid="{882E6237-3C96-400D-A634-769985CA8E26}" name="97"/>
-    <tableColumn id="21" xr3:uid="{BA361568-2509-4ECF-9965-69EA3644CBBC}" name="98"/>
-    <tableColumn id="22" xr3:uid="{A713FC84-A58F-42CA-8125-BDAC3307AB2D}" name="99"/>
-    <tableColumn id="23" xr3:uid="{810A57B1-2BBB-421B-8EA4-632D3E15F70C}" name="★2"/>
-    <tableColumn id="24" xr3:uid="{3E5E9002-3DBF-40CA-B760-E5447D15099C}" name="★3"/>
-    <tableColumn id="25" xr3:uid="{EDCE50E3-5CF3-4DB0-808E-79FF22DAEB16}" name="★4"/>
-    <tableColumn id="26" xr3:uid="{D835FEBD-D7A6-4665-864D-386375F3535B}" name="★5" dataDxfId="22"/>
+    <tableColumn id="9" xr3:uid="{EB7894A2-5261-491E-84A0-D8665EBA6661}" name="61-63"/>
+    <tableColumn id="11" xr3:uid="{EF63C3B4-6AB1-4407-A53A-15179A890598}" name="64-66"/>
+    <tableColumn id="12" xr3:uid="{CB92E0C8-A8AA-424D-97C5-AC3C04CD327C}" name="67-69"/>
+    <tableColumn id="13" xr3:uid="{86B602FA-60C5-4414-AB16-70F62753BADF}" name="70-74"/>
+    <tableColumn id="14" xr3:uid="{5100757D-B350-4AA4-991C-DADAB95F5E41}" name="75-79"/>
+    <tableColumn id="15" xr3:uid="{51B1C7C9-7D94-4954-872E-EFEE087E7251}" name="80-84"/>
+    <tableColumn id="16" xr3:uid="{7EB94AD7-6DA8-4314-A6D4-13E20D84F369}" name="85-89"/>
+    <tableColumn id="17" xr3:uid="{108A2761-76D1-41FC-8DAD-DE5C0BD2731A}" name="90-92"/>
+    <tableColumn id="18" xr3:uid="{A02D6A40-79CC-4695-A9C2-9FF62F9D859C}" name="93-94"/>
+    <tableColumn id="19" xr3:uid="{E6DC1908-AC0A-4802-BBB1-DA9F08429FCF}" name="95"/>
+    <tableColumn id="20" xr3:uid="{882E6237-3C96-400D-A634-769985CA8E26}" name="96"/>
+    <tableColumn id="21" xr3:uid="{BA361568-2509-4ECF-9965-69EA3644CBBC}" name="97"/>
+    <tableColumn id="22" xr3:uid="{A713FC84-A58F-42CA-8125-BDAC3307AB2D}" name="98"/>
+    <tableColumn id="23" xr3:uid="{810A57B1-2BBB-421B-8EA4-632D3E15F70C}" name="99"/>
+    <tableColumn id="24" xr3:uid="{3E5E9002-3DBF-40CA-B760-E5447D15099C}" name="★2"/>
+    <tableColumn id="25" xr3:uid="{EDCE50E3-5CF3-4DB0-808E-79FF22DAEB16}" name="★3"/>
+    <tableColumn id="26" xr3:uid="{D835FEBD-D7A6-4665-864D-386375F3535B}" name="★4" dataDxfId="22"/>
+    <tableColumn id="10" xr3:uid="{4A250526-90AB-4431-8E88-BB92E4E40DDB}" name="★5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3153,7 +3170,7 @@
         <v>104</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="C7" s="15" t="s">
         <v>99</v>
@@ -3323,7 +3340,7 @@
         <v>109</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="C10" s="15" t="s">
         <v>220</v>
@@ -3501,7 +3518,7 @@
         <v>116</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="C13" s="15" t="s">
         <v>220</v>
@@ -3688,7 +3705,7 @@
         <v>123</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>190</v>
@@ -3750,7 +3767,7 @@
         <v>126</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D17" s="15" t="s">
         <v>189</v>
@@ -3803,10 +3820,10 @@
         <v>127</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D18" s="15" t="s">
         <v>189</v>
@@ -3867,10 +3884,10 @@
         <v>129</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D19" s="15" t="s">
         <v>189</v>
@@ -3923,10 +3940,10 @@
         <v>131</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D20" s="15" t="s">
         <v>189</v>
@@ -3982,7 +3999,7 @@
         <v>134</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D21" s="15" t="s">
         <v>190</v>
@@ -4041,7 +4058,7 @@
         <v>135</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="C22" s="15" t="s">
         <v>137</v>
@@ -4099,7 +4116,7 @@
         <v>138</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="C23" s="15" t="s">
         <v>137</v>
@@ -4157,7 +4174,7 @@
         <v>140</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="C24" s="15" t="s">
         <v>137</v>
@@ -4215,7 +4232,7 @@
         <v>142</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="C25" s="15" t="s">
         <v>137</v>
@@ -4271,7 +4288,7 @@
         <v>144</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="C26" s="15" t="s">
         <v>137</v>
@@ -4331,7 +4348,7 @@
         <v>146</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="C27" s="15" t="s">
         <v>148</v>
@@ -4383,7 +4400,7 @@
         <v>149</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="C28" s="15" t="s">
         <v>148</v>
@@ -4626,7 +4643,9 @@
       <c r="G32" s="15">
         <v>92</v>
       </c>
-      <c r="H32" s="15"/>
+      <c r="H32" s="15">
+        <v>1</v>
+      </c>
       <c r="I32" s="15">
         <v>1</v>
       </c>
@@ -14246,8 +14265,12 @@
       <c r="F27" s="13">
         <v>75</v>
       </c>
-      <c r="G27" s="15"/>
-      <c r="H27" s="13"/>
+      <c r="G27" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="H27" s="13">
+        <v>80</v>
+      </c>
     </row>
     <row r="28" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="15" t="s">
@@ -14419,22 +14442,22 @@
     <row r="2" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:26" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="26" t="s">
+        <v>318</v>
+      </c>
+      <c r="B3" s="27" t="s">
+        <v>319</v>
+      </c>
+      <c r="C3" s="27" t="s">
         <v>320</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="D3" s="27" t="s">
         <v>321</v>
       </c>
-      <c r="C3" s="27" t="s">
+      <c r="E3" s="27" t="s">
         <v>322</v>
       </c>
-      <c r="D3" s="27" t="s">
+      <c r="F3" s="28" t="s">
         <v>323</v>
-      </c>
-      <c r="E3" s="27" t="s">
-        <v>324</v>
-      </c>
-      <c r="F3" s="28" t="s">
-        <v>325</v>
       </c>
       <c r="G3" s="22"/>
       <c r="H3" s="22"/>
@@ -14459,22 +14482,22 @@
     </row>
     <row r="4" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="24" t="s">
+        <v>324</v>
+      </c>
+      <c r="B4" s="22" t="s">
+        <v>325</v>
+      </c>
+      <c r="C4" s="22" t="s">
         <v>326</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="D4" s="22" t="s">
         <v>327</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="E4" s="22" t="s">
         <v>328</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="F4" s="25" t="s">
         <v>329</v>
-      </c>
-      <c r="E4" s="22" t="s">
-        <v>330</v>
-      </c>
-      <c r="F4" s="25" t="s">
-        <v>331</v>
       </c>
       <c r="G4" s="22"/>
       <c r="H4" s="22"/>
@@ -14499,22 +14522,22 @@
     </row>
     <row r="5" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="24" t="s">
+        <v>330</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>331</v>
+      </c>
+      <c r="C5" s="22" t="s">
         <v>332</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="D5" s="22" t="s">
         <v>333</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="E5" s="22" t="s">
         <v>334</v>
       </c>
-      <c r="D5" s="22" t="s">
+      <c r="F5" s="25" t="s">
         <v>335</v>
-      </c>
-      <c r="E5" s="22" t="s">
-        <v>336</v>
-      </c>
-      <c r="F5" s="25" t="s">
-        <v>337</v>
       </c>
       <c r="G5" s="22"/>
       <c r="H5" s="22"/>
@@ -14539,22 +14562,22 @@
     </row>
     <row r="6" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="24" t="s">
+        <v>336</v>
+      </c>
+      <c r="B6" s="22" t="s">
+        <v>337</v>
+      </c>
+      <c r="C6" s="22" t="s">
         <v>338</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="D6" s="22" t="s">
         <v>339</v>
       </c>
-      <c r="C6" s="22" t="s">
+      <c r="E6" s="22" t="s">
         <v>340</v>
       </c>
-      <c r="D6" s="22" t="s">
+      <c r="F6" s="25" t="s">
         <v>341</v>
-      </c>
-      <c r="E6" s="22" t="s">
-        <v>342</v>
-      </c>
-      <c r="F6" s="25" t="s">
-        <v>343</v>
       </c>
       <c r="G6" s="22"/>
       <c r="H6" s="22"/>
@@ -14579,22 +14602,22 @@
     </row>
     <row r="7" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="24" t="s">
+        <v>342</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>343</v>
+      </c>
+      <c r="C7" s="22" t="s">
         <v>344</v>
       </c>
-      <c r="B7" s="22" t="s">
+      <c r="D7" s="22" t="s">
         <v>345</v>
       </c>
-      <c r="C7" s="22" t="s">
+      <c r="E7" s="22" t="s">
         <v>346</v>
       </c>
-      <c r="D7" s="22" t="s">
+      <c r="F7" s="25" t="s">
         <v>347</v>
-      </c>
-      <c r="E7" s="22" t="s">
-        <v>348</v>
-      </c>
-      <c r="F7" s="25" t="s">
-        <v>349</v>
       </c>
       <c r="G7" s="22"/>
       <c r="H7" s="22"/>
@@ -14619,22 +14642,22 @@
     </row>
     <row r="8" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="24" t="s">
+        <v>348</v>
+      </c>
+      <c r="B8" s="22" t="s">
+        <v>349</v>
+      </c>
+      <c r="C8" s="22" t="s">
         <v>350</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="D8" s="22" t="s">
         <v>351</v>
       </c>
-      <c r="C8" s="22" t="s">
+      <c r="E8" s="22" t="s">
         <v>352</v>
       </c>
-      <c r="D8" s="22" t="s">
+      <c r="F8" s="25" t="s">
         <v>353</v>
-      </c>
-      <c r="E8" s="22" t="s">
-        <v>354</v>
-      </c>
-      <c r="F8" s="25" t="s">
-        <v>355</v>
       </c>
       <c r="G8" s="22"/>
       <c r="H8" s="22"/>
@@ -14659,22 +14682,22 @@
     </row>
     <row r="9" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="24" t="s">
+        <v>354</v>
+      </c>
+      <c r="B9" s="22" t="s">
+        <v>355</v>
+      </c>
+      <c r="C9" s="22" t="s">
         <v>356</v>
       </c>
-      <c r="B9" s="22" t="s">
+      <c r="D9" s="22" t="s">
         <v>357</v>
       </c>
-      <c r="C9" s="22" t="s">
+      <c r="E9" s="22" t="s">
         <v>358</v>
       </c>
-      <c r="D9" s="22" t="s">
+      <c r="F9" s="25" t="s">
         <v>359</v>
-      </c>
-      <c r="E9" s="22" t="s">
-        <v>360</v>
-      </c>
-      <c r="F9" s="25" t="s">
-        <v>361</v>
       </c>
       <c r="G9" s="22"/>
       <c r="H9" s="22"/>
@@ -14699,22 +14722,22 @@
     </row>
     <row r="10" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="24" t="s">
+        <v>360</v>
+      </c>
+      <c r="B10" s="22" t="s">
+        <v>361</v>
+      </c>
+      <c r="C10" s="22" t="s">
         <v>362</v>
       </c>
-      <c r="B10" s="22" t="s">
+      <c r="D10" s="22" t="s">
         <v>363</v>
       </c>
-      <c r="C10" s="22" t="s">
+      <c r="E10" s="22" t="s">
         <v>364</v>
       </c>
-      <c r="D10" s="22" t="s">
+      <c r="F10" s="25" t="s">
         <v>365</v>
-      </c>
-      <c r="E10" s="22" t="s">
-        <v>366</v>
-      </c>
-      <c r="F10" s="25" t="s">
-        <v>367</v>
       </c>
       <c r="G10" s="22"/>
       <c r="H10" s="22"/>
@@ -14739,22 +14762,22 @@
     </row>
     <row r="11" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="24" t="s">
+        <v>366</v>
+      </c>
+      <c r="B11" s="22" t="s">
+        <v>367</v>
+      </c>
+      <c r="C11" s="22" t="s">
         <v>368</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="D11" s="22" t="s">
         <v>369</v>
       </c>
-      <c r="C11" s="22" t="s">
+      <c r="E11" s="22" t="s">
         <v>370</v>
       </c>
-      <c r="D11" s="22" t="s">
+      <c r="F11" s="25" t="s">
         <v>371</v>
-      </c>
-      <c r="E11" s="22" t="s">
-        <v>372</v>
-      </c>
-      <c r="F11" s="25" t="s">
-        <v>373</v>
       </c>
       <c r="G11" s="22"/>
       <c r="H11" s="22"/>
@@ -14779,22 +14802,22 @@
     </row>
     <row r="12" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="29" t="s">
+        <v>372</v>
+      </c>
+      <c r="B12" s="30" t="s">
+        <v>373</v>
+      </c>
+      <c r="C12" s="30" t="s">
         <v>374</v>
       </c>
-      <c r="B12" s="30" t="s">
+      <c r="D12" s="30" t="s">
         <v>375</v>
       </c>
-      <c r="C12" s="30" t="s">
+      <c r="E12" s="30" t="s">
         <v>376</v>
       </c>
-      <c r="D12" s="30" t="s">
+      <c r="F12" s="31" t="s">
         <v>377</v>
-      </c>
-      <c r="E12" s="30" t="s">
-        <v>378</v>
-      </c>
-      <c r="F12" s="31" t="s">
-        <v>379</v>
       </c>
       <c r="G12" s="22"/>
       <c r="H12" s="22"/>
@@ -15136,7 +15159,7 @@
       <c r="H24" s="22"/>
       <c r="I24" s="22"/>
       <c r="J24" s="23" t="s">
-        <v>380</v>
+        <v>378</v>
       </c>
       <c r="K24" s="22"/>
       <c r="L24" s="22"/>
@@ -15166,7 +15189,7 @@
       <c r="H25" s="22"/>
       <c r="I25" s="22"/>
       <c r="J25" s="23" t="s">
-        <v>381</v>
+        <v>379</v>
       </c>
       <c r="K25" s="22"/>
       <c r="L25" s="22"/>
@@ -15196,7 +15219,7 @@
       <c r="H26" s="22"/>
       <c r="I26" s="22"/>
       <c r="J26" s="23" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
       <c r="K26" s="22"/>
       <c r="L26" s="22"/>
@@ -15226,7 +15249,7 @@
       <c r="H27" s="22"/>
       <c r="I27" s="22"/>
       <c r="J27" s="23" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="K27" s="22"/>
       <c r="L27" s="22"/>
@@ -15256,7 +15279,7 @@
       <c r="H28" s="22"/>
       <c r="I28" s="22"/>
       <c r="J28" s="23" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
       <c r="K28" s="22"/>
       <c r="L28" s="22"/>
@@ -15286,7 +15309,7 @@
       <c r="H29" s="22"/>
       <c r="I29" s="22"/>
       <c r="J29" s="23" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="K29" s="22"/>
       <c r="L29" s="22"/>
@@ -15316,7 +15339,7 @@
       <c r="H30" s="22"/>
       <c r="I30" s="22"/>
       <c r="J30" s="23" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="K30" s="22"/>
       <c r="L30" s="22"/>
@@ -15346,7 +15369,7 @@
       <c r="H31" s="22"/>
       <c r="I31" s="22"/>
       <c r="J31" s="23" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
       <c r="K31" s="22"/>
       <c r="L31" s="22"/>
@@ -15376,7 +15399,7 @@
       <c r="H32" s="22"/>
       <c r="I32" s="22"/>
       <c r="J32" s="23" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
       <c r="K32" s="22"/>
       <c r="L32" s="22"/>
@@ -15406,7 +15429,7 @@
       <c r="H33" s="22"/>
       <c r="I33" s="22"/>
       <c r="J33" s="23" t="s">
-        <v>389</v>
+        <v>387</v>
       </c>
       <c r="K33" s="22"/>
       <c r="L33" s="22"/>
@@ -15436,7 +15459,7 @@
       <c r="H34" s="22"/>
       <c r="I34" s="22"/>
       <c r="J34" s="23" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
       <c r="K34" s="22"/>
       <c r="L34" s="22"/>
@@ -15466,7 +15489,7 @@
       <c r="H35" s="22"/>
       <c r="I35" s="22"/>
       <c r="J35" s="23" t="s">
-        <v>391</v>
+        <v>389</v>
       </c>
       <c r="K35" s="22"/>
       <c r="L35" s="22"/>
@@ -15496,7 +15519,7 @@
       <c r="H36" s="22"/>
       <c r="I36" s="22"/>
       <c r="J36" s="23" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
       <c r="K36" s="22"/>
       <c r="L36" s="22"/>
@@ -15526,7 +15549,7 @@
       <c r="H37" s="22"/>
       <c r="I37" s="22"/>
       <c r="J37" s="23" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="K37" s="22"/>
       <c r="L37" s="22"/>
@@ -15556,7 +15579,7 @@
       <c r="H38" s="22"/>
       <c r="I38" s="22"/>
       <c r="J38" s="23" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
       <c r="K38" s="22"/>
       <c r="L38" s="22"/>
@@ -15586,7 +15609,7 @@
       <c r="H39" s="22"/>
       <c r="I39" s="22"/>
       <c r="J39" s="23" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="K39" s="22"/>
       <c r="L39" s="22"/>
@@ -42484,7 +42507,7 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -42492,10 +42515,10 @@
         <v>196</v>
       </c>
       <c r="B3" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="C3" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="D3" t="s">
         <v>208</v>
@@ -42521,10 +42544,10 @@
         <v>31</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="D4" s="19"/>
       <c r="E4" s="17"/>
@@ -42538,10 +42561,10 @@
         <v>31</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>131</v>
@@ -42567,10 +42590,10 @@
         <v>31</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>131</v>
@@ -42596,10 +42619,10 @@
         <v>31</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="D7" s="15" t="s">
         <v>149</v>
@@ -42625,10 +42648,10 @@
         <v>39</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="D8" s="19"/>
       <c r="E8" s="17"/>
@@ -42642,10 +42665,10 @@
         <v>39</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D9" s="15" t="s">
         <v>154</v>
@@ -42674,7 +42697,7 @@
         <v>247</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="D10" s="19" t="s">
         <v>107</v>
@@ -42700,10 +42723,10 @@
         <v>39</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="D11" s="15" t="s">
         <v>140</v>
@@ -42729,10 +42752,10 @@
         <v>44</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="D12" s="19"/>
       <c r="E12" s="17"/>
@@ -42746,10 +42769,10 @@
         <v>44</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D13" s="15" t="s">
         <v>149</v>
@@ -42775,10 +42798,10 @@
         <v>44</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="D14" s="19" t="s">
         <v>105</v>
@@ -42804,10 +42827,10 @@
         <v>44</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="D15" s="15" t="s">
         <v>154</v>
@@ -42833,10 +42856,10 @@
         <v>50</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="D16" s="19"/>
       <c r="E16" s="17"/>
@@ -42850,10 +42873,10 @@
         <v>50</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="D17" s="15" t="s">
         <v>100</v>
@@ -42879,10 +42902,10 @@
         <v>50</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="D18" s="19" t="s">
         <v>149</v>
@@ -42908,10 +42931,10 @@
         <v>50</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="D19" s="15" t="s">
         <v>104</v>
@@ -42937,10 +42960,10 @@
         <v>57</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C20" s="19" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="D20" s="19"/>
       <c r="E20" s="17"/>
@@ -42954,10 +42977,10 @@
         <v>57</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="D21" s="15" t="s">
         <v>154</v>
@@ -42983,10 +43006,10 @@
         <v>57</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C22" s="19" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="D22" s="19" t="s">
         <v>149</v>
@@ -43012,10 +43035,10 @@
         <v>57</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="D23" s="15" t="s">
         <v>135</v>
@@ -43041,10 +43064,10 @@
         <v>63</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="D24" s="19"/>
       <c r="E24" s="17"/>
@@ -43058,10 +43081,10 @@
         <v>63</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="D25" s="15" t="s">
         <v>100</v>
@@ -43087,10 +43110,10 @@
         <v>63</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C26" s="19" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="D26" s="19" t="s">
         <v>112</v>
@@ -43116,10 +43139,10 @@
         <v>63</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C27" s="15" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="D27" s="15" t="s">
         <v>97</v>
@@ -43145,10 +43168,10 @@
         <v>69</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C28" s="19" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="D28" s="19"/>
       <c r="E28" s="17"/>
@@ -43162,10 +43185,10 @@
         <v>69</v>
       </c>
       <c r="B29" s="15" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D29" s="15" t="s">
         <v>122</v>
@@ -43191,10 +43214,10 @@
         <v>69</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C30" s="19" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="D30" s="19" t="s">
         <v>125</v>
@@ -43220,10 +43243,10 @@
         <v>69</v>
       </c>
       <c r="B31" s="15" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C31" s="15" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="D31" s="15" t="s">
         <v>112</v>
@@ -43249,10 +43272,10 @@
         <v>75</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C32" s="19" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="D32" s="19"/>
       <c r="E32" s="17"/>
@@ -43266,10 +43289,10 @@
         <v>75</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C33" s="15" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="D33" s="15" t="s">
         <v>97</v>
@@ -43295,10 +43318,10 @@
         <v>75</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C34" s="19" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D34" s="19" t="s">
         <v>109</v>
@@ -43324,10 +43347,10 @@
         <v>75</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="D35" s="15" t="s">
         <v>102</v>
@@ -43353,10 +43376,10 @@
         <v>81</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C36" s="19" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="D36" s="19"/>
       <c r="E36" s="17"/>
@@ -43370,10 +43393,10 @@
         <v>81</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="D37" s="15" t="s">
         <v>146</v>
@@ -43399,10 +43422,10 @@
         <v>81</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C38" s="19" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="D38" s="19" t="s">
         <v>112</v>
@@ -43428,10 +43451,10 @@
         <v>81</v>
       </c>
       <c r="B39" s="15" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C39" s="15" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="D39" s="15" t="s">
         <v>109</v>
@@ -43457,10 +43480,10 @@
         <v>86</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C40" s="19" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="D40" s="19"/>
       <c r="E40" s="17"/>
@@ -43474,10 +43497,10 @@
         <v>86</v>
       </c>
       <c r="B41" s="15" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C41" s="15" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="D41" s="15" t="s">
         <v>104</v>
@@ -43503,10 +43526,10 @@
         <v>86</v>
       </c>
       <c r="B42" s="19" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C42" s="19" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="D42" s="19" t="s">
         <v>97</v>
@@ -43532,10 +43555,10 @@
         <v>86</v>
       </c>
       <c r="B43" s="15" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C43" s="15" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="D43" s="15" t="s">
         <v>109</v>
@@ -43558,13 +43581,13 @@
     </row>
     <row r="44" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="19" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="B44" s="19" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C44" s="19" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="D44" s="19"/>
       <c r="E44" s="17"/>
@@ -43575,13 +43598,13 @@
     </row>
     <row r="45" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="15" t="s">
+        <v>302</v>
+      </c>
+      <c r="B45" s="15" t="s">
         <v>304</v>
       </c>
-      <c r="B45" s="15" t="s">
-        <v>306</v>
-      </c>
       <c r="C45" s="15" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="D45" s="15" t="s">
         <v>97</v>
@@ -43604,13 +43627,13 @@
     </row>
     <row r="46" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="19" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="B46" s="19" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C46" s="19" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="D46" s="19" t="s">
         <v>122</v>
@@ -43633,13 +43656,13 @@
     </row>
     <row r="47" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="15" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="B47" s="15" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C47" s="15" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="D47" s="15" t="s">
         <v>149</v>
@@ -43806,7 +43829,7 @@
         <v>45</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>45</v>
@@ -43835,7 +43858,7 @@
         <v>51</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="D9" s="7" t="s">
         <v>51</v>
@@ -43864,7 +43887,7 @@
         <v>58</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="D10" s="7" t="s">
         <v>58</v>
@@ -43922,7 +43945,7 @@
         <v>70</v>
       </c>
       <c r="C12" s="21" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>70</v>
@@ -43951,7 +43974,7 @@
         <v>76</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="D13" s="7" t="s">
         <v>76</v>
@@ -43980,7 +44003,7 @@
         <v>82</v>
       </c>
       <c r="C14" s="21" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="D14" s="7" t="s">
         <v>82</v>
@@ -44009,7 +44032,7 @@
         <v>87</v>
       </c>
       <c r="C15" s="21" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>87</v>
@@ -44038,7 +44061,7 @@
         <v>92</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="D16" s="7" t="s">
         <v>92</v>
@@ -44511,7 +44534,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:Y41"/>
+  <dimension ref="A1:Z41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -44526,12 +44549,12 @@
     <col min="22" max="25" width="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>165</v>
       </c>
@@ -44556,59 +44579,62 @@
       <c r="H3" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="I3" s="5" t="s">
-        <v>249</v>
+      <c r="I3" s="32" t="s">
+        <v>171</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>250</v>
+        <v>172</v>
       </c>
       <c r="K3" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="L3" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="L3" s="5" t="s">
+      <c r="M3" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="M3" s="5" t="s">
+      <c r="N3" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="N3" s="5" t="s">
+      <c r="O3" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="O3" s="5" t="s">
+      <c r="P3" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="P3" s="5" t="s">
+      <c r="Q3" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="Q3" s="5" t="s">
+      <c r="R3" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="R3" s="5" t="s">
+      <c r="S3" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="S3" s="5" t="s">
+      <c r="T3" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="T3" s="5" t="s">
+      <c r="U3" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="U3" s="5" t="s">
+      <c r="V3" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="V3" s="8" t="s">
+      <c r="W3" s="8" t="s">
         <v>185</v>
       </c>
-      <c r="W3" s="5" t="s">
+      <c r="X3" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="X3" s="5" t="s">
+      <c r="Y3" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="Y3" s="5" t="s">
+      <c r="Z3" s="33" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>97</v>
       </c>
@@ -44630,24 +44656,23 @@
       <c r="G4">
         <v>92</v>
       </c>
-      <c r="K4">
+      <c r="L4">
         <v>6</v>
       </c>
-      <c r="L4">
+      <c r="M4">
         <v>8</v>
       </c>
-      <c r="M4">
+      <c r="N4">
         <v>10</v>
       </c>
-      <c r="N4">
+      <c r="O4">
         <v>15</v>
       </c>
-      <c r="O4">
+      <c r="P4">
         <v>20</v>
       </c>
-      <c r="Y4" s="13"/>
-    </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>100</v>
       </c>
@@ -44669,24 +44694,23 @@
       <c r="G5">
         <v>92</v>
       </c>
-      <c r="K5">
+      <c r="L5">
         <v>4</v>
       </c>
-      <c r="L5">
+      <c r="M5">
         <v>6</v>
       </c>
-      <c r="M5">
+      <c r="N5">
         <v>7</v>
       </c>
-      <c r="N5">
+      <c r="O5">
         <v>11</v>
       </c>
-      <c r="O5">
+      <c r="P5">
         <v>15</v>
       </c>
-      <c r="Y5" s="13"/>
-    </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>102</v>
       </c>
@@ -44709,44 +44733,46 @@
         <v>99</v>
       </c>
       <c r="J6">
+        <v>2</v>
+      </c>
+      <c r="K6">
+        <v>2</v>
+      </c>
+      <c r="L6">
         <v>3</v>
       </c>
-      <c r="K6">
-        <v>3</v>
-      </c>
-      <c r="L6">
+      <c r="M6">
         <v>4</v>
       </c>
-      <c r="M6">
+      <c r="N6">
         <v>5</v>
       </c>
-      <c r="N6">
+      <c r="O6">
         <v>8</v>
       </c>
-      <c r="O6">
+      <c r="P6">
         <v>11</v>
       </c>
-      <c r="P6">
+      <c r="Q6">
         <v>15</v>
       </c>
-      <c r="Q6">
+      <c r="R6">
         <v>20</v>
       </c>
-      <c r="R6">
+      <c r="S6">
         <v>25</v>
       </c>
-      <c r="S6">
+      <c r="T6">
         <v>30</v>
       </c>
-      <c r="T6">
+      <c r="U6">
         <v>35</v>
       </c>
-      <c r="U6">
+      <c r="V6">
         <v>40</v>
       </c>
-      <c r="Y6" s="13"/>
-    </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>104</v>
       </c>
@@ -44768,33 +44794,32 @@
       <c r="G7">
         <v>96</v>
       </c>
-      <c r="K7">
+      <c r="L7">
         <v>4</v>
       </c>
-      <c r="L7">
+      <c r="M7">
         <v>6</v>
       </c>
-      <c r="M7">
+      <c r="N7">
         <v>7</v>
       </c>
-      <c r="N7">
+      <c r="O7">
         <v>11</v>
       </c>
-      <c r="O7">
+      <c r="P7">
         <v>15</v>
       </c>
-      <c r="P7">
+      <c r="Q7">
         <v>20</v>
       </c>
-      <c r="Q7">
+      <c r="R7">
         <v>25</v>
       </c>
-      <c r="R7">
+      <c r="S7">
         <v>30</v>
       </c>
-      <c r="Y7" s="13"/>
-    </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>105</v>
       </c>
@@ -44817,26 +44842,28 @@
         <v>92</v>
       </c>
       <c r="J8">
+        <v>4</v>
+      </c>
+      <c r="K8">
         <v>5</v>
       </c>
-      <c r="K8">
+      <c r="L8">
         <v>6</v>
       </c>
-      <c r="L8">
+      <c r="M8">
         <v>8</v>
       </c>
-      <c r="M8">
+      <c r="N8">
         <v>10</v>
       </c>
-      <c r="N8">
+      <c r="O8">
         <v>15</v>
       </c>
-      <c r="O8">
+      <c r="P8">
         <v>20</v>
       </c>
-      <c r="Y8" s="13"/>
-    </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>107</v>
       </c>
@@ -44858,30 +44885,29 @@
       <c r="G9">
         <v>96</v>
       </c>
-      <c r="L9">
-        <v>3</v>
-      </c>
       <c r="M9">
         <v>3</v>
       </c>
       <c r="N9">
+        <v>3</v>
+      </c>
+      <c r="O9">
         <v>6</v>
       </c>
-      <c r="O9">
+      <c r="P9">
         <v>8</v>
       </c>
-      <c r="P9">
+      <c r="Q9">
         <v>10</v>
       </c>
-      <c r="Q9">
+      <c r="R9">
         <v>15</v>
       </c>
-      <c r="R9">
+      <c r="S9">
         <v>20</v>
       </c>
-      <c r="Y9" s="13"/>
-    </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>109</v>
       </c>
@@ -44903,24 +44929,23 @@
       <c r="G10">
         <v>90</v>
       </c>
-      <c r="K10">
+      <c r="L10">
         <v>3</v>
       </c>
-      <c r="L10">
+      <c r="M10">
         <v>4</v>
       </c>
-      <c r="M10">
+      <c r="N10">
         <v>5</v>
       </c>
-      <c r="N10">
+      <c r="O10">
         <v>8</v>
       </c>
-      <c r="O10">
+      <c r="P10">
         <v>11</v>
       </c>
-      <c r="Y10" s="13"/>
-    </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>112</v>
       </c>
@@ -44949,23 +44974,25 @@
         <v>3</v>
       </c>
       <c r="J11">
+        <v>4</v>
+      </c>
+      <c r="K11">
         <v>5</v>
       </c>
-      <c r="K11">
+      <c r="L11">
         <v>6</v>
       </c>
-      <c r="L11">
+      <c r="M11">
         <v>8</v>
       </c>
-      <c r="M11">
+      <c r="N11">
         <v>10</v>
       </c>
-      <c r="N11">
+      <c r="O11">
         <v>15</v>
       </c>
-      <c r="Y11" s="13"/>
-    </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>114</v>
       </c>
@@ -44991,23 +45018,25 @@
         <v>3</v>
       </c>
       <c r="K12">
+        <v>3</v>
+      </c>
+      <c r="L12">
         <v>4</v>
       </c>
-      <c r="L12">
+      <c r="M12">
         <v>6</v>
       </c>
-      <c r="M12">
+      <c r="N12">
         <v>7</v>
       </c>
-      <c r="N12">
+      <c r="O12">
         <v>11</v>
       </c>
-      <c r="O12">
+      <c r="P12">
         <v>15</v>
       </c>
-      <c r="Y12" s="13"/>
-    </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>116</v>
       </c>
@@ -45039,20 +45068,22 @@
         <v>3</v>
       </c>
       <c r="K13">
+        <v>3</v>
+      </c>
+      <c r="L13">
         <v>4</v>
       </c>
-      <c r="L13">
+      <c r="M13">
         <v>6</v>
       </c>
-      <c r="M13">
+      <c r="N13">
         <v>7</v>
       </c>
-      <c r="N13">
+      <c r="O13">
         <v>11</v>
       </c>
-      <c r="Y13" s="13"/>
-    </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>118</v>
       </c>
@@ -45084,14 +45115,16 @@
         <v>2</v>
       </c>
       <c r="K14">
+        <v>2</v>
+      </c>
+      <c r="L14">
         <v>3</v>
       </c>
-      <c r="L14">
+      <c r="M14">
         <v>4</v>
       </c>
-      <c r="Y14" s="13"/>
-    </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>120</v>
       </c>
@@ -45117,23 +45150,25 @@
         <v>2</v>
       </c>
       <c r="K15">
+        <v>2</v>
+      </c>
+      <c r="L15">
         <v>3</v>
       </c>
-      <c r="L15">
+      <c r="M15">
         <v>4</v>
       </c>
-      <c r="M15">
+      <c r="N15">
         <v>5</v>
       </c>
-      <c r="N15">
+      <c r="O15">
         <v>8</v>
       </c>
-      <c r="O15">
+      <c r="P15">
         <v>11</v>
       </c>
-      <c r="Y15" s="13"/>
-    </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>122</v>
       </c>
@@ -45155,21 +45190,20 @@
       <c r="G16">
         <v>92</v>
       </c>
-      <c r="L16">
+      <c r="M16">
         <v>6</v>
       </c>
-      <c r="M16">
+      <c r="N16">
         <v>7</v>
       </c>
-      <c r="N16">
+      <c r="O16">
         <v>11</v>
       </c>
-      <c r="O16">
+      <c r="P16">
         <v>15</v>
       </c>
-      <c r="Y16" s="13"/>
-    </row>
-    <row r="17" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>125</v>
       </c>
@@ -45201,23 +45235,25 @@
         <v>3</v>
       </c>
       <c r="K17">
+        <v>3</v>
+      </c>
+      <c r="L17">
         <v>4</v>
       </c>
-      <c r="L17">
+      <c r="M17">
         <v>6</v>
       </c>
-      <c r="M17">
+      <c r="N17">
         <v>7</v>
       </c>
-      <c r="N17">
+      <c r="O17">
         <v>11</v>
       </c>
-      <c r="O17">
+      <c r="P17">
         <v>15</v>
       </c>
-      <c r="Y17" s="13"/>
-    </row>
-    <row r="18" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>127</v>
       </c>
@@ -45246,26 +45282,28 @@
         <v>1</v>
       </c>
       <c r="J18">
+        <v>2</v>
+      </c>
+      <c r="K18">
+        <v>2</v>
+      </c>
+      <c r="L18">
         <v>3</v>
       </c>
-      <c r="K18">
-        <v>3</v>
-      </c>
-      <c r="L18">
+      <c r="M18">
         <v>4</v>
       </c>
-      <c r="M18">
+      <c r="N18">
         <v>5</v>
       </c>
-      <c r="N18">
+      <c r="O18">
         <v>8</v>
       </c>
-      <c r="O18">
+      <c r="P18">
         <v>11</v>
       </c>
-      <c r="Y18" s="13"/>
-    </row>
-    <row r="19" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>129</v>
       </c>
@@ -45287,30 +45325,29 @@
       <c r="G19">
         <v>96</v>
       </c>
-      <c r="L19">
+      <c r="M19">
         <v>8</v>
       </c>
-      <c r="M19">
+      <c r="N19">
         <v>10</v>
       </c>
-      <c r="N19">
+      <c r="O19">
         <v>15</v>
       </c>
-      <c r="O19">
+      <c r="P19">
         <v>20</v>
       </c>
-      <c r="P19">
+      <c r="Q19">
         <v>25</v>
       </c>
-      <c r="Q19">
+      <c r="R19">
         <v>30</v>
       </c>
-      <c r="R19">
+      <c r="S19">
         <v>35</v>
       </c>
-      <c r="Y19" s="13"/>
-    </row>
-    <row r="20" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>131</v>
       </c>
@@ -45332,30 +45369,29 @@
       <c r="G20">
         <v>96</v>
       </c>
-      <c r="L20">
-        <v>3</v>
-      </c>
       <c r="M20">
         <v>3</v>
       </c>
       <c r="N20">
+        <v>3</v>
+      </c>
+      <c r="O20">
         <v>6</v>
       </c>
-      <c r="O20">
+      <c r="P20">
         <v>8</v>
       </c>
-      <c r="P20">
+      <c r="Q20">
         <v>10</v>
       </c>
-      <c r="Q20">
+      <c r="R20">
         <v>15</v>
       </c>
-      <c r="R20">
+      <c r="S20">
         <v>20</v>
       </c>
-      <c r="Y20" s="13"/>
-    </row>
-    <row r="21" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>133</v>
       </c>
@@ -45384,23 +45420,25 @@
         <v>1</v>
       </c>
       <c r="J21">
+        <v>2</v>
+      </c>
+      <c r="K21">
+        <v>2</v>
+      </c>
+      <c r="L21">
         <v>3</v>
       </c>
-      <c r="K21">
-        <v>3</v>
-      </c>
-      <c r="L21">
+      <c r="M21">
         <v>4</v>
       </c>
-      <c r="M21">
+      <c r="N21">
         <v>5</v>
       </c>
-      <c r="N21">
+      <c r="O21">
         <v>8</v>
       </c>
-      <c r="Y21" s="13"/>
-    </row>
-    <row r="22" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>135</v>
       </c>
@@ -45422,30 +45460,29 @@
       <c r="G22">
         <v>96</v>
       </c>
-      <c r="L22">
+      <c r="M22">
         <v>8</v>
       </c>
-      <c r="M22">
+      <c r="N22">
         <v>10</v>
       </c>
-      <c r="N22">
+      <c r="O22">
         <v>15</v>
       </c>
-      <c r="O22">
+      <c r="P22">
         <v>20</v>
       </c>
-      <c r="P22">
+      <c r="Q22">
         <v>25</v>
       </c>
-      <c r="Q22">
+      <c r="R22">
         <v>30</v>
       </c>
-      <c r="R22">
+      <c r="S22">
         <v>35</v>
       </c>
-      <c r="Y22" s="13"/>
-    </row>
-    <row r="23" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>138</v>
       </c>
@@ -45467,30 +45504,29 @@
       <c r="G23">
         <v>96</v>
       </c>
-      <c r="L23">
+      <c r="M23">
         <v>6</v>
       </c>
-      <c r="M23">
+      <c r="N23">
         <v>7</v>
       </c>
-      <c r="N23">
+      <c r="O23">
         <v>11</v>
       </c>
-      <c r="O23">
+      <c r="P23">
         <v>15</v>
       </c>
-      <c r="P23">
+      <c r="Q23">
         <v>20</v>
       </c>
-      <c r="Q23">
+      <c r="R23">
         <v>25</v>
       </c>
-      <c r="R23">
+      <c r="S23">
         <v>30</v>
       </c>
-      <c r="Y23" s="13"/>
-    </row>
-    <row r="24" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>140</v>
       </c>
@@ -45512,39 +45548,38 @@
       <c r="G24">
         <v>99</v>
       </c>
-      <c r="L24">
-        <v>3</v>
-      </c>
       <c r="M24">
         <v>3</v>
       </c>
       <c r="N24">
+        <v>3</v>
+      </c>
+      <c r="O24">
         <v>6</v>
       </c>
-      <c r="O24">
+      <c r="P24">
         <v>8</v>
       </c>
-      <c r="P24">
+      <c r="Q24">
         <v>10</v>
       </c>
-      <c r="Q24">
+      <c r="R24">
         <v>15</v>
       </c>
-      <c r="R24">
+      <c r="S24">
         <v>20</v>
       </c>
-      <c r="S24">
+      <c r="T24">
         <v>25</v>
       </c>
-      <c r="T24">
+      <c r="U24">
         <v>30</v>
       </c>
-      <c r="U24">
+      <c r="V24">
         <v>35</v>
       </c>
-      <c r="Y24" s="13"/>
-    </row>
-    <row r="25" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>142</v>
       </c>
@@ -45566,36 +45601,38 @@
       <c r="G25">
         <v>99</v>
       </c>
-      <c r="L25">
+      <c r="M25">
         <v>3</v>
       </c>
-      <c r="M25">
+      <c r="N25">
+        <v>3</v>
+      </c>
+      <c r="O25">
         <v>6</v>
       </c>
-      <c r="N25">
+      <c r="P25">
         <v>8</v>
       </c>
-      <c r="O25">
+      <c r="Q25">
         <v>10</v>
       </c>
-      <c r="P25">
+      <c r="R25">
         <v>15</v>
       </c>
-      <c r="Q25">
+      <c r="S25">
         <v>20</v>
       </c>
-      <c r="R25">
+      <c r="T25">
         <v>25</v>
       </c>
-      <c r="S25">
+      <c r="U25">
         <v>30</v>
       </c>
-      <c r="T25">
+      <c r="V25">
         <v>35</v>
       </c>
-      <c r="Y25" s="13"/>
-    </row>
-    <row r="26" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>144</v>
       </c>
@@ -45617,30 +45654,29 @@
       <c r="G26">
         <v>96</v>
       </c>
-      <c r="L26">
+      <c r="M26">
         <v>6</v>
       </c>
-      <c r="M26">
+      <c r="N26">
         <v>7</v>
       </c>
-      <c r="N26">
+      <c r="O26">
         <v>11</v>
       </c>
-      <c r="O26">
+      <c r="P26">
         <v>15</v>
       </c>
-      <c r="P26">
+      <c r="Q26">
         <v>20</v>
       </c>
-      <c r="Q26">
+      <c r="R26">
         <v>25</v>
       </c>
-      <c r="R26">
+      <c r="S26">
         <v>30</v>
       </c>
-      <c r="Y26" s="13"/>
-    </row>
-    <row r="27" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>146</v>
       </c>
@@ -45662,24 +45698,23 @@
       <c r="G27">
         <v>92</v>
       </c>
-      <c r="K27">
+      <c r="L27">
         <v>6</v>
       </c>
-      <c r="L27">
+      <c r="M27">
         <v>8</v>
       </c>
-      <c r="M27">
+      <c r="N27">
         <v>10</v>
       </c>
-      <c r="N27">
+      <c r="O27">
         <v>15</v>
       </c>
-      <c r="O27">
+      <c r="P27">
         <v>20</v>
       </c>
-      <c r="Y27" s="13"/>
-    </row>
-    <row r="28" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>149</v>
       </c>
@@ -45701,24 +45736,23 @@
       <c r="G28">
         <v>92</v>
       </c>
-      <c r="K28">
+      <c r="L28">
         <v>6</v>
       </c>
-      <c r="L28">
+      <c r="M28">
         <v>8</v>
       </c>
-      <c r="M28">
+      <c r="N28">
         <v>10</v>
       </c>
-      <c r="N28">
+      <c r="O28">
         <v>15</v>
       </c>
-      <c r="O28">
+      <c r="P28">
         <v>20</v>
       </c>
-      <c r="Y28" s="13"/>
-    </row>
-    <row r="29" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>151</v>
       </c>
@@ -45740,39 +45774,38 @@
       <c r="G29">
         <v>99</v>
       </c>
-      <c r="L29">
+      <c r="M29">
         <v>4</v>
       </c>
-      <c r="M29">
+      <c r="N29">
         <v>5</v>
       </c>
-      <c r="N29">
+      <c r="O29">
         <v>8</v>
       </c>
-      <c r="O29">
+      <c r="P29">
         <v>11</v>
       </c>
-      <c r="P29">
+      <c r="Q29">
         <v>15</v>
       </c>
-      <c r="Q29">
+      <c r="R29">
         <v>20</v>
       </c>
-      <c r="R29">
+      <c r="S29">
         <v>25</v>
       </c>
-      <c r="S29">
+      <c r="T29">
         <v>30</v>
       </c>
-      <c r="T29">
+      <c r="U29">
         <v>35</v>
       </c>
-      <c r="U29">
+      <c r="V29">
         <v>40</v>
       </c>
-      <c r="Y29" s="13"/>
-    </row>
-    <row r="30" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>156</v>
       </c>
@@ -45795,23 +45828,28 @@
         <v>92</v>
       </c>
       <c r="J30">
+        <v>2</v>
+      </c>
+      <c r="K30">
+        <v>2</v>
+      </c>
+      <c r="L30">
         <v>3</v>
       </c>
-      <c r="K30">
+      <c r="M30">
         <v>4</v>
       </c>
-      <c r="L30">
+      <c r="N30">
         <v>5</v>
       </c>
-      <c r="M30">
+      <c r="O30">
         <v>8</v>
       </c>
-      <c r="N30">
+      <c r="P30">
         <v>11</v>
       </c>
-      <c r="Y30" s="13"/>
-    </row>
-    <row r="31" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>154</v>
       </c>
@@ -45833,33 +45871,32 @@
       <c r="G31">
         <v>96</v>
       </c>
-      <c r="K31">
+      <c r="L31">
         <v>4</v>
       </c>
-      <c r="L31">
+      <c r="M31">
         <v>6</v>
       </c>
-      <c r="M31">
+      <c r="N31">
         <v>7</v>
       </c>
-      <c r="N31">
+      <c r="O31">
         <v>11</v>
       </c>
-      <c r="O31">
+      <c r="P31">
         <v>15</v>
       </c>
-      <c r="P31">
+      <c r="Q31">
         <v>20</v>
       </c>
-      <c r="Q31">
+      <c r="R31">
         <v>25</v>
       </c>
-      <c r="R31">
+      <c r="S31">
         <v>30</v>
       </c>
-      <c r="Y31" s="13"/>
-    </row>
-    <row r="32" spans="1:25" x14ac:dyDescent="0.25">
+    </row>
+    <row r="32" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>158</v>
       </c>
@@ -45885,42 +45922,29 @@
         <v>2</v>
       </c>
       <c r="K32">
+        <v>2</v>
+      </c>
+      <c r="L32">
         <v>3</v>
       </c>
-      <c r="L32">
+      <c r="M32">
         <v>4</v>
       </c>
-      <c r="M32">
+      <c r="N32">
         <v>5</v>
       </c>
-      <c r="N32">
+      <c r="O32">
         <v>8</v>
       </c>
-      <c r="O32">
+      <c r="P32">
         <v>11</v>
       </c>
-      <c r="P32">
+      <c r="Q32">
         <v>15</v>
       </c>
-      <c r="Q32">
+      <c r="R32">
         <v>20</v>
       </c>
-      <c r="Y32" s="13"/>
-    </row>
-    <row r="33" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="Y33" s="13"/>
-    </row>
-    <row r="34" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="Y34" s="13"/>
-    </row>
-    <row r="35" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="Y35" s="13"/>
-    </row>
-    <row r="36" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="Y36" s="13"/>
-    </row>
-    <row r="37" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="Y37" s="13"/>
     </row>
     <row r="38" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
@@ -45944,13 +45968,12 @@
       <c r="G38">
         <v>4</v>
       </c>
-      <c r="W38">
+      <c r="X38">
         <v>10</v>
       </c>
-      <c r="X38">
+      <c r="Y38">
         <v>20</v>
       </c>
-      <c r="Y38" s="13"/>
     </row>
     <row r="39" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
@@ -45974,10 +45997,9 @@
       <c r="G39">
         <v>4</v>
       </c>
-      <c r="X39">
+      <c r="Y39">
         <v>25</v>
       </c>
-      <c r="Y39" s="13"/>
     </row>
     <row r="41" spans="1:25" x14ac:dyDescent="0.25">
       <c r="Y41" s="13"/>
@@ -47584,10 +47606,10 @@
         <v>190</v>
       </c>
       <c r="E30" s="15">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F30" s="15">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="G30" s="15">
         <v>99</v>
@@ -47646,13 +47668,13 @@
         <v>189</v>
       </c>
       <c r="E31" s="15">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="F31" s="15">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="G31" s="15">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="H31" s="15"/>
       <c r="I31" s="15"/>
@@ -47662,23 +47684,35 @@
         <v>3</v>
       </c>
       <c r="M31" s="15">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N31" s="15">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="O31" s="15">
+        <v>6</v>
+      </c>
+      <c r="P31" s="15">
         <v>8</v>
       </c>
-      <c r="P31" s="15">
-        <v>11</v>
-      </c>
-      <c r="Q31" s="15"/>
-      <c r="R31" s="15"/>
-      <c r="S31" s="15"/>
-      <c r="T31" s="15"/>
-      <c r="U31" s="15"/>
-      <c r="V31" s="15"/>
+      <c r="Q31" s="15">
+        <v>10</v>
+      </c>
+      <c r="R31" s="15">
+        <v>15</v>
+      </c>
+      <c r="S31" s="15">
+        <v>20</v>
+      </c>
+      <c r="T31" s="15">
+        <v>25</v>
+      </c>
+      <c r="U31" s="15">
+        <v>30</v>
+      </c>
+      <c r="V31" s="15">
+        <v>35</v>
+      </c>
       <c r="X31" s="15"/>
       <c r="Y31" s="15"/>
       <c r="Z31" s="15"/>
@@ -48340,7 +48374,7 @@
         <v>109</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="C10" s="15" t="s">
         <v>220</v>
@@ -48512,7 +48546,7 @@
         <v>116</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="C13" s="15" t="s">
         <v>220</v>
@@ -48697,7 +48731,7 @@
         <v>123</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>189</v>
@@ -48755,7 +48789,7 @@
         <v>126</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D17" s="15" t="s">
         <v>190</v>
@@ -48814,10 +48848,10 @@
         <v>127</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D18" s="15" t="s">
         <v>189</v>
@@ -48878,10 +48912,10 @@
         <v>129</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D19" s="15" t="s">
         <v>189</v>
@@ -48934,10 +48968,10 @@
         <v>131</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D20" s="15" t="s">
         <v>189</v>
@@ -48993,7 +49027,7 @@
         <v>134</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D21" s="15" t="s">
         <v>189</v>
@@ -49046,7 +49080,7 @@
         <v>135</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="C22" s="15" t="s">
         <v>137</v>
@@ -49104,7 +49138,7 @@
         <v>138</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="C23" s="15" t="s">
         <v>137</v>
@@ -49160,7 +49194,7 @@
         <v>140</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="C24" s="15" t="s">
         <v>137</v>
@@ -49218,7 +49252,7 @@
         <v>142</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="C25" s="15" t="s">
         <v>137</v>
@@ -49276,7 +49310,7 @@
         <v>144</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="C26" s="15" t="s">
         <v>137</v>
@@ -49332,7 +49366,7 @@
         <v>146</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="C27" s="15" t="s">
         <v>148</v>
@@ -49386,7 +49420,7 @@
         <v>149</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="C28" s="15" t="s">
         <v>148</v>
@@ -50184,7 +50218,7 @@
         <v>104</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="C7" s="15" t="s">
         <v>99</v>
@@ -50348,7 +50382,7 @@
         <v>109</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="C10" s="15" t="s">
         <v>220</v>
@@ -50512,7 +50546,7 @@
         <v>116</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="C13" s="15" t="s">
         <v>220</v>
@@ -50531,7 +50565,9 @@
       </c>
       <c r="H13" s="15"/>
       <c r="I13" s="15"/>
-      <c r="J13" s="15"/>
+      <c r="J13" s="15">
+        <v>3</v>
+      </c>
       <c r="K13" s="15">
         <v>3</v>
       </c>
@@ -50583,7 +50619,9 @@
       </c>
       <c r="H14" s="15"/>
       <c r="I14" s="15"/>
-      <c r="J14" s="15"/>
+      <c r="J14" s="15">
+        <v>2</v>
+      </c>
       <c r="K14" s="15">
         <v>2</v>
       </c>
@@ -50637,7 +50675,9 @@
       </c>
       <c r="H15" s="15"/>
       <c r="I15" s="15"/>
-      <c r="J15" s="15"/>
+      <c r="J15" s="15">
+        <v>2</v>
+      </c>
       <c r="K15" s="15">
         <v>2</v>
       </c>
@@ -50675,7 +50715,7 @@
         <v>123</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>189</v>
@@ -50691,7 +50731,9 @@
       </c>
       <c r="H16" s="15"/>
       <c r="I16" s="15"/>
-      <c r="J16" s="15"/>
+      <c r="J16" s="15">
+        <v>3</v>
+      </c>
       <c r="K16" s="15">
         <v>3</v>
       </c>
@@ -50729,7 +50771,7 @@
         <v>126</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D17" s="15" t="s">
         <v>189</v>
@@ -50788,10 +50830,10 @@
         <v>127</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D18" s="15" t="s">
         <v>189</v>
@@ -50852,10 +50894,10 @@
         <v>129</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D19" s="15" t="s">
         <v>189</v>
@@ -50908,10 +50950,10 @@
         <v>131</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D20" s="15" t="s">
         <v>189</v>
@@ -50963,7 +51005,7 @@
         <v>134</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D21" s="15" t="s">
         <v>189</v>
@@ -50979,7 +51021,9 @@
       </c>
       <c r="H21" s="15"/>
       <c r="I21" s="15"/>
-      <c r="J21" s="15"/>
+      <c r="J21" s="15">
+        <v>2</v>
+      </c>
       <c r="K21" s="15">
         <v>2</v>
       </c>
@@ -51014,7 +51058,7 @@
         <v>135</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="C22" s="15" t="s">
         <v>137</v>
@@ -51064,7 +51108,7 @@
         <v>138</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="C23" s="15" t="s">
         <v>137</v>
@@ -51083,7 +51127,9 @@
       </c>
       <c r="H23" s="15"/>
       <c r="I23" s="15"/>
-      <c r="J23" s="15"/>
+      <c r="J23" s="15">
+        <v>3</v>
+      </c>
       <c r="K23" s="15">
         <v>3</v>
       </c>
@@ -51118,7 +51164,7 @@
         <v>140</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="C24" s="15" t="s">
         <v>137</v>
@@ -51170,7 +51216,7 @@
         <v>142</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="C25" s="15" t="s">
         <v>137</v>
@@ -51222,7 +51268,7 @@
         <v>144</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="C26" s="15" t="s">
         <v>137</v>
@@ -51272,7 +51318,7 @@
         <v>146</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="C27" s="15" t="s">
         <v>148</v>
@@ -51322,7 +51368,7 @@
         <v>149</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="C28" s="15" t="s">
         <v>148</v>
@@ -51393,7 +51439,9 @@
       </c>
       <c r="H29" s="15"/>
       <c r="I29" s="15"/>
-      <c r="J29" s="15"/>
+      <c r="J29" s="15">
+        <v>2</v>
+      </c>
       <c r="K29" s="15">
         <v>2</v>
       </c>
@@ -52028,7 +52076,7 @@
         <v>104</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="C7" s="15" t="s">
         <v>99</v>
@@ -52210,7 +52258,7 @@
         <v>109</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="C10" s="15" t="s">
         <v>220</v>
@@ -52380,7 +52428,7 @@
         <v>116</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="C13" s="15" t="s">
         <v>220</v>
@@ -52555,7 +52603,7 @@
         <v>123</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>189</v>
@@ -52611,7 +52659,7 @@
         <v>126</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D17" s="15" t="s">
         <v>189</v>
@@ -52664,10 +52712,10 @@
         <v>127</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D18" s="15" t="s">
         <v>189</v>
@@ -52736,10 +52784,10 @@
         <v>129</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D19" s="15" t="s">
         <v>190</v>
@@ -52794,10 +52842,10 @@
         <v>131</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D20" s="15" t="s">
         <v>189</v>
@@ -52853,7 +52901,7 @@
         <v>134</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D21" s="15" t="s">
         <v>189</v>
@@ -52906,7 +52954,7 @@
         <v>135</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="C22" s="15" t="s">
         <v>137</v>
@@ -52968,7 +53016,7 @@
         <v>138</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="C23" s="15" t="s">
         <v>137</v>
@@ -53026,7 +53074,7 @@
         <v>140</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="C24" s="15" t="s">
         <v>137</v>
@@ -53088,7 +53136,7 @@
         <v>142</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="C25" s="15" t="s">
         <v>137</v>
@@ -53144,7 +53192,7 @@
         <v>144</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="C26" s="15" t="s">
         <v>137</v>
@@ -53194,7 +53242,7 @@
         <v>146</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="C27" s="15" t="s">
         <v>148</v>
@@ -53246,7 +53294,7 @@
         <v>149</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="C28" s="15" t="s">
         <v>148</v>
@@ -53972,7 +54020,7 @@
         <v>104</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="C7" s="15" t="s">
         <v>99</v>
@@ -54158,7 +54206,7 @@
         <v>109</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="C10" s="15" t="s">
         <v>220</v>
@@ -54328,7 +54376,7 @@
         <v>116</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="C13" s="15" t="s">
         <v>220</v>
@@ -54515,7 +54563,7 @@
         <v>123</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>189</v>
@@ -54577,7 +54625,7 @@
         <v>126</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D17" s="15" t="s">
         <v>189</v>
@@ -54624,10 +54672,10 @@
         <v>127</v>
       </c>
       <c r="B18" s="15" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D18" s="15" t="s">
         <v>189</v>
@@ -54686,10 +54734,10 @@
         <v>129</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D19" s="15" t="s">
         <v>189</v>
@@ -54742,10 +54790,10 @@
         <v>131</v>
       </c>
       <c r="B20" s="15" t="s">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D20" s="15" t="s">
         <v>190</v>
@@ -54807,7 +54855,7 @@
         <v>134</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D21" s="15" t="s">
         <v>189</v>
@@ -54862,7 +54910,7 @@
         <v>135</v>
       </c>
       <c r="B22" s="15" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="C22" s="15" t="s">
         <v>137</v>
@@ -54912,7 +54960,7 @@
         <v>138</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>402</v>
+        <v>400</v>
       </c>
       <c r="C23" s="15" t="s">
         <v>137</v>
@@ -54970,7 +55018,7 @@
         <v>140</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>403</v>
+        <v>401</v>
       </c>
       <c r="C24" s="15" t="s">
         <v>137</v>
@@ -55026,7 +55074,7 @@
         <v>142</v>
       </c>
       <c r="B25" s="15" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="C25" s="15" t="s">
         <v>137</v>
@@ -55078,7 +55126,7 @@
         <v>144</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="C26" s="15" t="s">
         <v>137</v>
@@ -55138,7 +55186,7 @@
         <v>146</v>
       </c>
       <c r="B27" s="15" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="C27" s="15" t="s">
         <v>148</v>
@@ -55190,7 +55238,7 @@
         <v>149</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="C28" s="15" t="s">
         <v>148</v>

</xml_diff>

<commit_message>
Ajout installations club et mise à jour composants
</commit_message>
<xml_diff>
--- a/data/fc27-data.xlsx
+++ b/data/fc27-data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexi\Desktop\Projets\builderproclubs\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\builderproclubs\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B13C90BD-E185-4075-B3FC-0136A503E02E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9C127F4-44B5-413F-BB07-5551298E2247}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="692" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="692" firstSheet="7" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lisez-moi" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,8 @@
     <sheet name="ddd" sheetId="21" r:id="rId18"/>
     <sheet name="TaillePoids" sheetId="23" r:id="rId19"/>
     <sheet name="Specialisations" sheetId="22" r:id="rId20"/>
-    <sheet name="Reglages" sheetId="20" r:id="rId21"/>
+    <sheet name="InstallationsClub" sheetId="24" r:id="rId21"/>
+    <sheet name="Reglages" sheetId="20" r:id="rId22"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Boss!$A$3:$Z$39</definedName>
@@ -53,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2626" uniqueCount="423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3039" uniqueCount="548">
   <si>
     <t>Base de données — FC 27 Constructeur de build</t>
   </si>
@@ -1548,12 +1549,460 @@
   <si>
     <t>190 cm,90 kg,-6,-6,-2,+6,+2,+6</t>
   </si>
+  <si>
+    <t>Installation</t>
+  </si>
+  <si>
+    <t>Niveau</t>
+  </si>
+  <si>
+    <t>Cout (€)</t>
+  </si>
+  <si>
+    <t>Bonus d'attributs</t>
+  </si>
+  <si>
+    <t>Style de jeu</t>
+  </si>
+  <si>
+    <t>Responsable du matériel</t>
+  </si>
+  <si>
+    <t>Niveau 1</t>
+  </si>
+  <si>
+    <t>Détente +2
+Endurance +2</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Niveau 2</t>
+  </si>
+  <si>
+    <t>Détente +3
+Endurance +3</t>
+  </si>
+  <si>
+    <t>Niveau 3</t>
+  </si>
+  <si>
+    <t>Détente +4
+Endurance +4</t>
+  </si>
+  <si>
+    <t>Entretien des terrains</t>
+  </si>
+  <si>
+    <t>Équilibre +2
+Conduite bal. +2</t>
+  </si>
+  <si>
+    <t>Équilibre +5
+Conduite bal. +5</t>
+  </si>
+  <si>
+    <t>Analyste des perf.</t>
+  </si>
+  <si>
+    <t>Vista +2
+Passes court. +2</t>
+  </si>
+  <si>
+    <t>Vista +3
+Passes court. +5</t>
+  </si>
+  <si>
+    <t>Vista +5
+Passes court. +5</t>
+  </si>
+  <si>
+    <t>Recruteur</t>
+  </si>
+  <si>
+    <t>Pos. off. +2
+Lucidité déf. +2</t>
+  </si>
+  <si>
+    <t>Pos. off. +5
+Lucidité déf. +5</t>
+  </si>
+  <si>
+    <t>Pos. off. +7
+Lucidité déf. +7</t>
+  </si>
+  <si>
+    <t>Psychologue du sport</t>
+  </si>
+  <si>
+    <t>Agressivité +2
+Calme +2</t>
+  </si>
+  <si>
+    <t>Agressivité +5
+Calme +5</t>
+  </si>
+  <si>
+    <t>Scientifique du sport</t>
+  </si>
+  <si>
+    <t>Accélération +2
+Réactivité +2</t>
+  </si>
+  <si>
+    <t>Accélération +5 
+Réactivité +5</t>
+  </si>
+  <si>
+    <t>Longue touche+</t>
+  </si>
+  <si>
+    <t>Coach tactique attaque</t>
+  </si>
+  <si>
+    <t>Pos. off. +2
+Vista +2</t>
+  </si>
+  <si>
+    <t>Pos. off. +5
+Vista +5</t>
+  </si>
+  <si>
+    <t>Attaque rapide</t>
+  </si>
+  <si>
+    <t>Coach tactique défense</t>
+  </si>
+  <si>
+    <t>Interceptions +2
+Lucidité déf. +2</t>
+  </si>
+  <si>
+    <t>Interceptions +5
+Lucidité déf. +5</t>
+  </si>
+  <si>
+    <t>Équipe de prép. physique</t>
+  </si>
+  <si>
+    <t>Détente +5
+Endurance +5</t>
+  </si>
+  <si>
+    <t>Coach G</t>
+  </si>
+  <si>
+    <t>Plongeons +2
+Pos. G +2</t>
+  </si>
+  <si>
+    <t>Plongeons +5
+Pos. G +5</t>
+  </si>
+  <si>
+    <t>Réflexes G</t>
+  </si>
+  <si>
+    <t>Coach passes</t>
+  </si>
+  <si>
+    <t>Passes long. +2
+Passes court. +2</t>
+  </si>
+  <si>
+    <t>Passes long. +5
+Passes court. +5</t>
+  </si>
+  <si>
+    <t>Coach tirs</t>
+  </si>
+  <si>
+    <t>Finition +2
+Tirs de loin +2</t>
+  </si>
+  <si>
+    <t>Finition +5
+Tirs de loin +5</t>
+  </si>
+  <si>
+    <t>Coach tacles</t>
+  </si>
+  <si>
+    <t>Tacles deb. +2
+Tacles gliss. +2</t>
+  </si>
+  <si>
+    <t>Tacles deb. +5
+Tacles gliss. +5</t>
+  </si>
+  <si>
+    <t>Coach technique</t>
+  </si>
+  <si>
+    <t>Conduite bal. +2
+Dribbles +2</t>
+  </si>
+  <si>
+    <t>Conduite bal. +5
+Dribbles +5</t>
+  </si>
+  <si>
+    <t>Piquets de slalom</t>
+  </si>
+  <si>
+    <t>Agilité +2
+Dribbles +2</t>
+  </si>
+  <si>
+    <t>Agilité +5
+Dribbles +5</t>
+  </si>
+  <si>
+    <t>Dribbleur classe</t>
+  </si>
+  <si>
+    <t>Canons à ballons</t>
+  </si>
+  <si>
+    <t>Jeu à la main +2
+Réflexes G +2</t>
+  </si>
+  <si>
+    <t>Jeu à la main +5
+Réflexes G +5</t>
+  </si>
+  <si>
+    <t>Longue relance</t>
+  </si>
+  <si>
+    <t>Filet de finition</t>
+  </si>
+  <si>
+    <t>Finition +2
+Effet +2</t>
+  </si>
+  <si>
+    <t>Finition +5
+Effet +5</t>
+  </si>
+  <si>
+    <t>Filet de futnet</t>
+  </si>
+  <si>
+    <t>Précis. tête +2
+Volées +2</t>
+  </si>
+  <si>
+    <t>Précis. tête +5
+Volées +5</t>
+  </si>
+  <si>
+    <t>Gilets GPS</t>
+  </si>
+  <si>
+    <t>Endurance +2
+Pos. off. +2</t>
+  </si>
+  <si>
+    <t>Endurance +5
+Pos. off. +5</t>
+  </si>
+  <si>
+    <t>Endurance +7
+Pos. off. +7</t>
+  </si>
+  <si>
+    <t>Mini-cages</t>
+  </si>
+  <si>
+    <t>Finition +2
+Passes court. +2</t>
+  </si>
+  <si>
+    <t>Finition +5
+Passes court. +5</t>
+  </si>
+  <si>
+    <t>Rebondisseurs</t>
+  </si>
+  <si>
+    <t>Réactivité +2
+Volées +2</t>
+  </si>
+  <si>
+    <t>Réactivité +5
+Volées +5</t>
+  </si>
+  <si>
+    <t>Mannequins coup de pied arrêté</t>
+  </si>
+  <si>
+    <t>Précision CF +2
+Pénaltys +2</t>
+  </si>
+  <si>
+    <t>Précision CF +5
+Pénaltys +5</t>
+  </si>
+  <si>
+    <t>Parachute de vitesse</t>
+  </si>
+  <si>
+    <t>Accélération +1
+Vit. sprint +1</t>
+  </si>
+  <si>
+    <t>Accélération +2
+Vit. sprint +2</t>
+  </si>
+  <si>
+    <t>Accélération +3
+Vit. sprint +3</t>
+  </si>
+  <si>
+    <t>Bottes de compression</t>
+  </si>
+  <si>
+    <t>Force +2
+P. de tir +2</t>
+  </si>
+  <si>
+    <t>Force +5
+P. de tir +5</t>
+  </si>
+  <si>
+    <t>Frappe lourde</t>
+  </si>
+  <si>
+    <t>Piste d'athlétisme</t>
+  </si>
+  <si>
+    <t>Vit. sprint +1
+Endurance +1</t>
+  </si>
+  <si>
+    <t>Vit. sprint +2
+Endurance +3</t>
+  </si>
+  <si>
+    <t>Vit. sprint +1
+Endurance +5</t>
+  </si>
+  <si>
+    <t>Endurance Max</t>
+  </si>
+  <si>
+    <t>Terrain d'entraînement</t>
+  </si>
+  <si>
+    <t>Centres +2
+Passes long. +2</t>
+  </si>
+  <si>
+    <t>Centres +5
+Passes long. +5</t>
+  </si>
+  <si>
+    <t>Passeur millimétré</t>
+  </si>
+  <si>
+    <t>Salle de musculation</t>
+  </si>
+  <si>
+    <t>Détente +2
+Force +2</t>
+  </si>
+  <si>
+    <t>Détente +5
+Force +5</t>
+  </si>
+  <si>
+    <t>Prof de yoga</t>
+  </si>
+  <si>
+    <t>Calme +2
+Équilibre +2</t>
+  </si>
+  <si>
+    <t>Calme +5
+Équilibre +5</t>
+  </si>
+  <si>
+    <t>Salle RV</t>
+  </si>
+  <si>
+    <t>Finition +2
+Passes court. +3</t>
+  </si>
+  <si>
+    <t>Finition +4
+Passes court. +5</t>
+  </si>
+  <si>
+    <t>Exercice de passe</t>
+  </si>
+  <si>
+    <t>Interceptions +3
+Passes long. +2</t>
+  </si>
+  <si>
+    <t>Interceptions +5
+Passes long. +5</t>
+  </si>
+  <si>
+    <t>Exercice Tir rasant appuyé</t>
+  </si>
+  <si>
+    <t>Équilibre +2
+Vista +3</t>
+  </si>
+  <si>
+    <t>Équilibre +5
+Vista +5</t>
+  </si>
+  <si>
+    <t>Tir rasant</t>
+  </si>
+  <si>
+    <t>Exercice de force</t>
+  </si>
+  <si>
+    <t>Force +2
+Tacles deb. +2</t>
+  </si>
+  <si>
+    <t>Force +4
+Tacles deb. +4</t>
+  </si>
+  <si>
+    <t>Exercice d'agilité</t>
+  </si>
+  <si>
+    <t>Agilité +2
+Conduite bal. +2</t>
+  </si>
+  <si>
+    <t>Agilité +3
+Conduite bal. +4</t>
+  </si>
+  <si>
+    <t>Exercice de finition rapide</t>
+  </si>
+  <si>
+    <t>Vit. sprint +2
+Finition +2</t>
+  </si>
+  <si>
+    <t>Vit. sprint +3
+Finition +3</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1612,8 +2061,32 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF2C481F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF2A3243"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF133819"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1646,8 +2119,26 @@
         <bgColor theme="0" tint="-0.14999847407452621"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF356854"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF6F8F9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="12">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -1796,11 +2287,176 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF284E3F"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF356854"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF284E3F"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF284E3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF356854"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF284E3F"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF284E3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF284E3F"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF284E3F"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF284E3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF284E3F"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF6F8F9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF6F8F9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF284E3F"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF6F8F9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF284E3F"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFF6F8F9"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF6F8F9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFF6F8F9"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFF6F8F9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF284E3F"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFF6F8F9"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF284E3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFF6F8F9"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF284E3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF284E3F"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF284E3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1870,6 +2526,72 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1886,22 +2608,152 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="10"/>
+        <sz val="11"/>
         <color theme="1"/>
-        <name val="Arial"/>
+        <name val="Calibri"/>
         <family val="2"/>
-        <scheme val="none"/>
+        <scheme val="minor"/>
       </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="medium">
-          <color rgb="FFCCCCCC"/>
-        </left>
-        <right style="medium">
-          <color rgb="FFCCCCCC"/>
-        </right>
-        <top/>
-        <bottom/>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="1"/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -1915,13 +2767,31 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="10"/>
+        <sz val="11"/>
         <color theme="1"/>
-        <name val="Arial"/>
+        <name val="Calibri"/>
         <family val="2"/>
-        <scheme val="none"/>
+        <scheme val="minor"/>
       </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -2138,13 +3008,6 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <bottom style="medium">
-          <color rgb="FFCCCCCC"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
         <left style="medium">
           <color rgb="FFCCCCCC"/>
         </left>
@@ -2170,151 +3033,18 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Calibri"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
       </font>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border outline="0">
-        <bottom style="thin">
-          <color theme="1"/>
+        <bottom style="medium">
+          <color rgb="FFCCCCCC"/>
         </bottom>
       </border>
     </dxf>
@@ -2329,31 +3059,23 @@
         <shadow val="0"/>
         <u val="none"/>
         <vertAlign val="baseline"/>
-        <sz val="11"/>
+        <sz val="10"/>
         <color theme="1"/>
-        <name val="Calibri"/>
+        <name val="Arial"/>
         <family val="2"/>
-        <scheme val="minor"/>
+        <scheme val="none"/>
       </font>
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="medium">
+          <color rgb="FFCCCCCC"/>
+        </left>
+        <right style="medium">
+          <color rgb="FFCCCCCC"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
     </dxf>
     <dxf>
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2514,33 +3236,33 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{37A655D1-0DF5-4AA5-9C00-06B8CC090F81}" name="Table7" displayName="Table7" ref="A3:F12" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1" headerRowBorderDxfId="9" tableBorderDxfId="10" totalsRowBorderDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{37A655D1-0DF5-4AA5-9C00-06B8CC090F81}" name="Table7" displayName="Table7" ref="A3:F12" totalsRowShown="0" headerRowDxfId="21" dataDxfId="19" headerRowBorderDxfId="20" tableBorderDxfId="18" totalsRowBorderDxfId="17">
   <autoFilter ref="A3:F12" xr:uid="{37A655D1-0DF5-4AA5-9C00-06B8CC090F81}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{F11B1075-68F6-4395-B0C8-031A344A1C23}" name="Taille/poids" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{C4B92BA3-B202-43A4-B535-66756F6F407B}" name="Poids min à Poids min+1" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{F6E0F7E8-5CE0-4563-8232-A8FE9F93B964}" name="Poids min+2 à Poids ref-1" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{9BBFA982-DA97-498B-BC86-CDA55BD7EA40}" name="Poids ref" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{6EB571C8-7488-4BEE-9D05-3D830C543BA2}" name="Poids ref+1 à Poids max-2" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{59D3449D-C179-4018-91A7-08DC076BDF10}" name="Poids max-1 à Poids max" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{F11B1075-68F6-4395-B0C8-031A344A1C23}" name="Taille/poids" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{C4B92BA3-B202-43A4-B535-66756F6F407B}" name="Poids min à Poids min+1" dataDxfId="15"/>
+    <tableColumn id="3" xr3:uid="{F6E0F7E8-5CE0-4563-8232-A8FE9F93B964}" name="Poids min+2 à Poids ref-1" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{9BBFA982-DA97-498B-BC86-CDA55BD7EA40}" name="Poids ref" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{6EB571C8-7488-4BEE-9D05-3D830C543BA2}" name="Poids ref+1 à Poids max-2" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{59D3449D-C179-4018-91A7-08DC076BDF10}" name="Poids max-1 à Poids max" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6A81EE77-924D-4A27-95C1-CE9387CD8489}" name="Table3" displayName="Table3" ref="A3:I47" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20" tableBorderDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6A81EE77-924D-4A27-95C1-CE9387CD8489}" name="Table3" displayName="Table3" ref="A3:I47" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9" tableBorderDxfId="8">
   <autoFilter ref="A3:I47" xr:uid="{6A81EE77-924D-4A27-95C1-CE9387CD8489}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{12AC2442-EFF1-4896-9682-029BD4855046}" name="archetype"/>
-    <tableColumn id="2" xr3:uid="{B0F8B123-2089-4583-98A2-1995CD85B977}" name="specialisation" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{D6662864-025C-46A1-8303-CE0241C67FAC}" name="archetype_gagne" dataDxfId="17"/>
-    <tableColumn id="4" xr3:uid="{097C53EC-F167-40A0-88C4-6CEFF6FF8BCE}" name="attribut_1" dataDxfId="16"/>
-    <tableColumn id="5" xr3:uid="{E92A705B-E623-4A97-8682-9EC30D60A096}" name="seuil_1" dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{BF3FD942-E38F-4482-BCB6-E799211ADE0D}" name="attribut_2" dataDxfId="14"/>
-    <tableColumn id="7" xr3:uid="{056E39F8-4575-4903-82BA-79D150ED3762}" name="seuil_2" dataDxfId="13"/>
-    <tableColumn id="8" xr3:uid="{EAE8CCB1-E087-4202-8112-99A7DBD7D58B}" name="attribut_3" dataDxfId="12"/>
-    <tableColumn id="9" xr3:uid="{105A4E71-173F-44F1-B3FE-A54F63DAC055}" name="seuil_3" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{B0F8B123-2089-4583-98A2-1995CD85B977}" name="specialisation" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{D6662864-025C-46A1-8303-CE0241C67FAC}" name="archetype_gagne" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{097C53EC-F167-40A0-88C4-6CEFF6FF8BCE}" name="attribut_1" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{E92A705B-E623-4A97-8682-9EC30D60A096}" name="seuil_1" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{BF3FD942-E38F-4482-BCB6-E799211ADE0D}" name="attribut_2" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{056E39F8-4575-4903-82BA-79D150ED3762}" name="seuil_2" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{EAE8CCB1-E087-4202-8112-99A7DBD7D58B}" name="attribut_3" dataDxfId="1"/>
+    <tableColumn id="9" xr3:uid="{105A4E71-173F-44F1-B3FE-A54F63DAC055}" name="seuil_3" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -15487,7 +16209,7 @@
       <c r="Y3" s="23"/>
       <c r="Z3" s="23"/>
     </row>
-    <row r="4" spans="1:26" ht="129" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="25" t="s">
         <v>353</v>
       </c>
@@ -15527,7 +16249,7 @@
       <c r="Y4" s="23"/>
       <c r="Z4" s="23"/>
     </row>
-    <row r="5" spans="1:26" ht="167.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="25" t="s">
         <v>359</v>
       </c>
@@ -15567,7 +16289,7 @@
       <c r="Y5" s="23"/>
       <c r="Z5" s="23"/>
     </row>
-    <row r="6" spans="1:26" ht="167.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="25" t="s">
         <v>365</v>
       </c>
@@ -15607,7 +16329,7 @@
       <c r="Y6" s="23"/>
       <c r="Z6" s="23"/>
     </row>
-    <row r="7" spans="1:26" ht="167.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="25" t="s">
         <v>371</v>
       </c>
@@ -15647,7 +16369,7 @@
       <c r="Y7" s="23"/>
       <c r="Z7" s="23"/>
     </row>
-    <row r="8" spans="1:26" ht="167.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="25" t="s">
         <v>377</v>
       </c>
@@ -15687,7 +16409,7 @@
       <c r="Y8" s="23"/>
       <c r="Z8" s="23"/>
     </row>
-    <row r="9" spans="1:26" ht="167.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="25" t="s">
         <v>383</v>
       </c>
@@ -15727,7 +16449,7 @@
       <c r="Y9" s="23"/>
       <c r="Z9" s="23"/>
     </row>
-    <row r="10" spans="1:26" ht="154.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="25" t="s">
         <v>389</v>
       </c>
@@ -15767,7 +16489,7 @@
       <c r="Y10" s="23"/>
       <c r="Z10" s="23"/>
     </row>
-    <row r="11" spans="1:26" ht="129" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="25" t="s">
         <v>395</v>
       </c>
@@ -15807,7 +16529,7 @@
       <c r="Y11" s="23"/>
       <c r="Z11" s="23"/>
     </row>
-    <row r="12" spans="1:26" ht="129" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:26" ht="78" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="30" t="s">
         <v>401</v>
       </c>
@@ -44462,7 +45184,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="19" t="s">
         <v>63</v>
       </c>
@@ -44479,7 +45201,7 @@
       <c r="H24" s="20"/>
       <c r="I24" s="18"/>
     </row>
-    <row r="25" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>63</v>
       </c>
@@ -44537,7 +45259,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>63</v>
       </c>
@@ -44566,7 +45288,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="19" t="s">
         <v>69</v>
       </c>
@@ -45095,6 +45817,1774 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{869A7E21-E2BD-40BD-B5E6-9B5F096E5A12}">
+  <dimension ref="A1:E103"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="23.28515625" customWidth="1"/>
+    <col min="2" max="2" width="10.7109375" customWidth="1"/>
+    <col min="3" max="3" width="8.7109375" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" customWidth="1"/>
+    <col min="5" max="5" width="15.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="33" t="s">
+        <v>423</v>
+      </c>
+      <c r="B1" s="34" t="s">
+        <v>424</v>
+      </c>
+      <c r="C1" s="34" t="s">
+        <v>425</v>
+      </c>
+      <c r="D1" s="34" t="s">
+        <v>426</v>
+      </c>
+      <c r="E1" s="35" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="36" t="s">
+        <v>428</v>
+      </c>
+      <c r="B2" s="38" t="s">
+        <v>429</v>
+      </c>
+      <c r="C2" s="39">
+        <v>200000</v>
+      </c>
+      <c r="D2" s="37" t="s">
+        <v>430</v>
+      </c>
+      <c r="E2" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="41" t="s">
+        <v>428</v>
+      </c>
+      <c r="B3" s="43" t="s">
+        <v>432</v>
+      </c>
+      <c r="C3" s="44">
+        <v>600000</v>
+      </c>
+      <c r="D3" s="42" t="s">
+        <v>433</v>
+      </c>
+      <c r="E3" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="36" t="s">
+        <v>428</v>
+      </c>
+      <c r="B4" s="46" t="s">
+        <v>434</v>
+      </c>
+      <c r="C4" s="39">
+        <v>1200000</v>
+      </c>
+      <c r="D4" s="37" t="s">
+        <v>435</v>
+      </c>
+      <c r="E4" s="40" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="41" t="s">
+        <v>436</v>
+      </c>
+      <c r="B5" s="47" t="s">
+        <v>429</v>
+      </c>
+      <c r="C5" s="44">
+        <v>200000</v>
+      </c>
+      <c r="D5" s="42" t="s">
+        <v>437</v>
+      </c>
+      <c r="E5" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="36" t="s">
+        <v>436</v>
+      </c>
+      <c r="B6" s="48" t="s">
+        <v>432</v>
+      </c>
+      <c r="C6" s="39">
+        <v>600000</v>
+      </c>
+      <c r="D6" s="37" t="s">
+        <v>438</v>
+      </c>
+      <c r="E6" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="41" t="s">
+        <v>436</v>
+      </c>
+      <c r="B7" s="49" t="s">
+        <v>434</v>
+      </c>
+      <c r="C7" s="44">
+        <v>1200000</v>
+      </c>
+      <c r="D7" s="42" t="s">
+        <v>438</v>
+      </c>
+      <c r="E7" s="45" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="36" t="s">
+        <v>439</v>
+      </c>
+      <c r="B8" s="38" t="s">
+        <v>429</v>
+      </c>
+      <c r="C8" s="39">
+        <v>200000</v>
+      </c>
+      <c r="D8" s="37" t="s">
+        <v>440</v>
+      </c>
+      <c r="E8" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="41" t="s">
+        <v>439</v>
+      </c>
+      <c r="B9" s="43" t="s">
+        <v>432</v>
+      </c>
+      <c r="C9" s="44">
+        <v>600000</v>
+      </c>
+      <c r="D9" s="42" t="s">
+        <v>441</v>
+      </c>
+      <c r="E9" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="36" t="s">
+        <v>439</v>
+      </c>
+      <c r="B10" s="46" t="s">
+        <v>434</v>
+      </c>
+      <c r="C10" s="39">
+        <v>1200000</v>
+      </c>
+      <c r="D10" s="37" t="s">
+        <v>442</v>
+      </c>
+      <c r="E10" s="40" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="41" t="s">
+        <v>443</v>
+      </c>
+      <c r="B11" s="47" t="s">
+        <v>429</v>
+      </c>
+      <c r="C11" s="44">
+        <v>100000</v>
+      </c>
+      <c r="D11" s="42" t="s">
+        <v>444</v>
+      </c>
+      <c r="E11" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="36" t="s">
+        <v>443</v>
+      </c>
+      <c r="B12" s="48" t="s">
+        <v>432</v>
+      </c>
+      <c r="C12" s="39">
+        <v>400000</v>
+      </c>
+      <c r="D12" s="37" t="s">
+        <v>445</v>
+      </c>
+      <c r="E12" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="41" t="s">
+        <v>443</v>
+      </c>
+      <c r="B13" s="49" t="s">
+        <v>434</v>
+      </c>
+      <c r="C13" s="44">
+        <v>1100000</v>
+      </c>
+      <c r="D13" s="42" t="s">
+        <v>446</v>
+      </c>
+      <c r="E13" s="45" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="36" t="s">
+        <v>447</v>
+      </c>
+      <c r="B14" s="38" t="s">
+        <v>429</v>
+      </c>
+      <c r="C14" s="39">
+        <v>100000</v>
+      </c>
+      <c r="D14" s="37" t="s">
+        <v>448</v>
+      </c>
+      <c r="E14" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="41" t="s">
+        <v>447</v>
+      </c>
+      <c r="B15" s="43" t="s">
+        <v>432</v>
+      </c>
+      <c r="C15" s="44">
+        <v>400000</v>
+      </c>
+      <c r="D15" s="42" t="s">
+        <v>449</v>
+      </c>
+      <c r="E15" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="36" t="s">
+        <v>447</v>
+      </c>
+      <c r="B16" s="46" t="s">
+        <v>434</v>
+      </c>
+      <c r="C16" s="39">
+        <v>1100000</v>
+      </c>
+      <c r="D16" s="37" t="s">
+        <v>449</v>
+      </c>
+      <c r="E16" s="40" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="41" t="s">
+        <v>450</v>
+      </c>
+      <c r="B17" s="47" t="s">
+        <v>429</v>
+      </c>
+      <c r="C17" s="44">
+        <v>200000</v>
+      </c>
+      <c r="D17" s="42" t="s">
+        <v>451</v>
+      </c>
+      <c r="E17" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="36" t="s">
+        <v>450</v>
+      </c>
+      <c r="B18" s="48" t="s">
+        <v>432</v>
+      </c>
+      <c r="C18" s="39">
+        <v>600000</v>
+      </c>
+      <c r="D18" s="37" t="s">
+        <v>452</v>
+      </c>
+      <c r="E18" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="41" t="s">
+        <v>450</v>
+      </c>
+      <c r="B19" s="49" t="s">
+        <v>434</v>
+      </c>
+      <c r="C19" s="44">
+        <v>1200000</v>
+      </c>
+      <c r="D19" s="42" t="s">
+        <v>452</v>
+      </c>
+      <c r="E19" s="45" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="36" t="s">
+        <v>454</v>
+      </c>
+      <c r="B20" s="38" t="s">
+        <v>429</v>
+      </c>
+      <c r="C20" s="39">
+        <v>100000</v>
+      </c>
+      <c r="D20" s="37" t="s">
+        <v>455</v>
+      </c>
+      <c r="E20" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="41" t="s">
+        <v>454</v>
+      </c>
+      <c r="B21" s="43" t="s">
+        <v>432</v>
+      </c>
+      <c r="C21" s="44">
+        <v>400000</v>
+      </c>
+      <c r="D21" s="42" t="s">
+        <v>456</v>
+      </c>
+      <c r="E21" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="36" t="s">
+        <v>454</v>
+      </c>
+      <c r="B22" s="46" t="s">
+        <v>434</v>
+      </c>
+      <c r="C22" s="39">
+        <v>1100000</v>
+      </c>
+      <c r="D22" s="37" t="s">
+        <v>456</v>
+      </c>
+      <c r="E22" s="40" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="41" t="s">
+        <v>458</v>
+      </c>
+      <c r="B23" s="47" t="s">
+        <v>429</v>
+      </c>
+      <c r="C23" s="44">
+        <v>100000</v>
+      </c>
+      <c r="D23" s="42" t="s">
+        <v>459</v>
+      </c>
+      <c r="E23" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="36" t="s">
+        <v>458</v>
+      </c>
+      <c r="B24" s="48" t="s">
+        <v>432</v>
+      </c>
+      <c r="C24" s="39">
+        <v>400000</v>
+      </c>
+      <c r="D24" s="37" t="s">
+        <v>460</v>
+      </c>
+      <c r="E24" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="41" t="s">
+        <v>458</v>
+      </c>
+      <c r="B25" s="49" t="s">
+        <v>434</v>
+      </c>
+      <c r="C25" s="44">
+        <v>1100000</v>
+      </c>
+      <c r="D25" s="42" t="s">
+        <v>460</v>
+      </c>
+      <c r="E25" s="45" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="36" t="s">
+        <v>461</v>
+      </c>
+      <c r="B26" s="38" t="s">
+        <v>429</v>
+      </c>
+      <c r="C26" s="39">
+        <v>200000</v>
+      </c>
+      <c r="D26" s="37" t="s">
+        <v>430</v>
+      </c>
+      <c r="E26" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="41" t="s">
+        <v>461</v>
+      </c>
+      <c r="B27" s="43" t="s">
+        <v>432</v>
+      </c>
+      <c r="C27" s="44">
+        <v>600000</v>
+      </c>
+      <c r="D27" s="42" t="s">
+        <v>462</v>
+      </c>
+      <c r="E27" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="36" t="s">
+        <v>461</v>
+      </c>
+      <c r="B28" s="46" t="s">
+        <v>434</v>
+      </c>
+      <c r="C28" s="39">
+        <v>1200000</v>
+      </c>
+      <c r="D28" s="37" t="s">
+        <v>462</v>
+      </c>
+      <c r="E28" s="40" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="41" t="s">
+        <v>463</v>
+      </c>
+      <c r="B29" s="47" t="s">
+        <v>429</v>
+      </c>
+      <c r="C29" s="44">
+        <v>100000</v>
+      </c>
+      <c r="D29" s="42" t="s">
+        <v>464</v>
+      </c>
+      <c r="E29" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="36" t="s">
+        <v>463</v>
+      </c>
+      <c r="B30" s="48" t="s">
+        <v>432</v>
+      </c>
+      <c r="C30" s="39">
+        <v>400000</v>
+      </c>
+      <c r="D30" s="37" t="s">
+        <v>465</v>
+      </c>
+      <c r="E30" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="41" t="s">
+        <v>463</v>
+      </c>
+      <c r="B31" s="49" t="s">
+        <v>434</v>
+      </c>
+      <c r="C31" s="44">
+        <v>1100000</v>
+      </c>
+      <c r="D31" s="42" t="s">
+        <v>465</v>
+      </c>
+      <c r="E31" s="45" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="36" t="s">
+        <v>467</v>
+      </c>
+      <c r="B32" s="38" t="s">
+        <v>429</v>
+      </c>
+      <c r="C32" s="39">
+        <v>200000</v>
+      </c>
+      <c r="D32" s="37" t="s">
+        <v>468</v>
+      </c>
+      <c r="E32" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="41" t="s">
+        <v>467</v>
+      </c>
+      <c r="B33" s="43" t="s">
+        <v>432</v>
+      </c>
+      <c r="C33" s="44">
+        <v>600000</v>
+      </c>
+      <c r="D33" s="42" t="s">
+        <v>469</v>
+      </c>
+      <c r="E33" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="36" t="s">
+        <v>467</v>
+      </c>
+      <c r="B34" s="46" t="s">
+        <v>434</v>
+      </c>
+      <c r="C34" s="39">
+        <v>1200000</v>
+      </c>
+      <c r="D34" s="37" t="s">
+        <v>469</v>
+      </c>
+      <c r="E34" s="40" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="41" t="s">
+        <v>470</v>
+      </c>
+      <c r="B35" s="47" t="s">
+        <v>429</v>
+      </c>
+      <c r="C35" s="44">
+        <v>300000</v>
+      </c>
+      <c r="D35" s="42" t="s">
+        <v>471</v>
+      </c>
+      <c r="E35" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="36" t="s">
+        <v>470</v>
+      </c>
+      <c r="B36" s="48" t="s">
+        <v>432</v>
+      </c>
+      <c r="C36" s="39">
+        <v>800000</v>
+      </c>
+      <c r="D36" s="37" t="s">
+        <v>472</v>
+      </c>
+      <c r="E36" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="41" t="s">
+        <v>470</v>
+      </c>
+      <c r="B37" s="49" t="s">
+        <v>434</v>
+      </c>
+      <c r="C37" s="44">
+        <v>1400000</v>
+      </c>
+      <c r="D37" s="42" t="s">
+        <v>472</v>
+      </c>
+      <c r="E37" s="45" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="36" t="s">
+        <v>473</v>
+      </c>
+      <c r="B38" s="38" t="s">
+        <v>429</v>
+      </c>
+      <c r="C38" s="39">
+        <v>300000</v>
+      </c>
+      <c r="D38" s="37" t="s">
+        <v>474</v>
+      </c>
+      <c r="E38" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="41" t="s">
+        <v>473</v>
+      </c>
+      <c r="B39" s="43" t="s">
+        <v>432</v>
+      </c>
+      <c r="C39" s="44">
+        <v>800000</v>
+      </c>
+      <c r="D39" s="42" t="s">
+        <v>475</v>
+      </c>
+      <c r="E39" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="36" t="s">
+        <v>473</v>
+      </c>
+      <c r="B40" s="46" t="s">
+        <v>434</v>
+      </c>
+      <c r="C40" s="39">
+        <v>1400000</v>
+      </c>
+      <c r="D40" s="37" t="s">
+        <v>475</v>
+      </c>
+      <c r="E40" s="40" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="41" t="s">
+        <v>476</v>
+      </c>
+      <c r="B41" s="47" t="s">
+        <v>429</v>
+      </c>
+      <c r="C41" s="44">
+        <v>300000</v>
+      </c>
+      <c r="D41" s="42" t="s">
+        <v>477</v>
+      </c>
+      <c r="E41" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="36" t="s">
+        <v>476</v>
+      </c>
+      <c r="B42" s="48" t="s">
+        <v>432</v>
+      </c>
+      <c r="C42" s="39">
+        <v>800000</v>
+      </c>
+      <c r="D42" s="37" t="s">
+        <v>478</v>
+      </c>
+      <c r="E42" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="41" t="s">
+        <v>476</v>
+      </c>
+      <c r="B43" s="49" t="s">
+        <v>434</v>
+      </c>
+      <c r="C43" s="44">
+        <v>1400000</v>
+      </c>
+      <c r="D43" s="42" t="s">
+        <v>478</v>
+      </c>
+      <c r="E43" s="45" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="36" t="s">
+        <v>479</v>
+      </c>
+      <c r="B44" s="38" t="s">
+        <v>429</v>
+      </c>
+      <c r="C44" s="39">
+        <v>300000</v>
+      </c>
+      <c r="D44" s="37" t="s">
+        <v>480</v>
+      </c>
+      <c r="E44" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="41" t="s">
+        <v>479</v>
+      </c>
+      <c r="B45" s="43" t="s">
+        <v>432</v>
+      </c>
+      <c r="C45" s="44">
+        <v>800000</v>
+      </c>
+      <c r="D45" s="42" t="s">
+        <v>481</v>
+      </c>
+      <c r="E45" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="36" t="s">
+        <v>479</v>
+      </c>
+      <c r="B46" s="46" t="s">
+        <v>434</v>
+      </c>
+      <c r="C46" s="39">
+        <v>1400000</v>
+      </c>
+      <c r="D46" s="37" t="s">
+        <v>481</v>
+      </c>
+      <c r="E46" s="40" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="41" t="s">
+        <v>483</v>
+      </c>
+      <c r="B47" s="47" t="s">
+        <v>429</v>
+      </c>
+      <c r="C47" s="44">
+        <v>100000</v>
+      </c>
+      <c r="D47" s="42" t="s">
+        <v>484</v>
+      </c>
+      <c r="E47" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="36" t="s">
+        <v>483</v>
+      </c>
+      <c r="B48" s="48" t="s">
+        <v>432</v>
+      </c>
+      <c r="C48" s="39">
+        <v>400000</v>
+      </c>
+      <c r="D48" s="37" t="s">
+        <v>485</v>
+      </c>
+      <c r="E48" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="41" t="s">
+        <v>483</v>
+      </c>
+      <c r="B49" s="49" t="s">
+        <v>434</v>
+      </c>
+      <c r="C49" s="44">
+        <v>1100000</v>
+      </c>
+      <c r="D49" s="42" t="s">
+        <v>485</v>
+      </c>
+      <c r="E49" s="45" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="36" t="s">
+        <v>487</v>
+      </c>
+      <c r="B50" s="38" t="s">
+        <v>429</v>
+      </c>
+      <c r="C50" s="39">
+        <v>300000</v>
+      </c>
+      <c r="D50" s="37" t="s">
+        <v>488</v>
+      </c>
+      <c r="E50" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="41" t="s">
+        <v>487</v>
+      </c>
+      <c r="B51" s="43" t="s">
+        <v>432</v>
+      </c>
+      <c r="C51" s="44">
+        <v>800000</v>
+      </c>
+      <c r="D51" s="42" t="s">
+        <v>489</v>
+      </c>
+      <c r="E51" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="36" t="s">
+        <v>487</v>
+      </c>
+      <c r="B52" s="46" t="s">
+        <v>434</v>
+      </c>
+      <c r="C52" s="39">
+        <v>1400000</v>
+      </c>
+      <c r="D52" s="37" t="s">
+        <v>489</v>
+      </c>
+      <c r="E52" s="40" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="41" t="s">
+        <v>490</v>
+      </c>
+      <c r="B53" s="47" t="s">
+        <v>429</v>
+      </c>
+      <c r="C53" s="44">
+        <v>100000</v>
+      </c>
+      <c r="D53" s="42" t="s">
+        <v>491</v>
+      </c>
+      <c r="E53" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="36" t="s">
+        <v>490</v>
+      </c>
+      <c r="B54" s="48" t="s">
+        <v>432</v>
+      </c>
+      <c r="C54" s="39">
+        <v>400000</v>
+      </c>
+      <c r="D54" s="37" t="s">
+        <v>492</v>
+      </c>
+      <c r="E54" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="41" t="s">
+        <v>490</v>
+      </c>
+      <c r="B55" s="49" t="s">
+        <v>434</v>
+      </c>
+      <c r="C55" s="44">
+        <v>1100000</v>
+      </c>
+      <c r="D55" s="42" t="s">
+        <v>492</v>
+      </c>
+      <c r="E55" s="45" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="36" t="s">
+        <v>493</v>
+      </c>
+      <c r="B56" s="38" t="s">
+        <v>429</v>
+      </c>
+      <c r="C56" s="39">
+        <v>200000</v>
+      </c>
+      <c r="D56" s="37" t="s">
+        <v>494</v>
+      </c>
+      <c r="E56" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="41" t="s">
+        <v>493</v>
+      </c>
+      <c r="B57" s="43" t="s">
+        <v>432</v>
+      </c>
+      <c r="C57" s="44">
+        <v>600000</v>
+      </c>
+      <c r="D57" s="42" t="s">
+        <v>495</v>
+      </c>
+      <c r="E57" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A58" s="36" t="s">
+        <v>493</v>
+      </c>
+      <c r="B58" s="46" t="s">
+        <v>434</v>
+      </c>
+      <c r="C58" s="39">
+        <v>1200000</v>
+      </c>
+      <c r="D58" s="37" t="s">
+        <v>496</v>
+      </c>
+      <c r="E58" s="40" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="41" t="s">
+        <v>497</v>
+      </c>
+      <c r="B59" s="47" t="s">
+        <v>429</v>
+      </c>
+      <c r="C59" s="44">
+        <v>300000</v>
+      </c>
+      <c r="D59" s="42" t="s">
+        <v>498</v>
+      </c>
+      <c r="E59" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="36" t="s">
+        <v>497</v>
+      </c>
+      <c r="B60" s="48" t="s">
+        <v>432</v>
+      </c>
+      <c r="C60" s="39">
+        <v>800000</v>
+      </c>
+      <c r="D60" s="37" t="s">
+        <v>499</v>
+      </c>
+      <c r="E60" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="41" t="s">
+        <v>497</v>
+      </c>
+      <c r="B61" s="49" t="s">
+        <v>434</v>
+      </c>
+      <c r="C61" s="44">
+        <v>1400000</v>
+      </c>
+      <c r="D61" s="42" t="s">
+        <v>499</v>
+      </c>
+      <c r="E61" s="45" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A62" s="36" t="s">
+        <v>500</v>
+      </c>
+      <c r="B62" s="38" t="s">
+        <v>429</v>
+      </c>
+      <c r="C62" s="39">
+        <v>100000</v>
+      </c>
+      <c r="D62" s="37" t="s">
+        <v>501</v>
+      </c>
+      <c r="E62" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="41" t="s">
+        <v>500</v>
+      </c>
+      <c r="B63" s="43" t="s">
+        <v>432</v>
+      </c>
+      <c r="C63" s="44">
+        <v>400000</v>
+      </c>
+      <c r="D63" s="42" t="s">
+        <v>502</v>
+      </c>
+      <c r="E63" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="36" t="s">
+        <v>500</v>
+      </c>
+      <c r="B64" s="46" t="s">
+        <v>434</v>
+      </c>
+      <c r="C64" s="39">
+        <v>1100000</v>
+      </c>
+      <c r="D64" s="37" t="s">
+        <v>502</v>
+      </c>
+      <c r="E64" s="40" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="41" t="s">
+        <v>503</v>
+      </c>
+      <c r="B65" s="47" t="s">
+        <v>429</v>
+      </c>
+      <c r="C65" s="44">
+        <v>200000</v>
+      </c>
+      <c r="D65" s="42" t="s">
+        <v>504</v>
+      </c>
+      <c r="E65" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A66" s="36" t="s">
+        <v>503</v>
+      </c>
+      <c r="B66" s="48" t="s">
+        <v>432</v>
+      </c>
+      <c r="C66" s="39">
+        <v>600000</v>
+      </c>
+      <c r="D66" s="37" t="s">
+        <v>505</v>
+      </c>
+      <c r="E66" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A67" s="41" t="s">
+        <v>503</v>
+      </c>
+      <c r="B67" s="49" t="s">
+        <v>434</v>
+      </c>
+      <c r="C67" s="44">
+        <v>1200000</v>
+      </c>
+      <c r="D67" s="42" t="s">
+        <v>505</v>
+      </c>
+      <c r="E67" s="45" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A68" s="36" t="s">
+        <v>506</v>
+      </c>
+      <c r="B68" s="38" t="s">
+        <v>429</v>
+      </c>
+      <c r="C68" s="39">
+        <v>300000</v>
+      </c>
+      <c r="D68" s="37" t="s">
+        <v>507</v>
+      </c>
+      <c r="E68" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="41" t="s">
+        <v>506</v>
+      </c>
+      <c r="B69" s="43" t="s">
+        <v>432</v>
+      </c>
+      <c r="C69" s="44">
+        <v>800000</v>
+      </c>
+      <c r="D69" s="42" t="s">
+        <v>508</v>
+      </c>
+      <c r="E69" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="36" t="s">
+        <v>506</v>
+      </c>
+      <c r="B70" s="46" t="s">
+        <v>434</v>
+      </c>
+      <c r="C70" s="39">
+        <v>1400000</v>
+      </c>
+      <c r="D70" s="37" t="s">
+        <v>509</v>
+      </c>
+      <c r="E70" s="40" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="41" t="s">
+        <v>510</v>
+      </c>
+      <c r="B71" s="47" t="s">
+        <v>429</v>
+      </c>
+      <c r="C71" s="44">
+        <v>200000</v>
+      </c>
+      <c r="D71" s="42" t="s">
+        <v>511</v>
+      </c>
+      <c r="E71" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="36" t="s">
+        <v>510</v>
+      </c>
+      <c r="B72" s="48" t="s">
+        <v>432</v>
+      </c>
+      <c r="C72" s="39">
+        <v>600000</v>
+      </c>
+      <c r="D72" s="37" t="s">
+        <v>512</v>
+      </c>
+      <c r="E72" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="41" t="s">
+        <v>510</v>
+      </c>
+      <c r="B73" s="49" t="s">
+        <v>434</v>
+      </c>
+      <c r="C73" s="44">
+        <v>1200000</v>
+      </c>
+      <c r="D73" s="42" t="s">
+        <v>512</v>
+      </c>
+      <c r="E73" s="45" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="36" t="s">
+        <v>514</v>
+      </c>
+      <c r="B74" s="38" t="s">
+        <v>429</v>
+      </c>
+      <c r="C74" s="39">
+        <v>300000</v>
+      </c>
+      <c r="D74" s="37" t="s">
+        <v>515</v>
+      </c>
+      <c r="E74" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A75" s="41" t="s">
+        <v>514</v>
+      </c>
+      <c r="B75" s="43" t="s">
+        <v>432</v>
+      </c>
+      <c r="C75" s="44">
+        <v>800000</v>
+      </c>
+      <c r="D75" s="42" t="s">
+        <v>516</v>
+      </c>
+      <c r="E75" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="36" t="s">
+        <v>514</v>
+      </c>
+      <c r="B76" s="46" t="s">
+        <v>434</v>
+      </c>
+      <c r="C76" s="39">
+        <v>1400000</v>
+      </c>
+      <c r="D76" s="37" t="s">
+        <v>517</v>
+      </c>
+      <c r="E76" s="40" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A77" s="41" t="s">
+        <v>519</v>
+      </c>
+      <c r="B77" s="47" t="s">
+        <v>429</v>
+      </c>
+      <c r="C77" s="44">
+        <v>200000</v>
+      </c>
+      <c r="D77" s="42" t="s">
+        <v>520</v>
+      </c>
+      <c r="E77" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A78" s="36" t="s">
+        <v>519</v>
+      </c>
+      <c r="B78" s="48" t="s">
+        <v>432</v>
+      </c>
+      <c r="C78" s="39">
+        <v>600000</v>
+      </c>
+      <c r="D78" s="37" t="s">
+        <v>521</v>
+      </c>
+      <c r="E78" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="41" t="s">
+        <v>519</v>
+      </c>
+      <c r="B79" s="49" t="s">
+        <v>434</v>
+      </c>
+      <c r="C79" s="44">
+        <v>1200000</v>
+      </c>
+      <c r="D79" s="42" t="s">
+        <v>521</v>
+      </c>
+      <c r="E79" s="45" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="36" t="s">
+        <v>523</v>
+      </c>
+      <c r="B80" s="38" t="s">
+        <v>429</v>
+      </c>
+      <c r="C80" s="39">
+        <v>200000</v>
+      </c>
+      <c r="D80" s="37" t="s">
+        <v>524</v>
+      </c>
+      <c r="E80" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="41" t="s">
+        <v>523</v>
+      </c>
+      <c r="B81" s="43" t="s">
+        <v>432</v>
+      </c>
+      <c r="C81" s="44">
+        <v>600000</v>
+      </c>
+      <c r="D81" s="42" t="s">
+        <v>525</v>
+      </c>
+      <c r="E81" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A82" s="36" t="s">
+        <v>523</v>
+      </c>
+      <c r="B82" s="46" t="s">
+        <v>434</v>
+      </c>
+      <c r="C82" s="39">
+        <v>1200000</v>
+      </c>
+      <c r="D82" s="37" t="s">
+        <v>525</v>
+      </c>
+      <c r="E82" s="40" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="41" t="s">
+        <v>526</v>
+      </c>
+      <c r="B83" s="47" t="s">
+        <v>429</v>
+      </c>
+      <c r="C83" s="44">
+        <v>200000</v>
+      </c>
+      <c r="D83" s="42" t="s">
+        <v>527</v>
+      </c>
+      <c r="E83" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A84" s="36" t="s">
+        <v>526</v>
+      </c>
+      <c r="B84" s="48" t="s">
+        <v>432</v>
+      </c>
+      <c r="C84" s="39">
+        <v>600000</v>
+      </c>
+      <c r="D84" s="37" t="s">
+        <v>528</v>
+      </c>
+      <c r="E84" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A85" s="41" t="s">
+        <v>526</v>
+      </c>
+      <c r="B85" s="49" t="s">
+        <v>434</v>
+      </c>
+      <c r="C85" s="44">
+        <v>1200000</v>
+      </c>
+      <c r="D85" s="42" t="s">
+        <v>528</v>
+      </c>
+      <c r="E85" s="45" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A86" s="36" t="s">
+        <v>529</v>
+      </c>
+      <c r="B86" s="38" t="s">
+        <v>429</v>
+      </c>
+      <c r="C86" s="39">
+        <v>200000</v>
+      </c>
+      <c r="D86" s="37" t="s">
+        <v>530</v>
+      </c>
+      <c r="E86" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="41" t="s">
+        <v>529</v>
+      </c>
+      <c r="B87" s="43" t="s">
+        <v>432</v>
+      </c>
+      <c r="C87" s="44">
+        <v>600000</v>
+      </c>
+      <c r="D87" s="42" t="s">
+        <v>531</v>
+      </c>
+      <c r="E87" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A88" s="36" t="s">
+        <v>529</v>
+      </c>
+      <c r="B88" s="46" t="s">
+        <v>434</v>
+      </c>
+      <c r="C88" s="39">
+        <v>1200000</v>
+      </c>
+      <c r="D88" s="37" t="s">
+        <v>531</v>
+      </c>
+      <c r="E88" s="40" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A89" s="41" t="s">
+        <v>532</v>
+      </c>
+      <c r="B89" s="47" t="s">
+        <v>429</v>
+      </c>
+      <c r="C89" s="44">
+        <v>200000</v>
+      </c>
+      <c r="D89" s="42" t="s">
+        <v>533</v>
+      </c>
+      <c r="E89" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A90" s="36" t="s">
+        <v>532</v>
+      </c>
+      <c r="B90" s="48" t="s">
+        <v>432</v>
+      </c>
+      <c r="C90" s="39">
+        <v>600000</v>
+      </c>
+      <c r="D90" s="37" t="s">
+        <v>534</v>
+      </c>
+      <c r="E90" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" ht="52.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A91" s="41" t="s">
+        <v>532</v>
+      </c>
+      <c r="B91" s="49" t="s">
+        <v>434</v>
+      </c>
+      <c r="C91" s="44">
+        <v>1200000</v>
+      </c>
+      <c r="D91" s="42" t="s">
+        <v>534</v>
+      </c>
+      <c r="E91" s="45" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A92" s="36" t="s">
+        <v>535</v>
+      </c>
+      <c r="B92" s="38" t="s">
+        <v>429</v>
+      </c>
+      <c r="C92" s="39">
+        <v>200000</v>
+      </c>
+      <c r="D92" s="37" t="s">
+        <v>536</v>
+      </c>
+      <c r="E92" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A93" s="41" t="s">
+        <v>535</v>
+      </c>
+      <c r="B93" s="43" t="s">
+        <v>432</v>
+      </c>
+      <c r="C93" s="44">
+        <v>600000</v>
+      </c>
+      <c r="D93" s="42" t="s">
+        <v>537</v>
+      </c>
+      <c r="E93" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A94" s="36" t="s">
+        <v>535</v>
+      </c>
+      <c r="B94" s="46" t="s">
+        <v>434</v>
+      </c>
+      <c r="C94" s="39">
+        <v>1200000</v>
+      </c>
+      <c r="D94" s="37" t="s">
+        <v>537</v>
+      </c>
+      <c r="E94" s="40" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A95" s="41" t="s">
+        <v>539</v>
+      </c>
+      <c r="B95" s="47" t="s">
+        <v>429</v>
+      </c>
+      <c r="C95" s="44">
+        <v>300000</v>
+      </c>
+      <c r="D95" s="42" t="s">
+        <v>540</v>
+      </c>
+      <c r="E95" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A96" s="36" t="s">
+        <v>539</v>
+      </c>
+      <c r="B96" s="48" t="s">
+        <v>432</v>
+      </c>
+      <c r="C96" s="39">
+        <v>800000</v>
+      </c>
+      <c r="D96" s="37" t="s">
+        <v>541</v>
+      </c>
+      <c r="E96" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A97" s="41" t="s">
+        <v>539</v>
+      </c>
+      <c r="B97" s="49" t="s">
+        <v>434</v>
+      </c>
+      <c r="C97" s="44">
+        <v>1400000</v>
+      </c>
+      <c r="D97" s="42" t="s">
+        <v>541</v>
+      </c>
+      <c r="E97" s="45" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A98" s="36" t="s">
+        <v>542</v>
+      </c>
+      <c r="B98" s="38" t="s">
+        <v>429</v>
+      </c>
+      <c r="C98" s="39">
+        <v>300000</v>
+      </c>
+      <c r="D98" s="37" t="s">
+        <v>543</v>
+      </c>
+      <c r="E98" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A99" s="41" t="s">
+        <v>542</v>
+      </c>
+      <c r="B99" s="43" t="s">
+        <v>432</v>
+      </c>
+      <c r="C99" s="44">
+        <v>800000</v>
+      </c>
+      <c r="D99" s="42" t="s">
+        <v>544</v>
+      </c>
+      <c r="E99" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" ht="39.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A100" s="36" t="s">
+        <v>542</v>
+      </c>
+      <c r="B100" s="46" t="s">
+        <v>434</v>
+      </c>
+      <c r="C100" s="39">
+        <v>1400000</v>
+      </c>
+      <c r="D100" s="37" t="s">
+        <v>544</v>
+      </c>
+      <c r="E100" s="40" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A101" s="41" t="s">
+        <v>545</v>
+      </c>
+      <c r="B101" s="47" t="s">
+        <v>429</v>
+      </c>
+      <c r="C101" s="44">
+        <v>300000</v>
+      </c>
+      <c r="D101" s="42" t="s">
+        <v>546</v>
+      </c>
+      <c r="E101" s="45" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A102" s="36" t="s">
+        <v>545</v>
+      </c>
+      <c r="B102" s="48" t="s">
+        <v>432</v>
+      </c>
+      <c r="C102" s="39">
+        <v>800000</v>
+      </c>
+      <c r="D102" s="37" t="s">
+        <v>547</v>
+      </c>
+      <c r="E102" s="40" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A103" s="50" t="s">
+        <v>545</v>
+      </c>
+      <c r="B103" s="52" t="s">
+        <v>434</v>
+      </c>
+      <c r="C103" s="53">
+        <v>1400000</v>
+      </c>
+      <c r="D103" s="51" t="s">
+        <v>547</v>
+      </c>
+      <c r="E103" s="54" t="s">
+        <v>240</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1300-000000000000}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
ajout maitrise et merge terminé
</commit_message>
<xml_diff>
--- a/data/fc27-data.xlsx
+++ b/data/fc27-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexi\Desktop\Projets\builderproclubs\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1DEEEE4-B9F9-4526-A165-CF969CF78946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E08B06B8-BC79-406B-9603-CE2676BDBB29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="692" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="692" firstSheet="3" activeTab="21" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lisez-moi" sheetId="1" r:id="rId1"/>
@@ -34,6 +34,7 @@
     <sheet name="InstallationsClub" sheetId="24" r:id="rId19"/>
     <sheet name="Specialisations" sheetId="22" r:id="rId20"/>
     <sheet name="Reglages" sheetId="20" r:id="rId21"/>
+    <sheet name="Maitrise" sheetId="25" r:id="rId22"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Boss!$A$3:$AA$39</definedName>
@@ -53,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2797" uniqueCount="534">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2843" uniqueCount="560">
   <si>
     <t>Base de données — FC 27 Constructeur de build</t>
   </si>
@@ -1954,12 +1955,90 @@
     <t>Vit. sprint +3
 Finition +3</t>
   </si>
+  <si>
+    <t>Catégorie</t>
+  </si>
+  <si>
+    <t>Archétype</t>
+  </si>
+  <si>
+    <t>Passes Longues +1; Tacle debout +1</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Tacle debout +1</t>
+  </si>
+  <si>
+    <t>Agréssivité +1; Force +1</t>
+  </si>
+  <si>
+    <t>Force +1</t>
+  </si>
+  <si>
+    <t>Tacle glissé +1; vitesse +1</t>
+  </si>
+  <si>
+    <t>vitesse +1</t>
+  </si>
+  <si>
+    <t>Milieu</t>
+  </si>
+  <si>
+    <t>Endurance +1; Interceptions +1</t>
+  </si>
+  <si>
+    <t>Interceptions +1</t>
+  </si>
+  <si>
+    <t>Lucidité défensive +1; Passes courtes +1</t>
+  </si>
+  <si>
+    <t>Passes courtes +1</t>
+  </si>
+  <si>
+    <t>Réactivité +1; Conduite de balle +1</t>
+  </si>
+  <si>
+    <t>Conduite de balle +1</t>
+  </si>
+  <si>
+    <t>Précision Coup Franc +1; Vista +1</t>
+  </si>
+  <si>
+    <t>Vista +1</t>
+  </si>
+  <si>
+    <t>Attaque</t>
+  </si>
+  <si>
+    <t>Centres +1; Dribbles +1</t>
+  </si>
+  <si>
+    <t>Dribbles +1</t>
+  </si>
+  <si>
+    <t>Effet +1; Accélération +1</t>
+  </si>
+  <si>
+    <t>Accélération +1</t>
+  </si>
+  <si>
+    <t>Calme +1; Finition +1</t>
+  </si>
+  <si>
+    <t>Finition +1</t>
+  </si>
+  <si>
+    <t>Équilibre +1; Détente +1</t>
+  </si>
+  <si>
+    <t>Détente +1</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2042,6 +2121,11 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Roboto"/>
+    </font>
   </fonts>
   <fills count="11">
     <fill>
@@ -2101,7 +2185,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="25">
+  <borders count="27">
     <border>
       <left/>
       <right/>
@@ -2441,11 +2525,41 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF284E3F"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF284E3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF284E3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2585,6 +2699,42 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="10" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -46614,6 +46764,190 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7175F6AB-B2AD-4E08-98F4-8E507E709BB2}">
+  <dimension ref="A2:D14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="3" max="3" width="35.140625" customWidth="1"/>
+    <col min="4" max="4" width="40.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="56" t="s">
+        <v>534</v>
+      </c>
+      <c r="B3" s="57" t="s">
+        <v>535</v>
+      </c>
+      <c r="C3" s="57">
+        <v>10</v>
+      </c>
+      <c r="D3" s="58">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="51.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="59" t="s">
+        <v>137</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="60" t="s">
+        <v>536</v>
+      </c>
+      <c r="D4" s="61" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="62" t="s">
+        <v>137</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="63" t="s">
+        <v>538</v>
+      </c>
+      <c r="D5" s="64" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="51.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="62" t="s">
+        <v>137</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6" s="63" t="s">
+        <v>540</v>
+      </c>
+      <c r="D6" s="64" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="51.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="59" t="s">
+        <v>542</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C7" s="60" t="s">
+        <v>543</v>
+      </c>
+      <c r="D7" s="61" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="77.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="59" t="s">
+        <v>542</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C8" s="60" t="s">
+        <v>545</v>
+      </c>
+      <c r="D8" s="61" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="64.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="62" t="s">
+        <v>542</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="63" t="s">
+        <v>547</v>
+      </c>
+      <c r="D9" s="64" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="51.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="59" t="s">
+        <v>542</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="C10" s="60" t="s">
+        <v>549</v>
+      </c>
+      <c r="D10" s="61" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="51.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="62" t="s">
+        <v>551</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C11" s="63" t="s">
+        <v>552</v>
+      </c>
+      <c r="D11" s="64" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="59" t="s">
+        <v>551</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="C12" s="60" t="s">
+        <v>554</v>
+      </c>
+      <c r="D12" s="61" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="62" t="s">
+        <v>551</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C13" s="63" t="s">
+        <v>556</v>
+      </c>
+      <c r="D13" s="64" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="51.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="65" t="s">
+        <v>551</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="C14" s="66" t="s">
+        <v>558</v>
+      </c>
+      <c r="D14" s="67" t="s">
+        <v>559</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C42"/>

</xml_diff>

<commit_message>
fais le loup méchant
</commit_message>
<xml_diff>
--- a/data/fc27-data.xlsx
+++ b/data/fc27-data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexi\Desktop\Projets\builderproclubs\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6205BC5-8772-4D46-A663-188774CBDB62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F04D5EC-5AE1-48FA-B040-0856D6565E2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="692" firstSheet="10" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2468" uniqueCount="580">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2421" uniqueCount="557">
   <si>
     <t>Installation</t>
   </si>
@@ -1950,123 +1950,6 @@
   <si>
     <t>Positionnement Off.</t>
   </si>
-  <si>
-    <t>conduite_balle</t>
-  </si>
-  <si>
-    <t>tirs_loin</t>
-  </si>
-  <si>
-    <t>interception</t>
-  </si>
-  <si>
-    <t>precis_tete</t>
-  </si>
-  <si>
-    <t>lucidite_def</t>
-  </si>
-  <si>
-    <t>tacles_deb</t>
-  </si>
-  <si>
-    <t>tacles_gliss</t>
-  </si>
-  <si>
-    <t>vit_sprint</t>
-  </si>
-  <si>
-    <t>taille</t>
-  </si>
-  <si>
-    <t>Corps</t>
-  </si>
-  <si>
-    <t>/</t>
-  </si>
-  <si>
-    <t>poids</t>
-  </si>
-  <si>
-    <t>70 kg</t>
-  </si>
-  <si>
-    <t>80 kg</t>
-  </si>
-  <si>
-    <t>177 cm</t>
-  </si>
-  <si>
-    <t>164 cm</t>
-  </si>
-  <si>
-    <t>190 cm</t>
-  </si>
-  <si>
-    <t>90 kg</t>
-  </si>
-  <si>
-    <t>Incohérences relevées (non corrigées) :</t>
-  </si>
-  <si>
-    <r>
-      <t>Vista</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> : limite max annoncée 92, mais la tranche source va jusqu'à "20 pour 96" → colonnes 93-94/95/96 renseignées malgré tout.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Interception...</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> : "15 pour 85" placé en colonne 85-89 par convention (pas de colonne 85 seule).</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Tacles deb. / Tacles gliss.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> : "8 pour 75" et "6 pour 75" placés en colonne 75-79.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Force</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> : "11 pour 90" placé en colonne 90-92.</t>
-    </r>
-  </si>
 </sst>
 </file>
 
@@ -17314,7 +17197,7 @@
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
+      <c r="A4" t="s">
         <v>240</v>
       </c>
       <c r="B4" s="15" t="s">
@@ -17373,7 +17256,7 @@
       <c r="Y4" s="15"/>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
+      <c r="A5" t="s">
         <v>243</v>
       </c>
       <c r="B5" s="15" t="s">
@@ -17426,7 +17309,7 @@
       <c r="Y5" s="15"/>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
+      <c r="A6" t="s">
         <v>245</v>
       </c>
       <c r="B6" s="15" t="s">
@@ -17485,8 +17368,8 @@
       <c r="Y6" s="15"/>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A7" s="15" t="s">
-        <v>557</v>
+      <c r="A7" t="s">
+        <v>247</v>
       </c>
       <c r="B7" s="15" t="s">
         <v>242</v>
@@ -17538,7 +17421,7 @@
       <c r="Y7" s="15"/>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A8" s="15" t="s">
+      <c r="A8" t="s">
         <v>248</v>
       </c>
       <c r="B8" s="15" t="s">
@@ -17597,7 +17480,7 @@
       <c r="Y8" s="15"/>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A9" s="15" t="s">
+      <c r="A9" t="s">
         <v>250</v>
       </c>
       <c r="B9" s="15" t="s">
@@ -17652,7 +17535,7 @@
       <c r="Y9" s="15"/>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A10" s="15" t="s">
+      <c r="A10" t="s">
         <v>252</v>
       </c>
       <c r="B10" s="15" t="s">
@@ -17703,7 +17586,7 @@
       <c r="Y10" s="15"/>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A11" s="15" t="s">
+      <c r="A11" t="s">
         <v>254</v>
       </c>
       <c r="B11" s="15" t="s">
@@ -17762,7 +17645,7 @@
       <c r="Y11" s="15"/>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A12" s="15" t="s">
+      <c r="A12" t="s">
         <v>256</v>
       </c>
       <c r="B12" s="15" t="s">
@@ -17815,8 +17698,8 @@
       <c r="Y12" s="15"/>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A13" s="15" t="s">
-        <v>558</v>
+      <c r="A13" t="s">
+        <v>258</v>
       </c>
       <c r="B13" s="15" t="s">
         <v>330</v>
@@ -17874,7 +17757,7 @@
       <c r="Y13" s="15"/>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A14" s="15" t="s">
+      <c r="A14" t="s">
         <v>260</v>
       </c>
       <c r="B14" s="15" t="s">
@@ -17929,7 +17812,7 @@
       <c r="Y14" s="15"/>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A15" s="15" t="s">
+      <c r="A15" t="s">
         <v>262</v>
       </c>
       <c r="B15" s="15" t="s">
@@ -17988,7 +17871,7 @@
       <c r="Y15" s="15"/>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A16" s="15" t="s">
+      <c r="A16" t="s">
         <v>264</v>
       </c>
       <c r="B16" s="15" t="s">
@@ -18041,7 +17924,7 @@
       <c r="Y16" s="15"/>
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A17" s="15" t="s">
+      <c r="A17" t="s">
         <v>267</v>
       </c>
       <c r="B17" s="15" t="s">
@@ -18100,7 +17983,7 @@
       <c r="Y17" s="15"/>
     </row>
     <row r="18" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A18" s="15" t="s">
+      <c r="A18" t="s">
         <v>269</v>
       </c>
       <c r="B18" s="15" t="s">
@@ -18163,7 +18046,7 @@
       <c r="Y18" s="15"/>
     </row>
     <row r="19" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A19" s="15" t="s">
+      <c r="A19" t="s">
         <v>270</v>
       </c>
       <c r="B19" s="15" t="s">
@@ -18216,7 +18099,7 @@
       <c r="Y19" s="15"/>
     </row>
     <row r="20" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A20" s="15" t="s">
+      <c r="A20" t="s">
         <v>272</v>
       </c>
       <c r="B20" s="15" t="s">
@@ -18269,7 +18152,7 @@
       <c r="Y20" s="15"/>
     </row>
     <row r="21" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A21" s="15" t="s">
+      <c r="A21" t="s">
         <v>274</v>
       </c>
       <c r="B21" s="15" t="s">
@@ -18322,8 +18205,8 @@
       <c r="Y21" s="15"/>
     </row>
     <row r="22" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A22" s="15" t="s">
-        <v>559</v>
+      <c r="A22" t="s">
+        <v>276</v>
       </c>
       <c r="B22" s="15" t="s">
         <v>278</v>
@@ -18377,8 +18260,8 @@
       <c r="Y22" s="15"/>
     </row>
     <row r="23" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A23" s="15" t="s">
-        <v>560</v>
+      <c r="A23" t="s">
+        <v>279</v>
       </c>
       <c r="B23" s="15" t="s">
         <v>278</v>
@@ -18432,8 +18315,8 @@
       <c r="Y23" s="15"/>
     </row>
     <row r="24" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A24" s="15" t="s">
-        <v>561</v>
+      <c r="A24" t="s">
+        <v>281</v>
       </c>
       <c r="B24" s="15" t="s">
         <v>278</v>
@@ -18487,8 +18370,8 @@
       <c r="Y24" s="15"/>
     </row>
     <row r="25" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A25" s="15" t="s">
-        <v>562</v>
+      <c r="A25" t="s">
+        <v>282</v>
       </c>
       <c r="B25" s="15" t="s">
         <v>278</v>
@@ -18540,8 +18423,8 @@
       <c r="Y25" s="15"/>
     </row>
     <row r="26" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A26" s="15" t="s">
-        <v>563</v>
+      <c r="A26" t="s">
+        <v>284</v>
       </c>
       <c r="B26" s="15" t="s">
         <v>278</v>
@@ -18591,7 +18474,7 @@
       <c r="Y26" s="15"/>
     </row>
     <row r="27" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A27" s="15" t="s">
+      <c r="A27" t="s">
         <v>286</v>
       </c>
       <c r="B27" s="15" t="s">
@@ -18650,8 +18533,8 @@
       <c r="Y27" s="15"/>
     </row>
     <row r="28" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A28" s="15" t="s">
-        <v>564</v>
+      <c r="A28" t="s">
+        <v>289</v>
       </c>
       <c r="B28" s="15" t="s">
         <v>288</v>
@@ -18701,7 +18584,7 @@
       <c r="Y28" s="15"/>
     </row>
     <row r="29" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A29" s="15" t="s">
+      <c r="A29" t="s">
         <v>291</v>
       </c>
       <c r="B29" s="15" t="s">
@@ -18756,7 +18639,7 @@
       <c r="Y29" s="15"/>
     </row>
     <row r="30" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A30" s="15" t="s">
+      <c r="A30" t="s">
         <v>296</v>
       </c>
       <c r="B30" s="15" t="s">
@@ -18809,7 +18692,7 @@
       <c r="Y30" s="15"/>
     </row>
     <row r="31" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A31" s="15" t="s">
+      <c r="A31" t="s">
         <v>294</v>
       </c>
       <c r="B31" s="15" t="s">
@@ -18862,7 +18745,7 @@
       <c r="Y31" s="15"/>
     </row>
     <row r="32" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A32" s="15" t="s">
+      <c r="A32" t="s">
         <v>298</v>
       </c>
       <c r="B32" s="15" t="s">
@@ -18919,7 +18802,7 @@
       <c r="Y32" s="15"/>
     </row>
     <row r="33" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A33" s="15" t="s">
+      <c r="A33" t="s">
         <v>299</v>
       </c>
       <c r="B33" s="15" t="s">
@@ -18962,7 +18845,7 @@
       </c>
     </row>
     <row r="34" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A34" s="15" t="s">
+      <c r="A34" t="s">
         <v>302</v>
       </c>
       <c r="B34" s="15" t="s">
@@ -19179,8 +19062,8 @@
         <v>327</v>
       </c>
     </row>
-    <row r="4" spans="1:25" ht="45" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
+    <row r="4" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>240</v>
       </c>
       <c r="B4" s="15" t="s">
@@ -19240,8 +19123,8 @@
       <c r="X4" s="15"/>
       <c r="Y4" s="15"/>
     </row>
-    <row r="5" spans="1:25" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
+    <row r="5" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>243</v>
       </c>
       <c r="B5" s="15" t="s">
@@ -19299,8 +19182,8 @@
       <c r="X5" s="15"/>
       <c r="Y5" s="15"/>
     </row>
-    <row r="6" spans="1:25" ht="45" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
+    <row r="6" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>245</v>
       </c>
       <c r="B6" s="15" t="s">
@@ -19358,9 +19241,9 @@
       <c r="X6" s="15"/>
       <c r="Y6" s="15"/>
     </row>
-    <row r="7" spans="1:25" ht="45" x14ac:dyDescent="0.25">
-      <c r="A7" s="15" t="s">
-        <v>557</v>
+    <row r="7" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>247</v>
       </c>
       <c r="B7" s="15" t="s">
         <v>242</v>
@@ -19411,8 +19294,8 @@
       <c r="X7" s="15"/>
       <c r="Y7" s="15"/>
     </row>
-    <row r="8" spans="1:25" ht="45" x14ac:dyDescent="0.25">
-      <c r="A8" s="15" t="s">
+    <row r="8" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>248</v>
       </c>
       <c r="B8" s="15" t="s">
@@ -19464,8 +19347,8 @@
       <c r="X8" s="15"/>
       <c r="Y8" s="15"/>
     </row>
-    <row r="9" spans="1:25" ht="45" x14ac:dyDescent="0.25">
-      <c r="A9" s="15" t="s">
+    <row r="9" spans="1:25" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>250</v>
       </c>
       <c r="B9" s="15" t="s">
@@ -19520,7 +19403,7 @@
       <c r="Y9" s="15"/>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A10" s="15" t="s">
+      <c r="A10" t="s">
         <v>252</v>
       </c>
       <c r="B10" s="15" t="s">
@@ -19571,7 +19454,7 @@
       <c r="Y10" s="15"/>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A11" s="15" t="s">
+      <c r="A11" t="s">
         <v>254</v>
       </c>
       <c r="B11" s="15" t="s">
@@ -19630,7 +19513,7 @@
       <c r="Y11" s="15"/>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A12" s="15" t="s">
+      <c r="A12" t="s">
         <v>256</v>
       </c>
       <c r="B12" s="15" t="s">
@@ -19679,8 +19562,8 @@
       <c r="Y12" s="15"/>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A13" s="15" t="s">
-        <v>558</v>
+      <c r="A13" t="s">
+        <v>258</v>
       </c>
       <c r="B13" s="15" t="s">
         <v>330</v>
@@ -19738,7 +19621,7 @@
       <c r="Y13" s="15"/>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A14" s="15" t="s">
+      <c r="A14" t="s">
         <v>260</v>
       </c>
       <c r="B14" s="15" t="s">
@@ -19793,7 +19676,7 @@
       <c r="Y14" s="15"/>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A15" s="15" t="s">
+      <c r="A15" t="s">
         <v>262</v>
       </c>
       <c r="B15" s="15" t="s">
@@ -19852,7 +19735,7 @@
       <c r="Y15" s="15"/>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A16" s="15" t="s">
+      <c r="A16" t="s">
         <v>264</v>
       </c>
       <c r="B16" s="15" t="s">
@@ -19905,7 +19788,7 @@
       <c r="Y16" s="15"/>
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A17" s="15" t="s">
+      <c r="A17" t="s">
         <v>267</v>
       </c>
       <c r="B17" s="15" t="s">
@@ -19958,7 +19841,7 @@
       <c r="Y17" s="15"/>
     </row>
     <row r="18" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A18" s="15" t="s">
+      <c r="A18" t="s">
         <v>269</v>
       </c>
       <c r="B18" s="15" t="s">
@@ -20023,7 +19906,7 @@
       <c r="Y18" s="15"/>
     </row>
     <row r="19" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A19" s="15" t="s">
+      <c r="A19" t="s">
         <v>270</v>
       </c>
       <c r="B19" s="15" t="s">
@@ -20076,7 +19959,7 @@
       <c r="Y19" s="15"/>
     </row>
     <row r="20" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A20" s="15" t="s">
+      <c r="A20" t="s">
         <v>272</v>
       </c>
       <c r="B20" s="15" t="s">
@@ -20133,7 +20016,7 @@
       <c r="Y20" s="15"/>
     </row>
     <row r="21" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A21" s="15" t="s">
+      <c r="A21" t="s">
         <v>274</v>
       </c>
       <c r="B21" s="15" t="s">
@@ -20191,9 +20074,9 @@
       <c r="X21" s="15"/>
       <c r="Y21" s="15"/>
     </row>
-    <row r="22" spans="1:25" ht="30" x14ac:dyDescent="0.25">
-      <c r="A22" s="15" t="s">
-        <v>559</v>
+    <row r="22" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>276</v>
       </c>
       <c r="B22" s="15" t="s">
         <v>278</v>
@@ -20244,9 +20127,9 @@
       <c r="X22" s="15"/>
       <c r="Y22" s="15"/>
     </row>
-    <row r="23" spans="1:25" ht="30" x14ac:dyDescent="0.25">
-      <c r="A23" s="15" t="s">
-        <v>560</v>
+    <row r="23" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>279</v>
       </c>
       <c r="B23" s="15" t="s">
         <v>278</v>
@@ -20295,9 +20178,9 @@
       <c r="X23" s="15"/>
       <c r="Y23" s="15"/>
     </row>
-    <row r="24" spans="1:25" ht="30" x14ac:dyDescent="0.25">
-      <c r="A24" s="15" t="s">
-        <v>561</v>
+    <row r="24" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>281</v>
       </c>
       <c r="B24" s="15" t="s">
         <v>278</v>
@@ -20348,9 +20231,9 @@
       <c r="X24" s="15"/>
       <c r="Y24" s="15"/>
     </row>
-    <row r="25" spans="1:25" ht="30" x14ac:dyDescent="0.25">
-      <c r="A25" s="15" t="s">
-        <v>562</v>
+    <row r="25" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>282</v>
       </c>
       <c r="B25" s="15" t="s">
         <v>278</v>
@@ -20399,9 +20282,9 @@
       <c r="X25" s="15"/>
       <c r="Y25" s="15"/>
     </row>
-    <row r="26" spans="1:25" ht="30" x14ac:dyDescent="0.25">
-      <c r="A26" s="15" t="s">
-        <v>563</v>
+    <row r="26" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>284</v>
       </c>
       <c r="B26" s="15" t="s">
         <v>278</v>
@@ -20450,8 +20333,8 @@
       <c r="X26" s="15"/>
       <c r="Y26" s="15"/>
     </row>
-    <row r="27" spans="1:25" ht="30" x14ac:dyDescent="0.25">
-      <c r="A27" s="15" t="s">
+    <row r="27" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>286</v>
       </c>
       <c r="B27" s="15" t="s">
@@ -20501,9 +20384,9 @@
       <c r="X27" s="15"/>
       <c r="Y27" s="15"/>
     </row>
-    <row r="28" spans="1:25" ht="30" x14ac:dyDescent="0.25">
-      <c r="A28" s="15" t="s">
-        <v>564</v>
+    <row r="28" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>289</v>
       </c>
       <c r="B28" s="15" t="s">
         <v>288</v>
@@ -20554,8 +20437,8 @@
       <c r="X28" s="15"/>
       <c r="Y28" s="15"/>
     </row>
-    <row r="29" spans="1:25" ht="30" x14ac:dyDescent="0.25">
-      <c r="A29" s="15" t="s">
+    <row r="29" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>291</v>
       </c>
       <c r="B29" s="15" t="s">
@@ -20609,8 +20492,8 @@
       <c r="X29" s="15"/>
       <c r="Y29" s="15"/>
     </row>
-    <row r="30" spans="1:25" ht="30" x14ac:dyDescent="0.25">
-      <c r="A30" s="15" t="s">
+    <row r="30" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>296</v>
       </c>
       <c r="B30" s="15" t="s">
@@ -20658,8 +20541,8 @@
       <c r="X30" s="15"/>
       <c r="Y30" s="15"/>
     </row>
-    <row r="31" spans="1:25" ht="30" x14ac:dyDescent="0.25">
-      <c r="A31" s="15" t="s">
+    <row r="31" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>294</v>
       </c>
       <c r="B31" s="15" t="s">
@@ -20711,8 +20594,8 @@
       <c r="X31" s="15"/>
       <c r="Y31" s="15"/>
     </row>
-    <row r="32" spans="1:25" ht="30" x14ac:dyDescent="0.25">
-      <c r="A32" s="15" t="s">
+    <row r="32" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>298</v>
       </c>
       <c r="B32" s="15" t="s">
@@ -20769,7 +20652,7 @@
       <c r="Y32" s="15"/>
     </row>
     <row r="33" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A33" s="15" t="s">
+      <c r="A33" t="s">
         <v>299</v>
       </c>
       <c r="B33" s="15" t="s">
@@ -20812,7 +20695,7 @@
       </c>
     </row>
     <row r="34" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A34" s="15" t="s">
+      <c r="A34" t="s">
         <v>302</v>
       </c>
       <c r="B34" s="15" t="s">
@@ -21425,7 +21308,7 @@
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
+      <c r="A4" t="s">
         <v>240</v>
       </c>
       <c r="B4" s="15" t="s">
@@ -21486,7 +21369,7 @@
       <c r="Y4" s="15"/>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
+      <c r="A5" t="s">
         <v>243</v>
       </c>
       <c r="B5" s="15" t="s">
@@ -21539,7 +21422,7 @@
       <c r="Y5" s="15"/>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
+      <c r="A6" t="s">
         <v>245</v>
       </c>
       <c r="B6" s="15" t="s">
@@ -21598,8 +21481,8 @@
       <c r="Y6" s="15"/>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A7" s="15" t="s">
-        <v>557</v>
+      <c r="A7" t="s">
+        <v>247</v>
       </c>
       <c r="B7" s="15" t="s">
         <v>242</v>
@@ -21651,7 +21534,7 @@
       <c r="Y7" s="15"/>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A8" s="15" t="s">
+      <c r="A8" t="s">
         <v>248</v>
       </c>
       <c r="B8" s="15" t="s">
@@ -21706,7 +21589,7 @@
       <c r="Y8" s="15"/>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A9" s="15" t="s">
+      <c r="A9" t="s">
         <v>250</v>
       </c>
       <c r="B9" s="15" t="s">
@@ -21765,7 +21648,7 @@
       <c r="Y9" s="15"/>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A10" s="15" t="s">
+      <c r="A10" t="s">
         <v>252</v>
       </c>
       <c r="B10" s="15" t="s">
@@ -21822,7 +21705,7 @@
       <c r="Y10" s="15"/>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A11" s="15" t="s">
+      <c r="A11" t="s">
         <v>254</v>
       </c>
       <c r="B11" s="15" t="s">
@@ -21881,7 +21764,7 @@
       <c r="Y11" s="15"/>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A12" s="15" t="s">
+      <c r="A12" t="s">
         <v>256</v>
       </c>
       <c r="B12" s="15" t="s">
@@ -21940,8 +21823,8 @@
       <c r="Y12" s="15"/>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A13" s="15" t="s">
-        <v>558</v>
+      <c r="A13" t="s">
+        <v>258</v>
       </c>
       <c r="B13" s="15" t="s">
         <v>330</v>
@@ -22001,7 +21884,7 @@
       <c r="Y13" s="15"/>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A14" s="15" t="s">
+      <c r="A14" t="s">
         <v>260</v>
       </c>
       <c r="B14" s="15" t="s">
@@ -22060,7 +21943,7 @@
       <c r="Y14" s="15"/>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A15" s="15" t="s">
+      <c r="A15" t="s">
         <v>262</v>
       </c>
       <c r="B15" s="15" t="s">
@@ -22119,7 +22002,7 @@
       <c r="Y15" s="15"/>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A16" s="15" t="s">
+      <c r="A16" t="s">
         <v>264</v>
       </c>
       <c r="B16" s="15" t="s">
@@ -22176,7 +22059,7 @@
       <c r="Y16" s="15"/>
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A17" s="15" t="s">
+      <c r="A17" t="s">
         <v>267</v>
       </c>
       <c r="B17" s="15" t="s">
@@ -22233,7 +22116,7 @@
       <c r="Y17" s="15"/>
     </row>
     <row r="18" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A18" s="15" t="s">
+      <c r="A18" t="s">
         <v>269</v>
       </c>
       <c r="B18" s="15" t="s">
@@ -22296,7 +22179,7 @@
       <c r="Y18" s="15"/>
     </row>
     <row r="19" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A19" s="15" t="s">
+      <c r="A19" t="s">
         <v>270</v>
       </c>
       <c r="B19" s="15" t="s">
@@ -22345,7 +22228,7 @@
       <c r="Y19" s="15"/>
     </row>
     <row r="20" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A20" s="15" t="s">
+      <c r="A20" t="s">
         <v>272</v>
       </c>
       <c r="B20" s="15" t="s">
@@ -22402,7 +22285,7 @@
       <c r="Y20" s="15"/>
     </row>
     <row r="21" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A21" s="15" t="s">
+      <c r="A21" t="s">
         <v>274</v>
       </c>
       <c r="B21" s="15" t="s">
@@ -22457,8 +22340,8 @@
       <c r="Y21" s="15"/>
     </row>
     <row r="22" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A22" s="15" t="s">
-        <v>559</v>
+      <c r="A22" t="s">
+        <v>276</v>
       </c>
       <c r="B22" s="15" t="s">
         <v>278</v>
@@ -22510,8 +22393,8 @@
       <c r="Y22" s="15"/>
     </row>
     <row r="23" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A23" s="15" t="s">
-        <v>560</v>
+      <c r="A23" t="s">
+        <v>279</v>
       </c>
       <c r="B23" s="15" t="s">
         <v>278</v>
@@ -22563,8 +22446,8 @@
       <c r="Y23" s="15"/>
     </row>
     <row r="24" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A24" s="15" t="s">
-        <v>561</v>
+      <c r="A24" t="s">
+        <v>281</v>
       </c>
       <c r="B24" s="15" t="s">
         <v>278</v>
@@ -22618,8 +22501,8 @@
       <c r="Y24" s="15"/>
     </row>
     <row r="25" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A25" s="15" t="s">
-        <v>562</v>
+      <c r="A25" t="s">
+        <v>282</v>
       </c>
       <c r="B25" s="15" t="s">
         <v>278</v>
@@ -22669,8 +22552,8 @@
       <c r="Y25" s="15"/>
     </row>
     <row r="26" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A26" s="15" t="s">
-        <v>563</v>
+      <c r="A26" t="s">
+        <v>284</v>
       </c>
       <c r="B26" s="15" t="s">
         <v>278</v>
@@ -22720,7 +22603,7 @@
       <c r="Y26" s="15"/>
     </row>
     <row r="27" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A27" s="15" t="s">
+      <c r="A27" t="s">
         <v>286</v>
       </c>
       <c r="B27" s="15" t="s">
@@ -22771,8 +22654,8 @@
       <c r="Y27" s="15"/>
     </row>
     <row r="28" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A28" s="15" t="s">
-        <v>564</v>
+      <c r="A28" t="s">
+        <v>289</v>
       </c>
       <c r="B28" s="15" t="s">
         <v>288</v>
@@ -22824,7 +22707,7 @@
       <c r="Y28" s="15"/>
     </row>
     <row r="29" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A29" s="15" t="s">
+      <c r="A29" t="s">
         <v>291</v>
       </c>
       <c r="B29" s="15" t="s">
@@ -22875,7 +22758,7 @@
       <c r="Y29" s="15"/>
     </row>
     <row r="30" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A30" s="15" t="s">
+      <c r="A30" t="s">
         <v>296</v>
       </c>
       <c r="B30" s="15" t="s">
@@ -22924,7 +22807,7 @@
       <c r="Y30" s="15"/>
     </row>
     <row r="31" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A31" s="15" t="s">
+      <c r="A31" t="s">
         <v>294</v>
       </c>
       <c r="B31" s="15" t="s">
@@ -22975,7 +22858,7 @@
       <c r="Y31" s="15"/>
     </row>
     <row r="32" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A32" s="15" t="s">
+      <c r="A32" t="s">
         <v>298</v>
       </c>
       <c r="B32" s="15" t="s">
@@ -23032,7 +22915,7 @@
       <c r="Y32" s="15"/>
     </row>
     <row r="33" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A33" s="15" t="s">
+      <c r="A33" t="s">
         <v>299</v>
       </c>
       <c r="B33" s="15" t="s">
@@ -23075,7 +22958,7 @@
       </c>
     </row>
     <row r="34" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A34" s="15" t="s">
+      <c r="A34" t="s">
         <v>302</v>
       </c>
       <c r="B34" s="15" t="s">
@@ -23118,170 +23001,76 @@
       </c>
     </row>
     <row r="35" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A35" s="15" t="s">
-        <v>565</v>
-      </c>
-      <c r="B35" s="15" t="s">
-        <v>566</v>
-      </c>
-      <c r="C35" s="15" t="s">
-        <v>328</v>
-      </c>
-      <c r="D35" s="15" t="s">
-        <v>571</v>
-      </c>
-      <c r="E35" s="15" t="s">
-        <v>572</v>
-      </c>
-      <c r="F35" s="15" t="s">
-        <v>573</v>
-      </c>
-      <c r="G35" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="H35" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="I35" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="J35" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="K35" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="L35" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="M35" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="N35" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="O35" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="P35" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="Q35" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="R35" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="S35" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="T35" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="U35" s="15" t="s">
-        <v>567</v>
-      </c>
+      <c r="A35" s="15"/>
+      <c r="B35" s="15"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="15"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="15"/>
+      <c r="H35" s="15"/>
+      <c r="I35" s="15"/>
+      <c r="J35" s="15"/>
+      <c r="K35" s="15"/>
+      <c r="L35" s="15"/>
+      <c r="M35" s="15"/>
+      <c r="N35" s="15"/>
+      <c r="O35" s="15"/>
+      <c r="P35" s="15"/>
+      <c r="Q35" s="15"/>
+      <c r="R35" s="15"/>
+      <c r="S35" s="15"/>
+      <c r="T35" s="15"/>
+      <c r="U35" s="15"/>
       <c r="V35" s="15"/>
       <c r="W35" s="15"/>
       <c r="X35" s="15"/>
       <c r="Y35" s="15"/>
     </row>
     <row r="36" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A36" s="15" t="s">
-        <v>568</v>
-      </c>
-      <c r="B36" s="15" t="s">
-        <v>566</v>
-      </c>
-      <c r="C36" s="15" t="s">
-        <v>328</v>
-      </c>
-      <c r="D36" s="15" t="s">
-        <v>570</v>
-      </c>
-      <c r="E36" s="15" t="s">
-        <v>569</v>
-      </c>
-      <c r="F36" s="15" t="s">
-        <v>574</v>
-      </c>
-      <c r="G36" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="H36" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="I36" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="J36" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="K36" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="L36" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="M36" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="N36" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="O36" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="P36" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="Q36" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="R36" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="S36" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="T36" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="U36" s="15" t="s">
-        <v>567</v>
-      </c>
+      <c r="A36" s="15"/>
+      <c r="B36" s="15"/>
+      <c r="C36" s="15"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="15"/>
+      <c r="F36" s="15"/>
+      <c r="G36" s="15"/>
+      <c r="H36" s="15"/>
+      <c r="I36" s="15"/>
+      <c r="J36" s="15"/>
+      <c r="K36" s="15"/>
+      <c r="L36" s="15"/>
+      <c r="M36" s="15"/>
+      <c r="N36" s="15"/>
+      <c r="O36" s="15"/>
+      <c r="P36" s="15"/>
+      <c r="Q36" s="15"/>
+      <c r="R36" s="15"/>
+      <c r="S36" s="15"/>
+      <c r="T36" s="15"/>
+      <c r="U36" s="15"/>
       <c r="V36" s="15"/>
       <c r="W36" s="15"/>
       <c r="X36" s="15"/>
       <c r="Y36" s="15"/>
     </row>
     <row r="38" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A38" s="45" t="s">
-        <v>575</v>
-      </c>
+      <c r="A38" s="45"/>
     </row>
     <row r="39" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A39" s="46"/>
     </row>
     <row r="40" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A40" s="47" t="s">
-        <v>576</v>
-      </c>
+      <c r="A40" s="47"/>
     </row>
     <row r="41" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A41" s="47" t="s">
-        <v>577</v>
-      </c>
+      <c r="A41" s="47"/>
     </row>
     <row r="42" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A42" s="47" t="s">
-        <v>578</v>
-      </c>
+      <c r="A42" s="47"/>
     </row>
     <row r="43" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A43" s="47" t="s">
-        <v>579</v>
-      </c>
+      <c r="A43" s="47"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:Y39" xr:uid="{00000000-0009-0000-0000-00000D000000}"/>
@@ -23386,7 +23175,7 @@
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
+      <c r="A4" t="s">
         <v>240</v>
       </c>
       <c r="B4" s="15" t="s">
@@ -23435,7 +23224,7 @@
       <c r="Y4" s="15"/>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
+      <c r="A5" t="s">
         <v>243</v>
       </c>
       <c r="B5" s="15" t="s">
@@ -23482,7 +23271,7 @@
       <c r="Y5" s="15"/>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
+      <c r="A6" t="s">
         <v>245</v>
       </c>
       <c r="B6" s="15" t="s">
@@ -23541,8 +23330,8 @@
       <c r="Y6" s="15"/>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A7" s="15" t="s">
-        <v>557</v>
+      <c r="A7" t="s">
+        <v>247</v>
       </c>
       <c r="B7" s="15" t="s">
         <v>242</v>
@@ -23590,7 +23379,7 @@
       <c r="Y7" s="15"/>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A8" s="15" t="s">
+      <c r="A8" t="s">
         <v>248</v>
       </c>
       <c r="B8" s="15" t="s">
@@ -23639,7 +23428,7 @@
       <c r="Y8" s="15"/>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A9" s="15" t="s">
+      <c r="A9" t="s">
         <v>250</v>
       </c>
       <c r="B9" s="15" t="s">
@@ -23694,7 +23483,7 @@
       <c r="Y9" s="15"/>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A10" s="15" t="s">
+      <c r="A10" t="s">
         <v>252</v>
       </c>
       <c r="B10" s="15" t="s">
@@ -23745,7 +23534,7 @@
       <c r="Y10" s="15"/>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A11" s="15" t="s">
+      <c r="A11" t="s">
         <v>254</v>
       </c>
       <c r="B11" s="15" t="s">
@@ -23806,7 +23595,7 @@
       <c r="Y11" s="15"/>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A12" s="15" t="s">
+      <c r="A12" t="s">
         <v>256</v>
       </c>
       <c r="B12" s="15" t="s">
@@ -23865,8 +23654,8 @@
       <c r="Y12" s="15"/>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A13" s="15" t="s">
-        <v>558</v>
+      <c r="A13" t="s">
+        <v>258</v>
       </c>
       <c r="B13" s="15" t="s">
         <v>330</v>
@@ -23922,7 +23711,7 @@
       <c r="Y13" s="15"/>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A14" s="15" t="s">
+      <c r="A14" t="s">
         <v>260</v>
       </c>
       <c r="B14" s="15" t="s">
@@ -23977,7 +23766,7 @@
       <c r="Y14" s="15"/>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A15" s="15" t="s">
+      <c r="A15" t="s">
         <v>262</v>
       </c>
       <c r="B15" s="15" t="s">
@@ -24036,7 +23825,7 @@
       <c r="Y15" s="15"/>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A16" s="15" t="s">
+      <c r="A16" t="s">
         <v>264</v>
       </c>
       <c r="B16" s="15" t="s">
@@ -24087,7 +23876,7 @@
       <c r="Y16" s="15"/>
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A17" s="15" t="s">
+      <c r="A17" t="s">
         <v>267</v>
       </c>
       <c r="B17" s="15" t="s">
@@ -24144,7 +23933,7 @@
       <c r="Y17" s="15"/>
     </row>
     <row r="18" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A18" s="15" t="s">
+      <c r="A18" t="s">
         <v>269</v>
       </c>
       <c r="B18" s="15" t="s">
@@ -24207,7 +23996,7 @@
       <c r="Y18" s="15"/>
     </row>
     <row r="19" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A19" s="15" t="s">
+      <c r="A19" t="s">
         <v>270</v>
       </c>
       <c r="B19" s="15" t="s">
@@ -24260,7 +24049,7 @@
       <c r="Y19" s="15"/>
     </row>
     <row r="20" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A20" s="15" t="s">
+      <c r="A20" t="s">
         <v>272</v>
       </c>
       <c r="B20" s="15" t="s">
@@ -24317,7 +24106,7 @@
       <c r="Y20" s="15"/>
     </row>
     <row r="21" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A21" s="15" t="s">
+      <c r="A21" t="s">
         <v>274</v>
       </c>
       <c r="B21" s="15" t="s">
@@ -24374,8 +24163,8 @@
       <c r="Y21" s="15"/>
     </row>
     <row r="22" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A22" s="15" t="s">
-        <v>559</v>
+      <c r="A22" t="s">
+        <v>276</v>
       </c>
       <c r="B22" s="15" t="s">
         <v>278</v>
@@ -24427,8 +24216,8 @@
       <c r="Y22" s="15"/>
     </row>
     <row r="23" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A23" s="15" t="s">
-        <v>560</v>
+      <c r="A23" t="s">
+        <v>279</v>
       </c>
       <c r="B23" s="15" t="s">
         <v>278</v>
@@ -24486,8 +24275,8 @@
       <c r="Y23" s="15"/>
     </row>
     <row r="24" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A24" s="15" t="s">
-        <v>561</v>
+      <c r="A24" t="s">
+        <v>281</v>
       </c>
       <c r="B24" s="15" t="s">
         <v>278</v>
@@ -24539,8 +24328,8 @@
       <c r="Y24" s="15"/>
     </row>
     <row r="25" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A25" s="15" t="s">
-        <v>562</v>
+      <c r="A25" t="s">
+        <v>282</v>
       </c>
       <c r="B25" s="15" t="s">
         <v>278</v>
@@ -24590,8 +24379,8 @@
       <c r="Y25" s="15"/>
     </row>
     <row r="26" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A26" s="15" t="s">
-        <v>563</v>
+      <c r="A26" t="s">
+        <v>284</v>
       </c>
       <c r="B26" s="15" t="s">
         <v>278</v>
@@ -24641,7 +24430,7 @@
       <c r="Y26" s="15"/>
     </row>
     <row r="27" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A27" s="15" t="s">
+      <c r="A27" t="s">
         <v>286</v>
       </c>
       <c r="B27" s="15" t="s">
@@ -24688,8 +24477,8 @@
       <c r="Y27" s="15"/>
     </row>
     <row r="28" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A28" s="15" t="s">
-        <v>564</v>
+      <c r="A28" t="s">
+        <v>289</v>
       </c>
       <c r="B28" s="15" t="s">
         <v>288</v>
@@ -24739,7 +24528,7 @@
       <c r="Y28" s="15"/>
     </row>
     <row r="29" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A29" s="15" t="s">
+      <c r="A29" t="s">
         <v>291</v>
       </c>
       <c r="B29" s="15" t="s">
@@ -24798,7 +24587,7 @@
       <c r="Y29" s="15"/>
     </row>
     <row r="30" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A30" s="15" t="s">
+      <c r="A30" t="s">
         <v>296</v>
       </c>
       <c r="B30" s="15" t="s">
@@ -24857,7 +24646,7 @@
       <c r="Y30" s="15"/>
     </row>
     <row r="31" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A31" s="15" t="s">
+      <c r="A31" t="s">
         <v>294</v>
       </c>
       <c r="B31" s="15" t="s">
@@ -24912,7 +24701,7 @@
       <c r="Y31" s="15"/>
     </row>
     <row r="32" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A32" s="15" t="s">
+      <c r="A32" t="s">
         <v>298</v>
       </c>
       <c r="B32" s="15" t="s">
@@ -24963,7 +24752,7 @@
       <c r="Y32" s="15"/>
     </row>
     <row r="33" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A33" s="15" t="s">
+      <c r="A33" t="s">
         <v>299</v>
       </c>
       <c r="B33" s="15" t="s">
@@ -25008,7 +24797,7 @@
       </c>
     </row>
     <row r="34" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A34" s="15" t="s">
+      <c r="A34" t="s">
         <v>302</v>
       </c>
       <c r="B34" s="15" t="s">

</xml_diff>

<commit_message>
fait le méchant loup
</commit_message>
<xml_diff>
--- a/data/fc27-data.xlsx
+++ b/data/fc27-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alexi\Desktop\Projets\builderproclubs\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F04D5EC-5AE1-48FA-B040-0856D6565E2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B22C0593-04A0-4B70-8147-D237C7E9DDBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="692" firstSheet="10" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="692" firstSheet="9" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lisez-moi" sheetId="1" r:id="rId1"/>
@@ -4579,7 +4579,7 @@
     </row>
     <row r="44" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="18" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B44" s="18" t="s">
         <v>464</v>
@@ -4595,8 +4595,8 @@
       <c r="I44" s="16"/>
     </row>
     <row r="45" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="15" t="s">
-        <v>236</v>
+      <c r="A45" s="18" t="s">
+        <v>234</v>
       </c>
       <c r="B45" s="15" t="s">
         <v>518</v>
@@ -4625,7 +4625,7 @@
     </row>
     <row r="46" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="18" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B46" s="18" t="s">
         <v>520</v>
@@ -4653,8 +4653,8 @@
       </c>
     </row>
     <row r="47" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="15" t="s">
-        <v>236</v>
+      <c r="A47" s="18" t="s">
+        <v>234</v>
       </c>
       <c r="B47" s="15" t="s">
         <v>521</v>

</xml_diff>